<commit_message>
Update model outputs 2026-06-15 18:06:54
</commit_message>
<xml_diff>
--- a/files/AFL_goalscorers.xlsx
+++ b/files/AFL_goalscorers.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="158">
   <si>
     <t xml:space="preserve">date_local</t>
   </si>
@@ -32,61 +32,403 @@
     <t xml:space="preserve">odds_3_plus</t>
   </si>
   <si>
-    <t xml:space="preserve">essendon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nate Caddy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hussien El Achkar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kyle Langford</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Harrison Jones</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sullivan Robey</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nik Cox</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Archer Day-Wicks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Archie Perkins</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Xavier Duursma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zach Merrett</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sam Durham</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elijah Tsatas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Will Setterfield</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nick Bryan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mason Redman</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Saad El-Hawli</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Max Kondogiannis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lachlan Blakiston</t>
+    <t xml:space="preserve">fremantle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Josh Treacy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jye Amiss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patrick Voss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Michael Frederick</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Isaiah Dudley</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shai Bolton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Murphy Reid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sam Switkowski</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luke Jackson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hayden Young</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mason Cox</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Andrew Brayshaw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nathan O'Driscoll</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jaeger O'Meara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neil Erasmus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corey Wagner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oscar McDonald</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alex Pearce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">geelong cats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jeremy Cameron</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shannon Neale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oliver Henry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shaun Mannagh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jack Martin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patrick Dangerfield</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oliver Dempsey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oliver Wiltshire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gryan Miers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jack Bowes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max Holmes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bailey Smith</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mark Blicavs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tom Atkins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jack Henry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oisin Mullin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tanner Bruhn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mark O'Connor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold coast suns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ben King</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ben Long</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jed Walter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bailey Humphrey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Christian Petracca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lachlan Gulbin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Will Graham</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leonardo Lombard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Touk Miller</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noah Anderson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ned Moyle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jai Murray</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matt Rowell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lachie Weller</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jarrod Witts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daniel Rioli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joel Jeffrey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">John Noble</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hawthorn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nick Watson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mabior Chol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mitch Lewis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jack Ginnivan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dylan Moore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Connor Macdonald</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cameron Nairn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Will Day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jai Newcombe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blake Hardwick</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ned Reeves</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lloyd Meek</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Josh Weddle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Massimo D'Ambrosio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cam Mackenzie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Josh Ward</t>
+  </si>
+  <si>
+    <t xml:space="preserve">James Sicily</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jarman Impey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adelaide crows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Riley Thilthorpe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Darcy Fogarty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Josh Rachele</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ben Keays</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luke Pedlar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toby Murray</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jordan Dawson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alex Neal-Bullen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jake Soligo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zac Taylor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brayden Cook</t>
+  </si>
+  <si>
+    <t xml:space="preserve">James Peatling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daniel Curtin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lachlan McAndrew</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sam Berry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luke Nankervis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hugo Hall-Kahan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nick Murray</t>
+  </si>
+  <si>
+    <t xml:space="preserve">carlton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Harry McKay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Will Hayward</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brodie Kemp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ben Ainsworth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jack Ison</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mitch McGovern</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flynn Young</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Talor Byrne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Francis Evans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jagga Smith</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patrick Cripps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blake Acres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marc Pittonet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">George Hewett</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sam Walsh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adam Cerra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oliver Florent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wade Derksen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">greater western sydney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toby Greene</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jake Stringer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aaron Cadman</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max Gruzewski</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phoenix Gothard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Callum Brown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brent Daniels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toby Bedford</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stephen Coniglio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toby McMullin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Harvey Thomas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finn Callaghan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conor Stone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leek Aleer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clayton Oliver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kieren Briggs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Harry Himmelberg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joe Fonti</t>
   </si>
   <si>
     <t xml:space="preserve">melbourne</t>
@@ -144,462 +486,6 @@
   </si>
   <si>
     <t xml:space="preserve">Koltyn Tholstrup</t>
-  </si>
-  <si>
-    <t xml:space="preserve">north melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nick Larkey</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paul Curtis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cooper Trembath</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jack Darling</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cameron Zurhaar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zane Duursma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jacob Konstanty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Charlie Spargo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Colby McKercher</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jy Simpkin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Harry Sheezel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luke Davies-Uniacke</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luke Parker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">George Wardlaw</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tristan Xerri</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dylan Stephens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wil Dawson</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zac Fisher</t>
-  </si>
-  <si>
-    <t xml:space="preserve">port adelaide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mitch Georgiades</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corey Durdin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jack Whitlock</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tom Cochrane</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jason Horne-Francis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Joe Berry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Joe Richards</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Christian Moraes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Todd Marshall</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Darcy Byrne-Jones</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ewan Mackinlay</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jordon Sweet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zak Butters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ollie Wines</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jase Burgoyne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jacob Wehr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Willem Drew</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jackson Mead</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sydney swans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Charlie Curnow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Joel Amartey</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Logan McDonald</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Isaac Heeney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hayden McLean</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Malcolm Rosas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chad Warner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Caiden Cleary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Justin McInerney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">James Jordon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jake Lloyd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">James Rowbottom</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brodie Grundy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Angus Sheldrick</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jai Serong</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nick Blakey</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Matt Roberts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sam Wicks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">west coast eagles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jake Waterman</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jobe Shanahan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Milan Murdock</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Harvey Johnston</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Malakai Champion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cooper Duff-Tytler</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elliot Yeo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Harley Reid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Willem Duursma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bailey J. Williams</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tom Cole</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Liam Baker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bo Allan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tim Kelly</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ryan Maric</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hamish Davis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brady Hough</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tom McCarthy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">brisbane lions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Logan Morris</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Charlie Cameron</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zac Bailey</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kai Lohmann</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cam Rayner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conor McKenna</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sam Draper</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Will Ashcroft</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Levi Ashcroft</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lachie Neale</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jarrod Berry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">James Tunstill</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bruce Reville</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Darcy Fort</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Josh Dunkley</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jaspa Fletcher</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ty Gallop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Darcy Gardiner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">greater western sydney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Toby Greene</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jake Stringer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aaron Cadman</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Max Gruzewski</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phoenix Gothard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Callum Brown</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brent Daniels</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Toby Bedford</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stephen Coniglio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Toby McMullin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Harvey Thomas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finn Callaghan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conor Stone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leek Aleer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clayton Oliver</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kieren Briggs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Harry Himmelberg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Joe Fonti</t>
-  </si>
-  <si>
-    <t xml:space="preserve">richmond</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Liam Fawcett</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Noah Roberts-Thomson</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mykelti Lefau</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seth Campbell</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jasper Alger</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sam Cumming</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Steely Green</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tyler Sonsie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tim Taranto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Noah Balta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oliver Hayes-Brown</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dion Prestia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jack Ross</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Patrick Retschko</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jacob Hopper</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sam Banks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jayden Short</t>
-  </si>
-  <si>
-    <t xml:space="preserve">James Trezise</t>
-  </si>
-  <si>
-    <t xml:space="preserve">st kilda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Liam Ryan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cooper Sharman</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mitch Owens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Max Hall</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campbell Lake</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Darcy Wilson</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mattaes Phillipou</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mason Wood</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nasiah Wanganeen-Milera</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rowan Marshall</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tom De Koning</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hugo Garcia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anthony Caminiti</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bradley Hill</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jack Silvagni</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alix Tauru</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marcus Windhager</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jack Sinclair</t>
   </si>
 </sst>
 </file>
@@ -965,7 +851,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>6</v>
@@ -974,18 +860,18 @@
         <v>7</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>1.43</v>
+        <v>1.21</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>2.95</v>
+        <v>1.91</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>8.23</v>
+        <v>3.87</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>6</v>
@@ -994,18 +880,18 @@
         <v>8</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1.66</v>
+        <v>1.25</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>4.25</v>
+        <v>2.07</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>15.05</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>6</v>
@@ -1014,18 +900,18 @@
         <v>9</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1.71</v>
+        <v>1.25</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>4.54</v>
+        <v>2.1</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>16.76</v>
+        <v>4.61</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>6</v>
@@ -1034,18 +920,18 @@
         <v>10</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>1.85</v>
+        <v>1.45</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>5.48</v>
+        <v>3.05</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>22.72</v>
+        <v>8.72</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>6</v>
@@ -1054,18 +940,18 @@
         <v>11</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>1.91</v>
+        <v>1.49</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>5.9</v>
+        <v>3.3</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>25.58</v>
+        <v>9.93</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>6</v>
@@ -1074,18 +960,18 @@
         <v>12</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>2.12</v>
+        <v>1.59</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>7.43</v>
+        <v>3.82</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>36.95</v>
+        <v>12.66</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>6</v>
@@ -1094,18 +980,18 @@
         <v>13</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>2.13</v>
+        <v>1.66</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>7.54</v>
+        <v>4.25</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>37.87</v>
+        <v>15.04</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>6</v>
@@ -1114,18 +1000,18 @@
         <v>14</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>2.17</v>
+        <v>1.81</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>7.79</v>
+        <v>5.18</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>39.88</v>
+        <v>20.75</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>6</v>
@@ -1134,18 +1020,18 @@
         <v>15</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>2.86</v>
+        <v>1.86</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>14.31</v>
+        <v>5.54</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>103.6</v>
+        <v>23.13</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>6</v>
@@ -1154,18 +1040,18 @@
         <v>16</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>3.07</v>
+        <v>2.31</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>16.64</v>
+        <v>8.99</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>130.93</v>
+        <v>49.97</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>6</v>
@@ -1174,18 +1060,18 @@
         <v>17</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>3.29</v>
+        <v>3.09</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>19.28</v>
+        <v>16.92</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>164.47</v>
+        <v>134.36</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>6</v>
@@ -1194,18 +1080,18 @@
         <v>18</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>4.16</v>
+        <v>3.51</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>31.74</v>
+        <v>22.11</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>354.81</v>
+        <v>203.3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>6</v>
@@ -1214,18 +1100,18 @@
         <v>19</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>4.7</v>
+        <v>3.87</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>40.91</v>
+        <v>27.3</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>523.54</v>
+        <v>281.39</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>6</v>
@@ -1234,18 +1120,18 @@
         <v>20</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.6</v>
+        <v>3.98</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>58.8</v>
+        <v>28.96</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>911.46</v>
+        <v>308.23</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>6</v>
@@ -1254,18 +1140,18 @@
         <v>21</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>6.53</v>
+        <v>4.06</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>80.71</v>
+        <v>30.16</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>1476.51</v>
+        <v>327.92</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>6</v>
@@ -1274,18 +1160,18 @@
         <v>22</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>7.43</v>
+        <v>6.13</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>105.34</v>
+        <v>70.91</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>2213.19</v>
+        <v>1212.32</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>6</v>
@@ -1294,18 +1180,18 @@
         <v>23</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>7.93</v>
+        <v>6.46</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>120.4</v>
+        <v>78.97</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>2710.82</v>
+        <v>1428.4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>6</v>
@@ -1314,18 +1200,18 @@
         <v>24</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>9.25</v>
+        <v>10.34</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>164.87</v>
+        <v>206.8</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>4365.31</v>
+        <v>6151.44</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>25</v>
@@ -1334,18 +1220,18 @@
         <v>26</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>1.24</v>
+        <v>1.08</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>2.03</v>
+        <v>1.38</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>4.34</v>
+        <v>2.12</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>25</v>
@@ -1354,18 +1240,18 @@
         <v>27</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>1.25</v>
+        <v>1.27</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>2.08</v>
+        <v>2.17</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>4.51</v>
+        <v>4.86</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>25</v>
@@ -1374,18 +1260,18 @@
         <v>28</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>1.29</v>
+        <v>1.32</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>2.28</v>
+        <v>2.43</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>5.31</v>
+        <v>5.92</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>25</v>
@@ -1394,18 +1280,18 @@
         <v>29</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>1.33</v>
+        <v>1.34</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>2.46</v>
+        <v>2.5</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>6.06</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>25</v>
@@ -1414,18 +1300,18 @@
         <v>30</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>1.45</v>
+        <v>1.47</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>3.08</v>
+        <v>3.16</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>8.83</v>
+        <v>9.22</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>25</v>
@@ -1437,15 +1323,15 @@
         <v>1.51</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>3.36</v>
+        <v>3.4</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>10.24</v>
+        <v>10.41</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>25</v>
@@ -1454,18 +1340,18 @@
         <v>32</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>1.57</v>
+        <v>1.65</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>3.69</v>
+        <v>4.2</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>11.97</v>
+        <v>14.75</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>25</v>
@@ -1474,18 +1360,18 @@
         <v>33</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>1.58</v>
+        <v>1.71</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>3.76</v>
+        <v>4.53</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>12.33</v>
+        <v>16.74</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>25</v>
@@ -1494,18 +1380,18 @@
         <v>34</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>1.75</v>
+        <v>2.09</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>4.81</v>
+        <v>7.22</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>18.4</v>
+        <v>35.31</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>25</v>
@@ -1514,18 +1400,18 @@
         <v>35</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>1.77</v>
+        <v>2.12</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>4.94</v>
+        <v>7.45</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>19.23</v>
+        <v>37.14</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>25</v>
@@ -1534,18 +1420,18 @@
         <v>36</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>2.24</v>
+        <v>2.88</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>8.38</v>
+        <v>14.56</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>44.75</v>
+        <v>106.35</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>25</v>
@@ -1554,18 +1440,18 @@
         <v>37</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>2.59</v>
+        <v>3.02</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>11.55</v>
+        <v>16.1</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>74.07</v>
+        <v>124.43</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>25</v>
@@ -1574,18 +1460,18 @@
         <v>38</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>2.71</v>
+        <v>3.43</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>12.74</v>
+        <v>21.15</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>86.42</v>
+        <v>189.8</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>25</v>
@@ -1594,18 +1480,18 @@
         <v>39</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>3.32</v>
+        <v>5.55</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>19.71</v>
+        <v>57.77</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>170.21</v>
+        <v>887.2</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>25</v>
@@ -1614,18 +1500,18 @@
         <v>40</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>3.39</v>
+        <v>6.01</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>20.6</v>
+        <v>68.1</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>182.24</v>
+        <v>1139.93</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>25</v>
@@ -1634,18 +1520,18 @@
         <v>41</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>3.42</v>
+        <v>6.09</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>21</v>
+        <v>69.96</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>187.8</v>
+        <v>1187.87</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>25</v>
@@ -1654,18 +1540,18 @@
         <v>42</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>3.71</v>
+        <v>7.5</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>24.97</v>
+        <v>107.27</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>245.28</v>
+        <v>2274.96</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46186</v>
+        <v>46191</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>25</v>
@@ -1674,18 +1560,18 @@
         <v>43</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>4.98</v>
+        <v>7.88</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>46.12</v>
+        <v>118.97</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>628.95</v>
+        <v>2662.01</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>44</v>
@@ -1694,18 +1580,18 @@
         <v>45</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>1.19</v>
+        <v>1.1</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>1.83</v>
+        <v>1.45</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>3.61</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>44</v>
@@ -1714,18 +1600,18 @@
         <v>46</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>1.32</v>
+        <v>1.33</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>2.42</v>
+        <v>2.46</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>5.88</v>
+        <v>6.06</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>44</v>
@@ -1740,12 +1626,12 @@
         <v>2.72</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>7.19</v>
+        <v>7.16</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>44</v>
@@ -1754,18 +1640,18 @@
         <v>48</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>1.48</v>
+        <v>1.6</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>3.21</v>
+        <v>3.89</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>9.46</v>
+        <v>13.02</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>44</v>
@@ -1774,18 +1660,18 @@
         <v>49</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>1.48</v>
+        <v>1.66</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>3.22</v>
+        <v>4.26</v>
       </c>
       <c r="F42" s="3" t="n">
-        <v>9.51</v>
+        <v>15.14</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>44</v>
@@ -1794,18 +1680,18 @@
         <v>50</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>1.65</v>
+        <v>1.76</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>4.19</v>
+        <v>4.87</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>14.7</v>
+        <v>18.77</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>44</v>
@@ -1814,18 +1700,18 @@
         <v>51</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>1.96</v>
+        <v>1.78</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>6.21</v>
+        <v>4.99</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>27.76</v>
+        <v>19.56</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>44</v>
@@ -1834,18 +1720,18 @@
         <v>52</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>2.02</v>
+        <v>1.87</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>6.64</v>
+        <v>5.59</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>30.91</v>
+        <v>23.5</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>44</v>
@@ -1854,18 +1740,18 @@
         <v>53</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>2.34</v>
+        <v>2.03</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>9.29</v>
+        <v>6.71</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>52.65</v>
+        <v>31.45</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B47" s="3" t="s">
         <v>44</v>
@@ -1874,18 +1760,18 @@
         <v>54</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>2.57</v>
+        <v>2.66</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>11.31</v>
+        <v>12.23</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>71.73</v>
+        <v>81.03</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B48" s="3" t="s">
         <v>44</v>
@@ -1894,18 +1780,18 @@
         <v>55</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>3.04</v>
+        <v>2.71</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>16.38</v>
+        <v>12.71</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>127.78</v>
+        <v>86.09</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B49" s="3" t="s">
         <v>44</v>
@@ -1914,18 +1800,18 @@
         <v>56</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>3.31</v>
+        <v>3.11</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>19.63</v>
+        <v>17.12</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>169.21</v>
+        <v>136.84</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>44</v>
@@ -1934,18 +1820,18 @@
         <v>57</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>3.38</v>
+        <v>3.19</v>
       </c>
       <c r="E50" s="3" t="n">
-        <v>20.47</v>
+        <v>18.05</v>
       </c>
       <c r="F50" s="3" t="n">
-        <v>180.51</v>
+        <v>148.58</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>44</v>
@@ -1954,18 +1840,18 @@
         <v>58</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>3.47</v>
+        <v>3.48</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>21.59</v>
+        <v>21.72</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>196</v>
+        <v>197.78</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B52" s="3" t="s">
         <v>44</v>
@@ -1974,18 +1860,18 @@
         <v>59</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>3.82</v>
+        <v>4.36</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>26.48</v>
+        <v>34.91</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>268.47</v>
+        <v>410.63</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>44</v>
@@ -1994,18 +1880,18 @@
         <v>60</v>
       </c>
       <c r="D53" s="3" t="n">
-        <v>4.57</v>
+        <v>4.67</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>38.68</v>
+        <v>40.43</v>
       </c>
       <c r="F53" s="3" t="n">
-        <v>480.51</v>
+        <v>514.13</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B54" s="3" t="s">
         <v>44</v>
@@ -2014,18 +1900,18 @@
         <v>61</v>
       </c>
       <c r="D54" s="3" t="n">
-        <v>4.87</v>
+        <v>4.72</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>44.14</v>
+        <v>41.31</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>588.15</v>
+        <v>531.33</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B55" s="3" t="s">
         <v>44</v>
@@ -2034,18 +1920,18 @@
         <v>62</v>
       </c>
       <c r="D55" s="3" t="n">
-        <v>6.43</v>
+        <v>4.95</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>78.21</v>
+        <v>45.61</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>1407.53</v>
+        <v>618.36</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B56" s="3" t="s">
         <v>63</v>
@@ -2054,18 +1940,18 @@
         <v>64</v>
       </c>
       <c r="D56" s="3" t="n">
-        <v>1.18</v>
+        <v>1.17</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>1.8</v>
+        <v>1.76</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>3.48</v>
+        <v>3.36</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B57" s="3" t="s">
         <v>63</v>
@@ -2074,18 +1960,18 @@
         <v>65</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>1.57</v>
+        <v>1.22</v>
       </c>
       <c r="E57" s="3" t="n">
-        <v>3.7</v>
+        <v>1.95</v>
       </c>
       <c r="F57" s="3" t="n">
-        <v>12.01</v>
+        <v>4.02</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B58" s="3" t="s">
         <v>63</v>
@@ -2094,18 +1980,18 @@
         <v>66</v>
       </c>
       <c r="D58" s="3" t="n">
-        <v>1.57</v>
+        <v>1.26</v>
       </c>
       <c r="E58" s="3" t="n">
-        <v>3.74</v>
+        <v>2.15</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>12.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B59" s="3" t="s">
         <v>63</v>
@@ -2114,18 +2000,18 @@
         <v>67</v>
       </c>
       <c r="D59" s="3" t="n">
-        <v>1.61</v>
+        <v>1.43</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>3.94</v>
+        <v>2.94</v>
       </c>
       <c r="F59" s="3" t="n">
-        <v>13.29</v>
+        <v>8.18</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B60" s="3" t="s">
         <v>63</v>
@@ -2134,18 +2020,18 @@
         <v>68</v>
       </c>
       <c r="D60" s="3" t="n">
-        <v>1.73</v>
+        <v>1.45</v>
       </c>
       <c r="E60" s="3" t="n">
-        <v>4.67</v>
+        <v>3.09</v>
       </c>
       <c r="F60" s="3" t="n">
-        <v>17.59</v>
+        <v>8.87</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B61" s="3" t="s">
         <v>63</v>
@@ -2154,18 +2040,18 @@
         <v>69</v>
       </c>
       <c r="D61" s="3" t="n">
-        <v>1.9</v>
+        <v>1.53</v>
       </c>
       <c r="E61" s="3" t="n">
-        <v>5.79</v>
+        <v>3.48</v>
       </c>
       <c r="F61" s="3" t="n">
-        <v>24.84</v>
+        <v>10.82</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B62" s="3" t="s">
         <v>63</v>
@@ -2174,18 +2060,18 @@
         <v>70</v>
       </c>
       <c r="D62" s="3" t="n">
-        <v>1.91</v>
+        <v>1.59</v>
       </c>
       <c r="E62" s="3" t="n">
-        <v>5.9</v>
+        <v>3.85</v>
       </c>
       <c r="F62" s="3" t="n">
-        <v>25.58</v>
+        <v>12.78</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B63" s="3" t="s">
         <v>63</v>
@@ -2194,18 +2080,18 @@
         <v>71</v>
       </c>
       <c r="D63" s="3" t="n">
-        <v>2.24</v>
+        <v>2.6</v>
       </c>
       <c r="E63" s="3" t="n">
-        <v>8.44</v>
+        <v>11.7</v>
       </c>
       <c r="F63" s="3" t="n">
-        <v>45.21</v>
+        <v>75.6</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B64" s="3" t="s">
         <v>63</v>
@@ -2214,18 +2100,18 @@
         <v>72</v>
       </c>
       <c r="D64" s="3" t="n">
-        <v>2.33</v>
+        <v>2.72</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>9.2</v>
+        <v>12.82</v>
       </c>
       <c r="F64" s="3" t="n">
-        <v>51.88</v>
+        <v>87.19</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B65" s="3" t="s">
         <v>63</v>
@@ -2234,18 +2120,18 @@
         <v>73</v>
       </c>
       <c r="D65" s="3" t="n">
-        <v>2.53</v>
+        <v>2.88</v>
       </c>
       <c r="E65" s="3" t="n">
-        <v>11.02</v>
+        <v>14.55</v>
       </c>
       <c r="F65" s="3" t="n">
-        <v>68.89</v>
+        <v>106.24</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B66" s="3" t="s">
         <v>63</v>
@@ -2254,18 +2140,18 @@
         <v>74</v>
       </c>
       <c r="D66" s="3" t="n">
-        <v>2.97</v>
+        <v>2.92</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>15.57</v>
+        <v>14.94</v>
       </c>
       <c r="F66" s="3" t="n">
-        <v>118.15</v>
+        <v>110.76</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B67" s="3" t="s">
         <v>63</v>
@@ -2274,18 +2160,18 @@
         <v>75</v>
       </c>
       <c r="D67" s="3" t="n">
-        <v>3.63</v>
+        <v>3.14</v>
       </c>
       <c r="E67" s="3" t="n">
-        <v>23.78</v>
+        <v>17.45</v>
       </c>
       <c r="F67" s="3" t="n">
-        <v>227.45</v>
+        <v>140.98</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B68" s="3" t="s">
         <v>63</v>
@@ -2294,18 +2180,18 @@
         <v>76</v>
       </c>
       <c r="D68" s="3" t="n">
-        <v>3.92</v>
+        <v>3.19</v>
       </c>
       <c r="E68" s="3" t="n">
-        <v>27.96</v>
+        <v>18.06</v>
       </c>
       <c r="F68" s="3" t="n">
-        <v>291.89</v>
+        <v>148.66</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B69" s="3" t="s">
         <v>63</v>
@@ -2314,18 +2200,18 @@
         <v>77</v>
       </c>
       <c r="D69" s="3" t="n">
-        <v>4.45</v>
+        <v>3.42</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>36.49</v>
+        <v>20.98</v>
       </c>
       <c r="F69" s="3" t="n">
-        <v>439.46</v>
+        <v>187.5</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B70" s="3" t="s">
         <v>63</v>
@@ -2334,18 +2220,18 @@
         <v>78</v>
       </c>
       <c r="D70" s="3" t="n">
-        <v>4.49</v>
+        <v>4.08</v>
       </c>
       <c r="E70" s="3" t="n">
-        <v>37.16</v>
+        <v>30.42</v>
       </c>
       <c r="F70" s="3" t="n">
-        <v>451.93</v>
+        <v>332.34</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B71" s="3" t="s">
         <v>63</v>
@@ -2354,18 +2240,18 @@
         <v>79</v>
       </c>
       <c r="D71" s="3" t="n">
-        <v>5.11</v>
+        <v>5.76</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>48.63</v>
+        <v>62.49</v>
       </c>
       <c r="F71" s="3" t="n">
-        <v>681.89</v>
+        <v>999.93</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B72" s="3" t="s">
         <v>63</v>
@@ -2374,18 +2260,18 @@
         <v>80</v>
       </c>
       <c r="D72" s="3" t="n">
-        <v>5.62</v>
+        <v>5.94</v>
       </c>
       <c r="E72" s="3" t="n">
-        <v>59.34</v>
+        <v>66.46</v>
       </c>
       <c r="F72" s="3" t="n">
-        <v>924.14</v>
+        <v>1098.47</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="n">
-        <v>46186</v>
+        <v>46192</v>
       </c>
       <c r="B73" s="3" t="s">
         <v>63</v>
@@ -2394,18 +2280,18 @@
         <v>81</v>
       </c>
       <c r="D73" s="3" t="n">
-        <v>7.61</v>
+        <v>6.8</v>
       </c>
       <c r="E73" s="3" t="n">
-        <v>110.62</v>
+        <v>87.92</v>
       </c>
       <c r="F73" s="3" t="n">
-        <v>2383.77</v>
+        <v>1681.74</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B74" s="3" t="s">
         <v>82</v>
@@ -2414,18 +2300,18 @@
         <v>83</v>
       </c>
       <c r="D74" s="3" t="n">
-        <v>1.17</v>
+        <v>1.19</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>1.73</v>
+        <v>1.84</v>
       </c>
       <c r="F74" s="3" t="n">
-        <v>3.25</v>
+        <v>3.63</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B75" s="3" t="s">
         <v>82</v>
@@ -2434,18 +2320,18 @@
         <v>84</v>
       </c>
       <c r="D75" s="3" t="n">
-        <v>1.3</v>
+        <v>1.26</v>
       </c>
       <c r="E75" s="3" t="n">
-        <v>2.33</v>
+        <v>2.15</v>
       </c>
       <c r="F75" s="3" t="n">
-        <v>5.51</v>
+        <v>4.78</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B76" s="3" t="s">
         <v>82</v>
@@ -2454,18 +2340,18 @@
         <v>85</v>
       </c>
       <c r="D76" s="3" t="n">
-        <v>1.38</v>
+        <v>1.27</v>
       </c>
       <c r="E76" s="3" t="n">
-        <v>2.71</v>
+        <v>2.17</v>
       </c>
       <c r="F76" s="3" t="n">
-        <v>7.13</v>
+        <v>4.85</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B77" s="3" t="s">
         <v>82</v>
@@ -2474,18 +2360,18 @@
         <v>86</v>
       </c>
       <c r="D77" s="3" t="n">
-        <v>1.39</v>
+        <v>1.35</v>
       </c>
       <c r="E77" s="3" t="n">
-        <v>2.78</v>
+        <v>2.56</v>
       </c>
       <c r="F77" s="3" t="n">
-        <v>7.45</v>
+        <v>6.47</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B78" s="3" t="s">
         <v>82</v>
@@ -2494,18 +2380,18 @@
         <v>87</v>
       </c>
       <c r="D78" s="3" t="n">
-        <v>1.43</v>
+        <v>1.49</v>
       </c>
       <c r="E78" s="3" t="n">
-        <v>2.98</v>
+        <v>3.25</v>
       </c>
       <c r="F78" s="3" t="n">
-        <v>8.38</v>
+        <v>9.7</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B79" s="3" t="s">
         <v>82</v>
@@ -2514,18 +2400,18 @@
         <v>88</v>
       </c>
       <c r="D79" s="3" t="n">
-        <v>1.53</v>
+        <v>1.59</v>
       </c>
       <c r="E79" s="3" t="n">
-        <v>3.47</v>
+        <v>3.81</v>
       </c>
       <c r="F79" s="3" t="n">
-        <v>10.81</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B80" s="3" t="s">
         <v>82</v>
@@ -2534,18 +2420,18 @@
         <v>89</v>
       </c>
       <c r="D80" s="3" t="n">
-        <v>1.56</v>
+        <v>1.79</v>
       </c>
       <c r="E80" s="3" t="n">
-        <v>3.68</v>
+        <v>5.08</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>11.88</v>
+        <v>20.13</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B81" s="3" t="s">
         <v>82</v>
@@ -2554,18 +2440,18 @@
         <v>90</v>
       </c>
       <c r="D81" s="3" t="n">
-        <v>2.23</v>
+        <v>1.8</v>
       </c>
       <c r="E81" s="3" t="n">
-        <v>8.28</v>
+        <v>5.11</v>
       </c>
       <c r="F81" s="3" t="n">
-        <v>43.86</v>
+        <v>20.33</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B82" s="3" t="s">
         <v>82</v>
@@ -2574,18 +2460,18 @@
         <v>91</v>
       </c>
       <c r="D82" s="3" t="n">
-        <v>2.31</v>
+        <v>1.95</v>
       </c>
       <c r="E82" s="3" t="n">
-        <v>8.96</v>
+        <v>6.18</v>
       </c>
       <c r="F82" s="3" t="n">
-        <v>49.74</v>
+        <v>27.54</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B83" s="3" t="s">
         <v>82</v>
@@ -2594,18 +2480,18 @@
         <v>92</v>
       </c>
       <c r="D83" s="3" t="n">
-        <v>2.46</v>
+        <v>1.96</v>
       </c>
       <c r="E83" s="3" t="n">
-        <v>10.36</v>
+        <v>6.23</v>
       </c>
       <c r="F83" s="3" t="n">
-        <v>62.53</v>
+        <v>27.93</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B84" s="3" t="s">
         <v>82</v>
@@ -2614,18 +2500,18 @@
         <v>93</v>
       </c>
       <c r="D84" s="3" t="n">
-        <v>2.52</v>
+        <v>2.55</v>
       </c>
       <c r="E84" s="3" t="n">
-        <v>10.87</v>
+        <v>11.16</v>
       </c>
       <c r="F84" s="3" t="n">
-        <v>67.43</v>
+        <v>70.26</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B85" s="3" t="s">
         <v>82</v>
@@ -2634,18 +2520,18 @@
         <v>94</v>
       </c>
       <c r="D85" s="3" t="n">
-        <v>2.74</v>
+        <v>2.73</v>
       </c>
       <c r="E85" s="3" t="n">
-        <v>13.02</v>
+        <v>12.98</v>
       </c>
       <c r="F85" s="3" t="n">
-        <v>89.39</v>
+        <v>88.92</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B86" s="3" t="s">
         <v>82</v>
@@ -2654,18 +2540,18 @@
         <v>95</v>
       </c>
       <c r="D86" s="3" t="n">
-        <v>3.2</v>
+        <v>2.92</v>
       </c>
       <c r="E86" s="3" t="n">
-        <v>18.19</v>
+        <v>14.95</v>
       </c>
       <c r="F86" s="3" t="n">
-        <v>150.39</v>
+        <v>110.92</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B87" s="3" t="s">
         <v>82</v>
@@ -2674,18 +2560,18 @@
         <v>96</v>
       </c>
       <c r="D87" s="3" t="n">
-        <v>3.88</v>
+        <v>3.1</v>
       </c>
       <c r="E87" s="3" t="n">
-        <v>27.33</v>
+        <v>17.07</v>
       </c>
       <c r="F87" s="3" t="n">
-        <v>281.84</v>
+        <v>136.19</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B88" s="3" t="s">
         <v>82</v>
@@ -2694,18 +2580,18 @@
         <v>97</v>
       </c>
       <c r="D88" s="3" t="n">
-        <v>3.92</v>
+        <v>3.76</v>
       </c>
       <c r="E88" s="3" t="n">
-        <v>27.92</v>
+        <v>25.63</v>
       </c>
       <c r="F88" s="3" t="n">
-        <v>291.37</v>
+        <v>255.36</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B89" s="3" t="s">
         <v>82</v>
@@ -2714,18 +2600,18 @@
         <v>98</v>
       </c>
       <c r="D89" s="3" t="n">
-        <v>4.76</v>
+        <v>7.03</v>
       </c>
       <c r="E89" s="3" t="n">
-        <v>42.07</v>
+        <v>94.15</v>
       </c>
       <c r="F89" s="3" t="n">
-        <v>546.37</v>
+        <v>1866.18</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B90" s="3" t="s">
         <v>82</v>
@@ -2734,18 +2620,18 @@
         <v>99</v>
       </c>
       <c r="D90" s="3" t="n">
-        <v>5.59</v>
+        <v>8.47</v>
       </c>
       <c r="E90" s="3" t="n">
-        <v>58.69</v>
+        <v>137.6</v>
       </c>
       <c r="F90" s="3" t="n">
-        <v>908.84</v>
+        <v>3319.31</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B91" s="3" t="s">
         <v>82</v>
@@ -2754,18 +2640,18 @@
         <v>100</v>
       </c>
       <c r="D91" s="3" t="n">
-        <v>7.3</v>
+        <v>8.96</v>
       </c>
       <c r="E91" s="3" t="n">
-        <v>101.46</v>
+        <v>154.35</v>
       </c>
       <c r="F91" s="3" t="n">
-        <v>2090.43</v>
+        <v>3950.34</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B92" s="3" t="s">
         <v>101</v>
@@ -2774,18 +2660,18 @@
         <v>102</v>
       </c>
       <c r="D92" s="3" t="n">
-        <v>1.25</v>
+        <v>1.4</v>
       </c>
       <c r="E92" s="3" t="n">
-        <v>2.09</v>
+        <v>2.82</v>
       </c>
       <c r="F92" s="3" t="n">
-        <v>4.55</v>
+        <v>7.64</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B93" s="3" t="s">
         <v>101</v>
@@ -2794,18 +2680,18 @@
         <v>103</v>
       </c>
       <c r="D93" s="3" t="n">
-        <v>1.56</v>
+        <v>1.59</v>
       </c>
       <c r="E93" s="3" t="n">
-        <v>3.68</v>
+        <v>3.86</v>
       </c>
       <c r="F93" s="3" t="n">
-        <v>11.89</v>
+        <v>12.84</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B94" s="3" t="s">
         <v>101</v>
@@ -2814,18 +2700,18 @@
         <v>104</v>
       </c>
       <c r="D94" s="3" t="n">
-        <v>1.64</v>
+        <v>1.7</v>
       </c>
       <c r="E94" s="3" t="n">
-        <v>4.11</v>
+        <v>4.47</v>
       </c>
       <c r="F94" s="3" t="n">
-        <v>14.24</v>
+        <v>16.36</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B95" s="3" t="s">
         <v>101</v>
@@ -2834,18 +2720,18 @@
         <v>105</v>
       </c>
       <c r="D95" s="3" t="n">
-        <v>1.85</v>
+        <v>1.78</v>
       </c>
       <c r="E95" s="3" t="n">
-        <v>5.48</v>
+        <v>5.02</v>
       </c>
       <c r="F95" s="3" t="n">
-        <v>22.73</v>
+        <v>19.74</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B96" s="3" t="s">
         <v>101</v>
@@ -2854,18 +2740,18 @@
         <v>106</v>
       </c>
       <c r="D96" s="3" t="n">
-        <v>1.92</v>
+        <v>1.81</v>
       </c>
       <c r="E96" s="3" t="n">
-        <v>5.97</v>
+        <v>5.22</v>
       </c>
       <c r="F96" s="3" t="n">
-        <v>26.05</v>
+        <v>20.99</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B97" s="3" t="s">
         <v>101</v>
@@ -2874,18 +2760,18 @@
         <v>107</v>
       </c>
       <c r="D97" s="3" t="n">
-        <v>2.05</v>
+        <v>1.84</v>
       </c>
       <c r="E97" s="3" t="n">
-        <v>6.88</v>
+        <v>5.36</v>
       </c>
       <c r="F97" s="3" t="n">
-        <v>32.73</v>
+        <v>21.97</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B98" s="3" t="s">
         <v>101</v>
@@ -2894,18 +2780,18 @@
         <v>108</v>
       </c>
       <c r="D98" s="3" t="n">
-        <v>2.23</v>
+        <v>1.91</v>
       </c>
       <c r="E98" s="3" t="n">
-        <v>8.34</v>
+        <v>5.89</v>
       </c>
       <c r="F98" s="3" t="n">
-        <v>44.41</v>
+        <v>25.51</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B99" s="3" t="s">
         <v>101</v>
@@ -2914,18 +2800,18 @@
         <v>109</v>
       </c>
       <c r="D99" s="3" t="n">
-        <v>2.32</v>
+        <v>1.92</v>
       </c>
       <c r="E99" s="3" t="n">
-        <v>9.08</v>
+        <v>5.92</v>
       </c>
       <c r="F99" s="3" t="n">
-        <v>50.82</v>
+        <v>25.71</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B100" s="3" t="s">
         <v>101</v>
@@ -2934,18 +2820,18 @@
         <v>110</v>
       </c>
       <c r="D100" s="3" t="n">
-        <v>2.55</v>
+        <v>2</v>
       </c>
       <c r="E100" s="3" t="n">
-        <v>11.16</v>
+        <v>6.54</v>
       </c>
       <c r="F100" s="3" t="n">
-        <v>70.25</v>
+        <v>30.2</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B101" s="3" t="s">
         <v>101</v>
@@ -2954,18 +2840,18 @@
         <v>111</v>
       </c>
       <c r="D101" s="3" t="n">
-        <v>2.87</v>
+        <v>2.44</v>
       </c>
       <c r="E101" s="3" t="n">
-        <v>14.39</v>
+        <v>10.1</v>
       </c>
       <c r="F101" s="3" t="n">
-        <v>104.46</v>
+        <v>60.06</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B102" s="3" t="s">
         <v>101</v>
@@ -2974,18 +2860,18 @@
         <v>112</v>
       </c>
       <c r="D102" s="3" t="n">
-        <v>2.87</v>
+        <v>2.71</v>
       </c>
       <c r="E102" s="3" t="n">
-        <v>14.39</v>
+        <v>12.77</v>
       </c>
       <c r="F102" s="3" t="n">
-        <v>104.52</v>
+        <v>86.73</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B103" s="3" t="s">
         <v>101</v>
@@ -2994,18 +2880,18 @@
         <v>113</v>
       </c>
       <c r="D103" s="3" t="n">
-        <v>3.8</v>
+        <v>3.85</v>
       </c>
       <c r="E103" s="3" t="n">
-        <v>26.29</v>
+        <v>26.97</v>
       </c>
       <c r="F103" s="3" t="n">
-        <v>265.5</v>
+        <v>276.15</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B104" s="3" t="s">
         <v>101</v>
@@ -3014,18 +2900,18 @@
         <v>114</v>
       </c>
       <c r="D104" s="3" t="n">
-        <v>3.98</v>
+        <v>3.87</v>
       </c>
       <c r="E104" s="3" t="n">
-        <v>28.91</v>
+        <v>27.21</v>
       </c>
       <c r="F104" s="3" t="n">
-        <v>307.36</v>
+        <v>280</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B105" s="3" t="s">
         <v>101</v>
@@ -3034,18 +2920,18 @@
         <v>115</v>
       </c>
       <c r="D105" s="3" t="n">
-        <v>4.65</v>
+        <v>4</v>
       </c>
       <c r="E105" s="3" t="n">
-        <v>40.09</v>
+        <v>29.23</v>
       </c>
       <c r="F105" s="3" t="n">
-        <v>507.62</v>
+        <v>312.5</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B106" s="3" t="s">
         <v>101</v>
@@ -3054,18 +2940,18 @@
         <v>116</v>
       </c>
       <c r="D106" s="3" t="n">
-        <v>4.81</v>
+        <v>4.45</v>
       </c>
       <c r="E106" s="3" t="n">
-        <v>42.94</v>
+        <v>36.47</v>
       </c>
       <c r="F106" s="3" t="n">
-        <v>563.89</v>
+        <v>438.95</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B107" s="3" t="s">
         <v>101</v>
@@ -3074,18 +2960,18 @@
         <v>117</v>
       </c>
       <c r="D107" s="3" t="n">
-        <v>5.35</v>
+        <v>4.5</v>
       </c>
       <c r="E107" s="3" t="n">
-        <v>53.63</v>
+        <v>37.36</v>
       </c>
       <c r="F107" s="3" t="n">
-        <v>791.96</v>
+        <v>455.61</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B108" s="3" t="s">
         <v>101</v>
@@ -3094,18 +2980,18 @@
         <v>118</v>
       </c>
       <c r="D108" s="3" t="n">
-        <v>9.96</v>
+        <v>9.04</v>
       </c>
       <c r="E108" s="3" t="n">
-        <v>191.62</v>
+        <v>157.36</v>
       </c>
       <c r="F108" s="3" t="n">
-        <v>5481.19</v>
+        <v>4067.67</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="n">
-        <v>46186</v>
+        <v>46193</v>
       </c>
       <c r="B109" s="3" t="s">
         <v>101</v>
@@ -3114,18 +3000,18 @@
         <v>119</v>
       </c>
       <c r="D109" s="3" t="n">
-        <v>13.04</v>
+        <v>12.71</v>
       </c>
       <c r="E109" s="3" t="n">
-        <v>331.25</v>
+        <v>314.37</v>
       </c>
       <c r="F109" s="3" t="n">
-        <v>12538.11</v>
+        <v>11586.34</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B110" s="3" t="s">
         <v>120</v>
@@ -3134,18 +3020,18 @@
         <v>121</v>
       </c>
       <c r="D110" s="3" t="n">
-        <v>1.1</v>
+        <v>1.18</v>
       </c>
       <c r="E110" s="3" t="n">
-        <v>1.43</v>
+        <v>1.8</v>
       </c>
       <c r="F110" s="3" t="n">
-        <v>2.28</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B111" s="3" t="s">
         <v>120</v>
@@ -3154,18 +3040,18 @@
         <v>122</v>
       </c>
       <c r="D111" s="3" t="n">
-        <v>1.13</v>
+        <v>1.19</v>
       </c>
       <c r="E111" s="3" t="n">
-        <v>1.59</v>
+        <v>1.85</v>
       </c>
       <c r="F111" s="3" t="n">
-        <v>2.78</v>
+        <v>3.66</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B112" s="3" t="s">
         <v>120</v>
@@ -3177,15 +3063,15 @@
         <v>1.22</v>
       </c>
       <c r="E112" s="3" t="n">
-        <v>1.95</v>
+        <v>1.96</v>
       </c>
       <c r="F112" s="3" t="n">
-        <v>4.02</v>
+        <v>4.06</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B113" s="3" t="s">
         <v>120</v>
@@ -3194,18 +3080,18 @@
         <v>124</v>
       </c>
       <c r="D113" s="3" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="E113" s="3" t="n">
-        <v>1.98</v>
+        <v>2.21</v>
       </c>
       <c r="F113" s="3" t="n">
-        <v>4.13</v>
+        <v>5.03</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B114" s="3" t="s">
         <v>120</v>
@@ -3214,18 +3100,18 @@
         <v>125</v>
       </c>
       <c r="D114" s="3" t="n">
-        <v>1.28</v>
+        <v>1.36</v>
       </c>
       <c r="E114" s="3" t="n">
-        <v>2.21</v>
+        <v>2.61</v>
       </c>
       <c r="F114" s="3" t="n">
-        <v>5.02</v>
+        <v>6.71</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B115" s="3" t="s">
         <v>120</v>
@@ -3234,18 +3120,18 @@
         <v>126</v>
       </c>
       <c r="D115" s="3" t="n">
-        <v>1.57</v>
+        <v>1.41</v>
       </c>
       <c r="E115" s="3" t="n">
-        <v>3.72</v>
+        <v>2.88</v>
       </c>
       <c r="F115" s="3" t="n">
-        <v>12.09</v>
+        <v>7.91</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B116" s="3" t="s">
         <v>120</v>
@@ -3254,18 +3140,18 @@
         <v>127</v>
       </c>
       <c r="D116" s="3" t="n">
-        <v>1.79</v>
+        <v>1.43</v>
       </c>
       <c r="E116" s="3" t="n">
-        <v>5.03</v>
+        <v>2.94</v>
       </c>
       <c r="F116" s="3" t="n">
-        <v>19.83</v>
+        <v>8.17</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B117" s="3" t="s">
         <v>120</v>
@@ -3274,18 +3160,18 @@
         <v>128</v>
       </c>
       <c r="D117" s="3" t="n">
-        <v>2.24</v>
+        <v>1.62</v>
       </c>
       <c r="E117" s="3" t="n">
-        <v>8.42</v>
+        <v>3.98</v>
       </c>
       <c r="F117" s="3" t="n">
-        <v>45.1</v>
+        <v>13.51</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B118" s="3" t="s">
         <v>120</v>
@@ -3294,18 +3180,18 @@
         <v>129</v>
       </c>
       <c r="D118" s="3" t="n">
-        <v>2.36</v>
+        <v>2.01</v>
       </c>
       <c r="E118" s="3" t="n">
-        <v>9.39</v>
+        <v>6.63</v>
       </c>
       <c r="F118" s="3" t="n">
-        <v>53.58</v>
+        <v>30.82</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B119" s="3" t="s">
         <v>120</v>
@@ -3314,18 +3200,18 @@
         <v>130</v>
       </c>
       <c r="D119" s="3" t="n">
-        <v>2.69</v>
+        <v>2.07</v>
       </c>
       <c r="E119" s="3" t="n">
-        <v>12.57</v>
+        <v>7.01</v>
       </c>
       <c r="F119" s="3" t="n">
-        <v>84.64</v>
+        <v>33.69</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B120" s="3" t="s">
         <v>120</v>
@@ -3334,18 +3220,18 @@
         <v>131</v>
       </c>
       <c r="D120" s="3" t="n">
-        <v>2.74</v>
+        <v>2.44</v>
       </c>
       <c r="E120" s="3" t="n">
-        <v>13.05</v>
+        <v>10.11</v>
       </c>
       <c r="F120" s="3" t="n">
-        <v>89.74</v>
+        <v>60.13</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B121" s="3" t="s">
         <v>120</v>
@@ -3354,18 +3240,18 @@
         <v>132</v>
       </c>
       <c r="D121" s="3" t="n">
-        <v>2.79</v>
+        <v>3.08</v>
       </c>
       <c r="E121" s="3" t="n">
-        <v>13.61</v>
+        <v>16.73</v>
       </c>
       <c r="F121" s="3" t="n">
-        <v>95.81</v>
+        <v>132.09</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B122" s="3" t="s">
         <v>120</v>
@@ -3374,18 +3260,18 @@
         <v>133</v>
       </c>
       <c r="D122" s="3" t="n">
-        <v>2.88</v>
+        <v>3.64</v>
       </c>
       <c r="E122" s="3" t="n">
-        <v>14.49</v>
+        <v>24</v>
       </c>
       <c r="F122" s="3" t="n">
-        <v>105.59</v>
+        <v>230.76</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B123" s="3" t="s">
         <v>120</v>
@@ -3394,18 +3280,18 @@
         <v>134</v>
       </c>
       <c r="D123" s="3" t="n">
-        <v>3</v>
+        <v>3.87</v>
       </c>
       <c r="E123" s="3" t="n">
-        <v>15.85</v>
+        <v>27.3</v>
       </c>
       <c r="F123" s="3" t="n">
-        <v>121.35</v>
+        <v>281.46</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B124" s="3" t="s">
         <v>120</v>
@@ -3414,18 +3300,18 @@
         <v>135</v>
       </c>
       <c r="D124" s="3" t="n">
-        <v>3.75</v>
+        <v>4.08</v>
       </c>
       <c r="E124" s="3" t="n">
-        <v>25.54</v>
+        <v>30.41</v>
       </c>
       <c r="F124" s="3" t="n">
-        <v>254.01</v>
+        <v>332.26</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B125" s="3" t="s">
         <v>120</v>
@@ -3434,18 +3320,18 @@
         <v>136</v>
       </c>
       <c r="D125" s="3" t="n">
-        <v>3.96</v>
+        <v>4.21</v>
       </c>
       <c r="E125" s="3" t="n">
-        <v>28.53</v>
+        <v>32.55</v>
       </c>
       <c r="F125" s="3" t="n">
-        <v>301.08</v>
+        <v>368.82</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B126" s="3" t="s">
         <v>120</v>
@@ -3454,18 +3340,18 @@
         <v>137</v>
       </c>
       <c r="D126" s="3" t="n">
-        <v>4.37</v>
+        <v>6.35</v>
       </c>
       <c r="E126" s="3" t="n">
-        <v>35.15</v>
+        <v>76.27</v>
       </c>
       <c r="F126" s="3" t="n">
-        <v>414.95</v>
+        <v>1354.59</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B127" s="3" t="s">
         <v>120</v>
@@ -3474,18 +3360,18 @@
         <v>138</v>
       </c>
       <c r="D127" s="3" t="n">
-        <v>5.02</v>
+        <v>11.52</v>
       </c>
       <c r="E127" s="3" t="n">
-        <v>46.87</v>
+        <v>257.55</v>
       </c>
       <c r="F127" s="3" t="n">
-        <v>644.7</v>
+        <v>8572.97</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B128" s="3" t="s">
         <v>139</v>
@@ -3494,18 +3380,18 @@
         <v>140</v>
       </c>
       <c r="D128" s="3" t="n">
-        <v>1.22</v>
+        <v>1.37</v>
       </c>
       <c r="E128" s="3" t="n">
-        <v>1.95</v>
+        <v>2.67</v>
       </c>
       <c r="F128" s="3" t="n">
-        <v>4.04</v>
+        <v>6.96</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B129" s="3" t="s">
         <v>139</v>
@@ -3514,18 +3400,18 @@
         <v>141</v>
       </c>
       <c r="D129" s="3" t="n">
-        <v>1.23</v>
+        <v>1.39</v>
       </c>
       <c r="E129" s="3" t="n">
-        <v>2</v>
+        <v>2.74</v>
       </c>
       <c r="F129" s="3" t="n">
-        <v>4.23</v>
+        <v>7.27</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B130" s="3" t="s">
         <v>139</v>
@@ -3534,18 +3420,18 @@
         <v>142</v>
       </c>
       <c r="D130" s="3" t="n">
-        <v>1.26</v>
+        <v>1.45</v>
       </c>
       <c r="E130" s="3" t="n">
-        <v>2.13</v>
+        <v>3.06</v>
       </c>
       <c r="F130" s="3" t="n">
-        <v>4.72</v>
+        <v>8.74</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B131" s="3" t="s">
         <v>139</v>
@@ -3554,18 +3440,18 @@
         <v>143</v>
       </c>
       <c r="D131" s="3" t="n">
-        <v>1.32</v>
+        <v>1.5</v>
       </c>
       <c r="E131" s="3" t="n">
-        <v>2.42</v>
+        <v>3.32</v>
       </c>
       <c r="F131" s="3" t="n">
-        <v>5.89</v>
+        <v>10.05</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B132" s="3" t="s">
         <v>139</v>
@@ -3574,18 +3460,18 @@
         <v>144</v>
       </c>
       <c r="D132" s="3" t="n">
-        <v>1.42</v>
+        <v>1.66</v>
       </c>
       <c r="E132" s="3" t="n">
-        <v>2.89</v>
+        <v>4.26</v>
       </c>
       <c r="F132" s="3" t="n">
-        <v>7.94</v>
+        <v>15.09</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B133" s="3" t="s">
         <v>139</v>
@@ -3594,18 +3480,18 @@
         <v>145</v>
       </c>
       <c r="D133" s="3" t="n">
-        <v>1.48</v>
+        <v>1.73</v>
       </c>
       <c r="E133" s="3" t="n">
-        <v>3.2</v>
+        <v>4.69</v>
       </c>
       <c r="F133" s="3" t="n">
-        <v>9.42</v>
+        <v>17.67</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B134" s="3" t="s">
         <v>139</v>
@@ -3614,18 +3500,18 @@
         <v>146</v>
       </c>
       <c r="D134" s="3" t="n">
-        <v>1.49</v>
+        <v>1.81</v>
       </c>
       <c r="E134" s="3" t="n">
-        <v>3.26</v>
+        <v>5.2</v>
       </c>
       <c r="F134" s="3" t="n">
-        <v>9.73</v>
+        <v>20.86</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B135" s="3" t="s">
         <v>139</v>
@@ -3634,18 +3520,18 @@
         <v>147</v>
       </c>
       <c r="D135" s="3" t="n">
-        <v>1.7</v>
+        <v>1.83</v>
       </c>
       <c r="E135" s="3" t="n">
-        <v>4.47</v>
+        <v>5.3</v>
       </c>
       <c r="F135" s="3" t="n">
-        <v>16.33</v>
+        <v>21.52</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B136" s="3" t="s">
         <v>139</v>
@@ -3654,18 +3540,18 @@
         <v>148</v>
       </c>
       <c r="D136" s="3" t="n">
-        <v>2.14</v>
+        <v>2.06</v>
       </c>
       <c r="E136" s="3" t="n">
-        <v>7.56</v>
+        <v>6.93</v>
       </c>
       <c r="F136" s="3" t="n">
-        <v>38.03</v>
+        <v>33.1</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B137" s="3" t="s">
         <v>139</v>
@@ -3674,18 +3560,18 @@
         <v>149</v>
       </c>
       <c r="D137" s="3" t="n">
-        <v>2.19</v>
+        <v>2.07</v>
       </c>
       <c r="E137" s="3" t="n">
-        <v>8.02</v>
+        <v>7.08</v>
       </c>
       <c r="F137" s="3" t="n">
-        <v>41.77</v>
+        <v>34.24</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B138" s="3" t="s">
         <v>139</v>
@@ -3694,18 +3580,18 @@
         <v>150</v>
       </c>
       <c r="D138" s="3" t="n">
-        <v>2.59</v>
+        <v>2.68</v>
       </c>
       <c r="E138" s="3" t="n">
-        <v>11.55</v>
+        <v>12.49</v>
       </c>
       <c r="F138" s="3" t="n">
-        <v>74.16</v>
+        <v>83.79</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B139" s="3" t="s">
         <v>139</v>
@@ -3714,18 +3600,18 @@
         <v>151</v>
       </c>
       <c r="D139" s="3" t="n">
-        <v>3.29</v>
+        <v>3.13</v>
       </c>
       <c r="E139" s="3" t="n">
-        <v>19.29</v>
+        <v>17.37</v>
       </c>
       <c r="F139" s="3" t="n">
-        <v>164.6</v>
+        <v>139.92</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B140" s="3" t="s">
         <v>139</v>
@@ -3734,18 +3620,18 @@
         <v>152</v>
       </c>
       <c r="D140" s="3" t="n">
-        <v>3.91</v>
+        <v>3.28</v>
       </c>
       <c r="E140" s="3" t="n">
-        <v>27.9</v>
+        <v>19.22</v>
       </c>
       <c r="F140" s="3" t="n">
-        <v>291.02</v>
+        <v>163.77</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B141" s="3" t="s">
         <v>139</v>
@@ -3754,18 +3640,18 @@
         <v>153</v>
       </c>
       <c r="D141" s="3" t="n">
-        <v>4.16</v>
+        <v>4.07</v>
       </c>
       <c r="E141" s="3" t="n">
-        <v>31.73</v>
+        <v>30.25</v>
       </c>
       <c r="F141" s="3" t="n">
-        <v>354.66</v>
+        <v>329.47</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B142" s="3" t="s">
         <v>139</v>
@@ -3774,18 +3660,18 @@
         <v>154</v>
       </c>
       <c r="D142" s="3" t="n">
-        <v>4.38</v>
+        <v>4.14</v>
       </c>
       <c r="E142" s="3" t="n">
-        <v>35.35</v>
+        <v>31.46</v>
       </c>
       <c r="F142" s="3" t="n">
-        <v>418.49</v>
+        <v>349.91</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B143" s="3" t="s">
         <v>139</v>
@@ -3794,18 +3680,18 @@
         <v>155</v>
       </c>
       <c r="D143" s="3" t="n">
-        <v>4.53</v>
+        <v>4.2</v>
       </c>
       <c r="E143" s="3" t="n">
-        <v>37.86</v>
+        <v>32.32</v>
       </c>
       <c r="F143" s="3" t="n">
-        <v>464.93</v>
+        <v>364.71</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B144" s="3" t="s">
         <v>139</v>
@@ -3814,18 +3700,18 @@
         <v>156</v>
       </c>
       <c r="D144" s="3" t="n">
-        <v>6.83</v>
+        <v>4.55</v>
       </c>
       <c r="E144" s="3" t="n">
-        <v>88.7</v>
+        <v>38.29</v>
       </c>
       <c r="F144" s="3" t="n">
-        <v>1704.49</v>
+        <v>473.14</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
-        <v>46187</v>
+        <v>46193</v>
       </c>
       <c r="B145" s="3" t="s">
         <v>139</v>
@@ -3834,733 +3720,13 @@
         <v>157</v>
       </c>
       <c r="D145" s="3" t="n">
-        <v>12.47</v>
+        <v>6.18</v>
       </c>
       <c r="E145" s="3" t="n">
-        <v>302.65</v>
+        <v>72.04</v>
       </c>
       <c r="F145" s="3" t="n">
-        <v>10940.12</v>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B146" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C146" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="D146" s="3" t="n">
-        <v>1.57</v>
-      </c>
-      <c r="E146" s="3" t="n">
-        <v>3.73</v>
-      </c>
-      <c r="F146" s="3" t="n">
-        <v>12.14</v>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B147" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C147" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="D147" s="3" t="n">
-        <v>1.64</v>
-      </c>
-      <c r="E147" s="3" t="n">
-        <v>4.15</v>
-      </c>
-      <c r="F147" s="3" t="n">
-        <v>14.46</v>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B148" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C148" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="D148" s="3" t="n">
-        <v>1.67</v>
-      </c>
-      <c r="E148" s="3" t="n">
-        <v>4.28</v>
-      </c>
-      <c r="F148" s="3" t="n">
-        <v>15.25</v>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B149" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C149" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="D149" s="3" t="n">
-        <v>1.74</v>
-      </c>
-      <c r="E149" s="3" t="n">
-        <v>4.72</v>
-      </c>
-      <c r="F149" s="3" t="n">
-        <v>17.86</v>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B150" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C150" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="D150" s="3" t="n">
-        <v>1.77</v>
-      </c>
-      <c r="E150" s="3" t="n">
-        <v>4.93</v>
-      </c>
-      <c r="F150" s="3" t="n">
-        <v>19.17</v>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B151" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C151" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="D151" s="3" t="n">
-        <v>1.83</v>
-      </c>
-      <c r="E151" s="3" t="n">
-        <v>5.35</v>
-      </c>
-      <c r="F151" s="3" t="n">
-        <v>21.88</v>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B152" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C152" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="D152" s="3" t="n">
-        <v>1.88</v>
-      </c>
-      <c r="E152" s="3" t="n">
-        <v>5.67</v>
-      </c>
-      <c r="F152" s="3" t="n">
-        <v>24.03</v>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B153" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C153" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="D153" s="3" t="n">
-        <v>2.72</v>
-      </c>
-      <c r="E153" s="3" t="n">
-        <v>12.87</v>
-      </c>
-      <c r="F153" s="3" t="n">
-        <v>87.76</v>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B154" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C154" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="D154" s="3" t="n">
-        <v>2.87</v>
-      </c>
-      <c r="E154" s="3" t="n">
-        <v>14.39</v>
-      </c>
-      <c r="F154" s="3" t="n">
-        <v>104.42</v>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B155" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C155" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="D155" s="3" t="n">
-        <v>3.83</v>
-      </c>
-      <c r="E155" s="3" t="n">
-        <v>26.71</v>
-      </c>
-      <c r="F155" s="3" t="n">
-        <v>272.17</v>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B156" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C156" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="D156" s="3" t="n">
-        <v>4.26</v>
-      </c>
-      <c r="E156" s="3" t="n">
-        <v>33.37</v>
-      </c>
-      <c r="F156" s="3" t="n">
-        <v>383.03</v>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B157" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C157" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="D157" s="3" t="n">
-        <v>4.37</v>
-      </c>
-      <c r="E157" s="3" t="n">
-        <v>35.15</v>
-      </c>
-      <c r="F157" s="3" t="n">
-        <v>414.86</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B158" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C158" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="D158" s="3" t="n">
-        <v>4.44</v>
-      </c>
-      <c r="E158" s="3" t="n">
-        <v>36.32</v>
-      </c>
-      <c r="F158" s="3" t="n">
-        <v>436.3</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B159" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C159" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="D159" s="3" t="n">
-        <v>5.02</v>
-      </c>
-      <c r="E159" s="3" t="n">
-        <v>47.01</v>
-      </c>
-      <c r="F159" s="3" t="n">
-        <v>647.57</v>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B160" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C160" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="D160" s="3" t="n">
-        <v>5.32</v>
-      </c>
-      <c r="E160" s="3" t="n">
-        <v>53.03</v>
-      </c>
-      <c r="F160" s="3" t="n">
-        <v>778.38</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B161" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C161" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="D161" s="3" t="n">
-        <v>5.45</v>
-      </c>
-      <c r="E161" s="3" t="n">
-        <v>55.66</v>
-      </c>
-      <c r="F161" s="3" t="n">
-        <v>838.22</v>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B162" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C162" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="D162" s="3" t="n">
-        <v>7.75</v>
-      </c>
-      <c r="E162" s="3" t="n">
-        <v>114.7</v>
-      </c>
-      <c r="F162" s="3" t="n">
-        <v>2518.35</v>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B163" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="C163" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="D163" s="3" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="E163" s="3" t="n">
-        <v>256.91</v>
-      </c>
-      <c r="F163" s="3" t="n">
-        <v>8540.54</v>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B164" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C164" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="D164" s="3" t="n">
-        <v>1.39</v>
-      </c>
-      <c r="E164" s="3" t="n">
-        <v>2.74</v>
-      </c>
-      <c r="F164" s="3" t="n">
-        <v>7.26</v>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B165" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C165" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="D165" s="3" t="n">
-        <v>1.41</v>
-      </c>
-      <c r="E165" s="3" t="n">
-        <v>2.84</v>
-      </c>
-      <c r="F165" s="3" t="n">
-        <v>7.73</v>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B166" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C166" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="D166" s="3" t="n">
-        <v>1.41</v>
-      </c>
-      <c r="E166" s="3" t="n">
-        <v>2.87</v>
-      </c>
-      <c r="F166" s="3" t="n">
-        <v>7.85</v>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B167" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C167" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="D167" s="3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="E167" s="3" t="n">
-        <v>3.33</v>
-      </c>
-      <c r="F167" s="3" t="n">
-        <v>10.09</v>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B168" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C168" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="D168" s="3" t="n">
-        <v>1.58</v>
-      </c>
-      <c r="E168" s="3" t="n">
-        <v>3.77</v>
-      </c>
-      <c r="F168" s="3" t="n">
-        <v>12.36</v>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B169" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C169" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="D169" s="3" t="n">
-        <v>1.62</v>
-      </c>
-      <c r="E169" s="3" t="n">
-        <v>3.98</v>
-      </c>
-      <c r="F169" s="3" t="n">
-        <v>13.5</v>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B170" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C170" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="D170" s="3" t="n">
-        <v>1.81</v>
-      </c>
-      <c r="E170" s="3" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="F170" s="3" t="n">
-        <v>20.89</v>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B171" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C171" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="D171" s="3" t="n">
-        <v>1.99</v>
-      </c>
-      <c r="E171" s="3" t="n">
-        <v>6.43</v>
-      </c>
-      <c r="F171" s="3" t="n">
-        <v>29.37</v>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B172" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C172" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="D172" s="3" t="n">
-        <v>2.41</v>
-      </c>
-      <c r="E172" s="3" t="n">
-        <v>9.87</v>
-      </c>
-      <c r="F172" s="3" t="n">
-        <v>57.89</v>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B173" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C173" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="D173" s="3" t="n">
-        <v>2.61</v>
-      </c>
-      <c r="E173" s="3" t="n">
-        <v>11.71</v>
-      </c>
-      <c r="F173" s="3" t="n">
-        <v>75.7</v>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B174" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C174" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="D174" s="3" t="n">
-        <v>2.65</v>
-      </c>
-      <c r="E174" s="3" t="n">
-        <v>12.11</v>
-      </c>
-      <c r="F174" s="3" t="n">
-        <v>79.83</v>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B175" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C175" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="D175" s="3" t="n">
-        <v>3.39</v>
-      </c>
-      <c r="E175" s="3" t="n">
-        <v>20.65</v>
-      </c>
-      <c r="F175" s="3" t="n">
-        <v>182.88</v>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B176" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C176" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="D176" s="3" t="n">
-        <v>3.58</v>
-      </c>
-      <c r="E176" s="3" t="n">
-        <v>23.18</v>
-      </c>
-      <c r="F176" s="3" t="n">
-        <v>218.69</v>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B177" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C177" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="D177" s="3" t="n">
-        <v>3.69</v>
-      </c>
-      <c r="E177" s="3" t="n">
-        <v>24.59</v>
-      </c>
-      <c r="F177" s="3" t="n">
-        <v>239.59</v>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B178" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C178" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="D178" s="3" t="n">
-        <v>4.13</v>
-      </c>
-      <c r="E178" s="3" t="n">
-        <v>31.3</v>
-      </c>
-      <c r="F178" s="3" t="n">
-        <v>347.18</v>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B179" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C179" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="D179" s="3" t="n">
-        <v>4.59</v>
-      </c>
-      <c r="E179" s="3" t="n">
-        <v>39.03</v>
-      </c>
-      <c r="F179" s="3" t="n">
-        <v>487.17</v>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B180" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C180" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="D180" s="3" t="n">
-        <v>4.63</v>
-      </c>
-      <c r="E180" s="3" t="n">
-        <v>39.6</v>
-      </c>
-      <c r="F180" s="3" t="n">
-        <v>498.05</v>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" s="1" t="n">
-        <v>46187</v>
-      </c>
-      <c r="B181" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="C181" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="D181" s="3" t="n">
-        <v>4.77</v>
-      </c>
-      <c r="E181" s="3" t="n">
-        <v>42.14</v>
-      </c>
-      <c r="F181" s="3" t="n">
-        <v>547.82</v>
+        <v>1242</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-06-19 13:33:11
</commit_message>
<xml_diff>
--- a/files/AFL_goalscorers.xlsx
+++ b/files/AFL_goalscorers.xlsx
@@ -2306,7 +2306,7 @@
         <v>1.84</v>
       </c>
       <c r="F74" s="3" t="n">
-        <v>3.63</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="75">
@@ -2326,7 +2326,7 @@
         <v>2.15</v>
       </c>
       <c r="F75" s="3" t="n">
-        <v>4.78</v>
+        <v>4.79</v>
       </c>
     </row>
     <row r="76">
@@ -2346,7 +2346,7 @@
         <v>2.17</v>
       </c>
       <c r="F76" s="3" t="n">
-        <v>4.85</v>
+        <v>4.86</v>
       </c>
     </row>
     <row r="77">
@@ -2366,7 +2366,7 @@
         <v>2.56</v>
       </c>
       <c r="F77" s="3" t="n">
-        <v>6.47</v>
+        <v>6.49</v>
       </c>
     </row>
     <row r="78">
@@ -2383,10 +2383,10 @@
         <v>1.49</v>
       </c>
       <c r="E78" s="3" t="n">
-        <v>3.25</v>
+        <v>3.26</v>
       </c>
       <c r="F78" s="3" t="n">
-        <v>9.7</v>
+        <v>9.72</v>
       </c>
     </row>
     <row r="79">
@@ -2403,10 +2403,10 @@
         <v>1.59</v>
       </c>
       <c r="E79" s="3" t="n">
-        <v>3.81</v>
+        <v>3.82</v>
       </c>
       <c r="F79" s="3" t="n">
-        <v>12.6</v>
+        <v>12.63</v>
       </c>
     </row>
     <row r="80">
@@ -2423,10 +2423,10 @@
         <v>1.79</v>
       </c>
       <c r="E80" s="3" t="n">
-        <v>5.08</v>
+        <v>5.09</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>20.13</v>
+        <v>20.17</v>
       </c>
     </row>
     <row r="81">
@@ -2443,10 +2443,10 @@
         <v>1.8</v>
       </c>
       <c r="E81" s="3" t="n">
-        <v>5.11</v>
+        <v>5.12</v>
       </c>
       <c r="F81" s="3" t="n">
-        <v>20.33</v>
+        <v>20.37</v>
       </c>
     </row>
     <row r="82">
@@ -2463,10 +2463,10 @@
         <v>1.95</v>
       </c>
       <c r="E82" s="3" t="n">
-        <v>6.18</v>
+        <v>6.19</v>
       </c>
       <c r="F82" s="3" t="n">
-        <v>27.54</v>
+        <v>27.61</v>
       </c>
     </row>
     <row r="83">
@@ -2483,10 +2483,10 @@
         <v>1.96</v>
       </c>
       <c r="E83" s="3" t="n">
-        <v>6.23</v>
+        <v>6.24</v>
       </c>
       <c r="F83" s="3" t="n">
-        <v>27.93</v>
+        <v>28</v>
       </c>
     </row>
     <row r="84">
@@ -2503,10 +2503,10 @@
         <v>2.55</v>
       </c>
       <c r="E84" s="3" t="n">
-        <v>11.16</v>
+        <v>11.18</v>
       </c>
       <c r="F84" s="3" t="n">
-        <v>70.26</v>
+        <v>70.44</v>
       </c>
     </row>
     <row r="85">
@@ -2523,10 +2523,10 @@
         <v>2.73</v>
       </c>
       <c r="E85" s="3" t="n">
-        <v>12.98</v>
+        <v>13</v>
       </c>
       <c r="F85" s="3" t="n">
-        <v>88.92</v>
+        <v>89.15</v>
       </c>
     </row>
     <row r="86">
@@ -2543,10 +2543,10 @@
         <v>2.92</v>
       </c>
       <c r="E86" s="3" t="n">
-        <v>14.95</v>
+        <v>14.98</v>
       </c>
       <c r="F86" s="3" t="n">
-        <v>110.92</v>
+        <v>111.22</v>
       </c>
     </row>
     <row r="87">
@@ -2560,13 +2560,13 @@
         <v>96</v>
       </c>
       <c r="D87" s="3" t="n">
-        <v>3.1</v>
+        <v>3.11</v>
       </c>
       <c r="E87" s="3" t="n">
-        <v>17.07</v>
+        <v>17.1</v>
       </c>
       <c r="F87" s="3" t="n">
-        <v>136.19</v>
+        <v>136.55</v>
       </c>
     </row>
     <row r="88">
@@ -2583,10 +2583,10 @@
         <v>3.76</v>
       </c>
       <c r="E88" s="3" t="n">
-        <v>25.63</v>
+        <v>25.68</v>
       </c>
       <c r="F88" s="3" t="n">
-        <v>255.36</v>
+        <v>256.06</v>
       </c>
     </row>
     <row r="89">
@@ -2600,13 +2600,13 @@
         <v>98</v>
       </c>
       <c r="D89" s="3" t="n">
-        <v>7.03</v>
+        <v>7.04</v>
       </c>
       <c r="E89" s="3" t="n">
-        <v>94.15</v>
+        <v>94.33</v>
       </c>
       <c r="F89" s="3" t="n">
-        <v>1866.18</v>
+        <v>1871.52</v>
       </c>
     </row>
     <row r="90">
@@ -2623,10 +2623,10 @@
         <v>8.47</v>
       </c>
       <c r="E90" s="3" t="n">
-        <v>137.6</v>
+        <v>137.86</v>
       </c>
       <c r="F90" s="3" t="n">
-        <v>3319.31</v>
+        <v>3328.86</v>
       </c>
     </row>
     <row r="91">
@@ -2643,10 +2643,10 @@
         <v>8.96</v>
       </c>
       <c r="E91" s="3" t="n">
-        <v>154.35</v>
+        <v>154.64</v>
       </c>
       <c r="F91" s="3" t="n">
-        <v>3950.34</v>
+        <v>3961.73</v>
       </c>
     </row>
     <row r="92">
@@ -3383,10 +3383,10 @@
         <v>1.37</v>
       </c>
       <c r="E128" s="3" t="n">
-        <v>2.67</v>
+        <v>2.68</v>
       </c>
       <c r="F128" s="3" t="n">
-        <v>6.96</v>
+        <v>6.98</v>
       </c>
     </row>
     <row r="129">
@@ -3403,10 +3403,10 @@
         <v>1.39</v>
       </c>
       <c r="E129" s="3" t="n">
-        <v>2.74</v>
+        <v>2.75</v>
       </c>
       <c r="F129" s="3" t="n">
-        <v>7.27</v>
+        <v>7.29</v>
       </c>
     </row>
     <row r="130">
@@ -3426,7 +3426,7 @@
         <v>3.06</v>
       </c>
       <c r="F130" s="3" t="n">
-        <v>8.74</v>
+        <v>8.77</v>
       </c>
     </row>
     <row r="131">
@@ -3443,10 +3443,10 @@
         <v>1.5</v>
       </c>
       <c r="E131" s="3" t="n">
-        <v>3.32</v>
+        <v>3.33</v>
       </c>
       <c r="F131" s="3" t="n">
-        <v>10.05</v>
+        <v>10.09</v>
       </c>
     </row>
     <row r="132">
@@ -3466,7 +3466,7 @@
         <v>4.26</v>
       </c>
       <c r="F132" s="3" t="n">
-        <v>15.09</v>
+        <v>15.14</v>
       </c>
     </row>
     <row r="133">
@@ -3483,10 +3483,10 @@
         <v>1.73</v>
       </c>
       <c r="E133" s="3" t="n">
-        <v>4.69</v>
+        <v>4.7</v>
       </c>
       <c r="F133" s="3" t="n">
-        <v>17.67</v>
+        <v>17.73</v>
       </c>
     </row>
     <row r="134">
@@ -3503,10 +3503,10 @@
         <v>1.81</v>
       </c>
       <c r="E134" s="3" t="n">
-        <v>5.2</v>
+        <v>5.21</v>
       </c>
       <c r="F134" s="3" t="n">
-        <v>20.86</v>
+        <v>20.94</v>
       </c>
     </row>
     <row r="135">
@@ -3523,10 +3523,10 @@
         <v>1.83</v>
       </c>
       <c r="E135" s="3" t="n">
-        <v>5.3</v>
+        <v>5.31</v>
       </c>
       <c r="F135" s="3" t="n">
-        <v>21.52</v>
+        <v>21.6</v>
       </c>
     </row>
     <row r="136">
@@ -3543,10 +3543,10 @@
         <v>2.06</v>
       </c>
       <c r="E136" s="3" t="n">
-        <v>6.93</v>
+        <v>6.95</v>
       </c>
       <c r="F136" s="3" t="n">
-        <v>33.1</v>
+        <v>33.22</v>
       </c>
     </row>
     <row r="137">
@@ -3560,13 +3560,13 @@
         <v>149</v>
       </c>
       <c r="D137" s="3" t="n">
-        <v>2.07</v>
+        <v>2.08</v>
       </c>
       <c r="E137" s="3" t="n">
-        <v>7.08</v>
+        <v>7.1</v>
       </c>
       <c r="F137" s="3" t="n">
-        <v>34.24</v>
+        <v>34.37</v>
       </c>
     </row>
     <row r="138">
@@ -3580,13 +3580,13 @@
         <v>150</v>
       </c>
       <c r="D138" s="3" t="n">
-        <v>2.68</v>
+        <v>2.69</v>
       </c>
       <c r="E138" s="3" t="n">
-        <v>12.49</v>
+        <v>12.52</v>
       </c>
       <c r="F138" s="3" t="n">
-        <v>83.79</v>
+        <v>84.12</v>
       </c>
     </row>
     <row r="139">
@@ -3603,10 +3603,10 @@
         <v>3.13</v>
       </c>
       <c r="E139" s="3" t="n">
-        <v>17.37</v>
+        <v>17.41</v>
       </c>
       <c r="F139" s="3" t="n">
-        <v>139.92</v>
+        <v>140.49</v>
       </c>
     </row>
     <row r="140">
@@ -3620,13 +3620,13 @@
         <v>152</v>
       </c>
       <c r="D140" s="3" t="n">
-        <v>3.28</v>
+        <v>3.29</v>
       </c>
       <c r="E140" s="3" t="n">
-        <v>19.22</v>
+        <v>19.27</v>
       </c>
       <c r="F140" s="3" t="n">
-        <v>163.77</v>
+        <v>164.44</v>
       </c>
     </row>
     <row r="141">
@@ -3643,10 +3643,10 @@
         <v>4.07</v>
       </c>
       <c r="E141" s="3" t="n">
-        <v>30.25</v>
+        <v>30.33</v>
       </c>
       <c r="F141" s="3" t="n">
-        <v>329.47</v>
+        <v>330.84</v>
       </c>
     </row>
     <row r="142">
@@ -3660,13 +3660,13 @@
         <v>154</v>
       </c>
       <c r="D142" s="3" t="n">
-        <v>4.14</v>
+        <v>4.15</v>
       </c>
       <c r="E142" s="3" t="n">
-        <v>31.46</v>
+        <v>31.54</v>
       </c>
       <c r="F142" s="3" t="n">
-        <v>349.91</v>
+        <v>351.37</v>
       </c>
     </row>
     <row r="143">
@@ -3683,10 +3683,10 @@
         <v>4.2</v>
       </c>
       <c r="E143" s="3" t="n">
-        <v>32.32</v>
+        <v>32.4</v>
       </c>
       <c r="F143" s="3" t="n">
-        <v>364.71</v>
+        <v>366.23</v>
       </c>
     </row>
     <row r="144">
@@ -3700,13 +3700,13 @@
         <v>156</v>
       </c>
       <c r="D144" s="3" t="n">
-        <v>4.55</v>
+        <v>4.56</v>
       </c>
       <c r="E144" s="3" t="n">
-        <v>38.29</v>
+        <v>38.4</v>
       </c>
       <c r="F144" s="3" t="n">
-        <v>473.14</v>
+        <v>475.12</v>
       </c>
     </row>
     <row r="145">
@@ -3723,10 +3723,10 @@
         <v>6.18</v>
       </c>
       <c r="E145" s="3" t="n">
-        <v>72.04</v>
+        <v>72.24</v>
       </c>
       <c r="F145" s="3" t="n">
-        <v>1242</v>
+        <v>1247.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-08-11 21:07:55
</commit_message>
<xml_diff>
--- a/files/AFL_goalscorers.xlsx
+++ b/files/AFL_goalscorers.xlsx
@@ -2302,7 +2302,7 @@
         <v>2.65</v>
       </c>
       <c r="G38" t="n">
-        <v>6.87</v>
+        <v>6.85</v>
       </c>
     </row>
     <row r="39">
@@ -2319,13 +2319,13 @@
         <v>49</v>
       </c>
       <c r="E39" t="n">
-        <v>1.53</v>
+        <v>1.52</v>
       </c>
       <c r="F39" t="n">
-        <v>3.47</v>
+        <v>3.46</v>
       </c>
       <c r="G39" t="n">
-        <v>10.78</v>
+        <v>10.75</v>
       </c>
     </row>
     <row r="40">
@@ -2345,10 +2345,10 @@
         <v>1.76</v>
       </c>
       <c r="F40" t="n">
-        <v>4.89</v>
+        <v>4.88</v>
       </c>
       <c r="G40" t="n">
-        <v>18.89</v>
+        <v>18.83</v>
       </c>
     </row>
     <row r="41">
@@ -2368,10 +2368,10 @@
         <v>1.85</v>
       </c>
       <c r="F41" t="n">
-        <v>5.46</v>
+        <v>5.45</v>
       </c>
       <c r="G41" t="n">
-        <v>22.59</v>
+        <v>22.53</v>
       </c>
     </row>
     <row r="42">
@@ -2391,10 +2391,10 @@
         <v>1.96</v>
       </c>
       <c r="F42" t="n">
-        <v>6.24</v>
+        <v>6.23</v>
       </c>
       <c r="G42" t="n">
-        <v>28.01</v>
+        <v>27.92</v>
       </c>
     </row>
     <row r="43">
@@ -2414,10 +2414,10 @@
         <v>2.05</v>
       </c>
       <c r="F43" t="n">
-        <v>6.91</v>
+        <v>6.9</v>
       </c>
       <c r="G43" t="n">
-        <v>32.95</v>
+        <v>32.85</v>
       </c>
     </row>
     <row r="44">
@@ -2437,10 +2437,10 @@
         <v>2.08</v>
       </c>
       <c r="F44" t="n">
-        <v>7.14</v>
+        <v>7.13</v>
       </c>
       <c r="G44" t="n">
-        <v>34.72</v>
+        <v>34.61</v>
       </c>
     </row>
     <row r="45">
@@ -2460,10 +2460,10 @@
         <v>2.09</v>
       </c>
       <c r="F45" t="n">
-        <v>7.18</v>
+        <v>7.17</v>
       </c>
       <c r="G45" t="n">
-        <v>35.05</v>
+        <v>34.94</v>
       </c>
     </row>
     <row r="46">
@@ -2483,10 +2483,10 @@
         <v>2.35</v>
       </c>
       <c r="F46" t="n">
-        <v>9.31</v>
+        <v>9.3</v>
       </c>
       <c r="G46" t="n">
-        <v>52.87</v>
+        <v>52.7</v>
       </c>
     </row>
     <row r="47">
@@ -2506,10 +2506,10 @@
         <v>3.14</v>
       </c>
       <c r="F47" t="n">
-        <v>17.48</v>
+        <v>17.44</v>
       </c>
       <c r="G47" t="n">
-        <v>141.29</v>
+        <v>140.82</v>
       </c>
     </row>
     <row r="48">
@@ -2526,13 +2526,13 @@
         <v>58</v>
       </c>
       <c r="E48" t="n">
-        <v>3.21</v>
+        <v>3.2</v>
       </c>
       <c r="F48" t="n">
-        <v>18.3</v>
+        <v>18.26</v>
       </c>
       <c r="G48" t="n">
-        <v>151.74</v>
+        <v>151.23</v>
       </c>
     </row>
     <row r="49">
@@ -2549,13 +2549,13 @@
         <v>59</v>
       </c>
       <c r="E49" t="n">
-        <v>4.4</v>
+        <v>4.39</v>
       </c>
       <c r="F49" t="n">
-        <v>35.6</v>
+        <v>35.52</v>
       </c>
       <c r="G49" t="n">
-        <v>423</v>
+        <v>421.55</v>
       </c>
     </row>
     <row r="50">
@@ -2575,10 +2575,10 @@
         <v>4.64</v>
       </c>
       <c r="F50" t="n">
-        <v>39.93</v>
+        <v>39.84</v>
       </c>
       <c r="G50" t="n">
-        <v>504.43</v>
+        <v>502.69</v>
       </c>
     </row>
     <row r="51">
@@ -2595,13 +2595,13 @@
         <v>61</v>
       </c>
       <c r="E51" t="n">
-        <v>6.88</v>
+        <v>6.87</v>
       </c>
       <c r="F51" t="n">
-        <v>90.01</v>
+        <v>89.8</v>
       </c>
       <c r="G51" t="n">
-        <v>1742.86</v>
+        <v>1736.73</v>
       </c>
     </row>
     <row r="52">
@@ -2618,13 +2618,13 @@
         <v>62</v>
       </c>
       <c r="E52" t="n">
-        <v>7.16</v>
+        <v>7.15</v>
       </c>
       <c r="F52" t="n">
-        <v>97.59</v>
+        <v>97.36</v>
       </c>
       <c r="G52" t="n">
-        <v>1970.51</v>
+        <v>1963.57</v>
       </c>
     </row>
     <row r="53">
@@ -2641,13 +2641,13 @@
         <v>63</v>
       </c>
       <c r="E53" t="n">
-        <v>7.19</v>
+        <v>7.18</v>
       </c>
       <c r="F53" t="n">
-        <v>98.44</v>
+        <v>98.21</v>
       </c>
       <c r="G53" t="n">
-        <v>1996.7</v>
+        <v>1989.67</v>
       </c>
     </row>
     <row r="54">
@@ -2664,13 +2664,13 @@
         <v>64</v>
       </c>
       <c r="E54" t="n">
-        <v>10.54</v>
+        <v>10.53</v>
       </c>
       <c r="F54" t="n">
-        <v>214.96</v>
+        <v>214.45</v>
       </c>
       <c r="G54" t="n">
-        <v>6522.35</v>
+        <v>6499.08</v>
       </c>
     </row>
     <row r="55">
@@ -2687,13 +2687,13 @@
         <v>65</v>
       </c>
       <c r="E55" t="n">
-        <v>11.86</v>
+        <v>11.85</v>
       </c>
       <c r="F55" t="n">
-        <v>273.47</v>
+        <v>272.83</v>
       </c>
       <c r="G55" t="n">
-        <v>9386.38</v>
+        <v>9352.78</v>
       </c>
     </row>
     <row r="56">
@@ -2785,7 +2785,7 @@
         <v>2.81</v>
       </c>
       <c r="G59" t="n">
-        <v>7.6</v>
+        <v>7.59</v>
       </c>
     </row>
     <row r="60">
@@ -2808,7 +2808,7 @@
         <v>3.15</v>
       </c>
       <c r="G60" t="n">
-        <v>9.21</v>
+        <v>9.2</v>
       </c>
     </row>
     <row r="61">
@@ -2831,7 +2831,7 @@
         <v>3.36</v>
       </c>
       <c r="G61" t="n">
-        <v>10.24</v>
+        <v>10.22</v>
       </c>
     </row>
     <row r="62">
@@ -2854,7 +2854,7 @@
         <v>3.37</v>
       </c>
       <c r="G62" t="n">
-        <v>10.28</v>
+        <v>10.27</v>
       </c>
     </row>
     <row r="63">
@@ -2877,7 +2877,7 @@
         <v>4.04</v>
       </c>
       <c r="G63" t="n">
-        <v>13.87</v>
+        <v>13.85</v>
       </c>
     </row>
     <row r="64">
@@ -2900,7 +2900,7 @@
         <v>5.03</v>
       </c>
       <c r="G64" t="n">
-        <v>19.82</v>
+        <v>19.79</v>
       </c>
     </row>
     <row r="65">
@@ -2923,7 +2923,7 @@
         <v>5.19</v>
       </c>
       <c r="G65" t="n">
-        <v>20.84</v>
+        <v>20.81</v>
       </c>
     </row>
     <row r="66">
@@ -2943,10 +2943,10 @@
         <v>1.91</v>
       </c>
       <c r="F66" t="n">
-        <v>5.9</v>
+        <v>5.89</v>
       </c>
       <c r="G66" t="n">
-        <v>25.58</v>
+        <v>25.55</v>
       </c>
     </row>
     <row r="67">
@@ -2966,10 +2966,10 @@
         <v>2.05</v>
       </c>
       <c r="F67" t="n">
-        <v>6.93</v>
+        <v>6.92</v>
       </c>
       <c r="G67" t="n">
-        <v>33.08</v>
+        <v>33.03</v>
       </c>
     </row>
     <row r="68">
@@ -2989,10 +2989,10 @@
         <v>2.87</v>
       </c>
       <c r="F68" t="n">
-        <v>14.42</v>
+        <v>14.4</v>
       </c>
       <c r="G68" t="n">
-        <v>104.78</v>
+        <v>104.62</v>
       </c>
     </row>
     <row r="69">
@@ -3012,10 +3012,10 @@
         <v>3.11</v>
       </c>
       <c r="F69" t="n">
-        <v>17.17</v>
+        <v>17.16</v>
       </c>
       <c r="G69" t="n">
-        <v>137.5</v>
+        <v>137.28</v>
       </c>
     </row>
     <row r="70">
@@ -3032,13 +3032,13 @@
         <v>81</v>
       </c>
       <c r="E70" t="n">
-        <v>3.2</v>
+        <v>3.19</v>
       </c>
       <c r="F70" t="n">
-        <v>18.17</v>
+        <v>18.15</v>
       </c>
       <c r="G70" t="n">
-        <v>150.11</v>
+        <v>149.87</v>
       </c>
     </row>
     <row r="71">
@@ -3058,10 +3058,10 @@
         <v>4.27</v>
       </c>
       <c r="F71" t="n">
-        <v>33.55</v>
+        <v>33.51</v>
       </c>
       <c r="G71" t="n">
-        <v>386.23</v>
+        <v>385.61</v>
       </c>
     </row>
     <row r="72">
@@ -3081,10 +3081,10 @@
         <v>4.79</v>
       </c>
       <c r="F72" t="n">
-        <v>42.61</v>
+        <v>42.57</v>
       </c>
       <c r="G72" t="n">
-        <v>557.3</v>
+        <v>556.39</v>
       </c>
     </row>
     <row r="73">
@@ -3104,10 +3104,10 @@
         <v>7.53</v>
       </c>
       <c r="F73" t="n">
-        <v>108.36</v>
+        <v>108.24</v>
       </c>
       <c r="G73" t="n">
-        <v>2310.21</v>
+        <v>2306.35</v>
       </c>
     </row>
     <row r="74">
@@ -3452,7 +3452,7 @@
         <v>31.12</v>
       </c>
       <c r="G88" t="n">
-        <v>344.24</v>
+        <v>344.25</v>
       </c>
     </row>
     <row r="89">
@@ -3475,7 +3475,7 @@
         <v>51.84</v>
       </c>
       <c r="G89" t="n">
-        <v>751.87</v>
+        <v>751.89</v>
       </c>
     </row>
     <row r="90">
@@ -3498,7 +3498,7 @@
         <v>111.17</v>
       </c>
       <c r="G90" t="n">
-        <v>2401.72</v>
+        <v>2401.76</v>
       </c>
     </row>
     <row r="91">
@@ -3518,10 +3518,10 @@
         <v>10.08</v>
       </c>
       <c r="F91" t="n">
-        <v>196.43</v>
+        <v>196.44</v>
       </c>
       <c r="G91" t="n">
-        <v>5691.1</v>
+        <v>5691.2</v>
       </c>
     </row>
     <row r="92">
@@ -3751,7 +3751,7 @@
         <v>18.24</v>
       </c>
       <c r="G101" t="n">
-        <v>150.94</v>
+        <v>150.93</v>
       </c>
     </row>
     <row r="102">
@@ -3797,7 +3797,7 @@
         <v>24.55</v>
       </c>
       <c r="G103" t="n">
-        <v>238.92</v>
+        <v>238.91</v>
       </c>
     </row>
     <row r="104">
@@ -3889,7 +3889,7 @@
         <v>70.5</v>
       </c>
       <c r="G107" t="n">
-        <v>1201.85</v>
+        <v>1201.83</v>
       </c>
     </row>
     <row r="108">
@@ -3912,7 +3912,7 @@
         <v>112.77</v>
       </c>
       <c r="G108" t="n">
-        <v>2454.44</v>
+        <v>2454.4</v>
       </c>
     </row>
     <row r="109">
@@ -3935,7 +3935,7 @@
         <v>230.64</v>
       </c>
       <c r="G109" t="n">
-        <v>7255.32</v>
+        <v>7255.21</v>
       </c>
     </row>
     <row r="110">
@@ -4142,7 +4142,7 @@
         <v>10.32</v>
       </c>
       <c r="G118" t="n">
-        <v>62.14</v>
+        <v>62.15</v>
       </c>
     </row>
     <row r="119">
@@ -4349,7 +4349,7 @@
         <v>200.8</v>
       </c>
       <c r="G127" t="n">
-        <v>5883.61</v>
+        <v>5883.63</v>
       </c>
     </row>
     <row r="128">
@@ -4510,7 +4510,7 @@
         <v>9.49</v>
       </c>
       <c r="G134" t="n">
-        <v>54.44</v>
+        <v>54.43</v>
       </c>
     </row>
     <row r="135">
@@ -4694,7 +4694,7 @@
         <v>42.58</v>
       </c>
       <c r="G142" t="n">
-        <v>556.55</v>
+        <v>556.54</v>
       </c>
     </row>
     <row r="143">
@@ -4717,7 +4717,7 @@
         <v>125.74</v>
       </c>
       <c r="G143" t="n">
-        <v>2895.34</v>
+        <v>2895.33</v>
       </c>
     </row>
     <row r="144">
@@ -4740,7 +4740,7 @@
         <v>291.12</v>
       </c>
       <c r="G144" t="n">
-        <v>10316.5</v>
+        <v>10316.44</v>
       </c>
     </row>
     <row r="145">
@@ -4760,10 +4760,10 @@
         <v>14.38</v>
       </c>
       <c r="F145" t="n">
-        <v>403.64</v>
+        <v>403.63</v>
       </c>
       <c r="G145" t="n">
-        <v>16897.2</v>
+        <v>16897.1</v>
       </c>
     </row>
     <row r="146">
@@ -4786,7 +4786,7 @@
         <v>2.28</v>
       </c>
       <c r="G146" t="n">
-        <v>5.32</v>
+        <v>5.31</v>
       </c>
     </row>
     <row r="147">
@@ -4809,7 +4809,7 @@
         <v>2.41</v>
       </c>
       <c r="G147" t="n">
-        <v>5.84</v>
+        <v>5.83</v>
       </c>
     </row>
     <row r="148">
@@ -4832,7 +4832,7 @@
         <v>3.23</v>
       </c>
       <c r="G148" t="n">
-        <v>9.59</v>
+        <v>9.57</v>
       </c>
     </row>
     <row r="149">
@@ -4852,10 +4852,10 @@
         <v>1.59</v>
       </c>
       <c r="F149" t="n">
-        <v>3.85</v>
+        <v>3.84</v>
       </c>
       <c r="G149" t="n">
-        <v>12.79</v>
+        <v>12.76</v>
       </c>
     </row>
     <row r="150">
@@ -4875,10 +4875,10 @@
         <v>1.74</v>
       </c>
       <c r="F150" t="n">
-        <v>4.76</v>
+        <v>4.75</v>
       </c>
       <c r="G150" t="n">
-        <v>18.11</v>
+        <v>18.07</v>
       </c>
     </row>
     <row r="151">
@@ -4898,10 +4898,10 @@
         <v>1.8</v>
       </c>
       <c r="F151" t="n">
-        <v>5.11</v>
+        <v>5.1</v>
       </c>
       <c r="G151" t="n">
-        <v>20.3</v>
+        <v>20.26</v>
       </c>
     </row>
     <row r="152">
@@ -4924,7 +4924,7 @@
         <v>5.4</v>
       </c>
       <c r="G152" t="n">
-        <v>22.23</v>
+        <v>22.18</v>
       </c>
     </row>
     <row r="153">
@@ -4944,10 +4944,10 @@
         <v>1.98</v>
       </c>
       <c r="F153" t="n">
-        <v>6.35</v>
+        <v>6.34</v>
       </c>
       <c r="G153" t="n">
-        <v>28.78</v>
+        <v>28.71</v>
       </c>
     </row>
     <row r="154">
@@ -4964,13 +4964,13 @@
         <v>173</v>
       </c>
       <c r="E154" t="n">
-        <v>1.99</v>
+        <v>1.98</v>
       </c>
       <c r="F154" t="n">
-        <v>6.41</v>
+        <v>6.4</v>
       </c>
       <c r="G154" t="n">
-        <v>29.25</v>
+        <v>29.18</v>
       </c>
     </row>
     <row r="155">
@@ -4990,10 +4990,10 @@
         <v>2.34</v>
       </c>
       <c r="F155" t="n">
-        <v>9.27</v>
+        <v>9.25</v>
       </c>
       <c r="G155" t="n">
-        <v>52.43</v>
+        <v>52.31</v>
       </c>
     </row>
     <row r="156">
@@ -5010,13 +5010,13 @@
         <v>175</v>
       </c>
       <c r="E156" t="n">
-        <v>3.24</v>
+        <v>3.23</v>
       </c>
       <c r="F156" t="n">
-        <v>18.65</v>
+        <v>18.62</v>
       </c>
       <c r="G156" t="n">
-        <v>156.23</v>
+        <v>155.85</v>
       </c>
     </row>
     <row r="157">
@@ -5033,13 +5033,13 @@
         <v>176</v>
       </c>
       <c r="E157" t="n">
-        <v>3.5</v>
+        <v>3.49</v>
       </c>
       <c r="F157" t="n">
-        <v>21.99</v>
+        <v>21.95</v>
       </c>
       <c r="G157" t="n">
-        <v>201.56</v>
+        <v>201.07</v>
       </c>
     </row>
     <row r="158">
@@ -5059,10 +5059,10 @@
         <v>3.71</v>
       </c>
       <c r="F158" t="n">
-        <v>24.96</v>
+        <v>24.92</v>
       </c>
       <c r="G158" t="n">
-        <v>245.13</v>
+        <v>244.52</v>
       </c>
     </row>
     <row r="159">
@@ -5082,10 +5082,10 @@
         <v>3.9</v>
       </c>
       <c r="F159" t="n">
-        <v>27.76</v>
+        <v>27.72</v>
       </c>
       <c r="G159" t="n">
-        <v>288.79</v>
+        <v>288.08</v>
       </c>
     </row>
     <row r="160">
@@ -5105,10 +5105,10 @@
         <v>4.05</v>
       </c>
       <c r="F160" t="n">
-        <v>30.03</v>
+        <v>29.98</v>
       </c>
       <c r="G160" t="n">
-        <v>325.76</v>
+        <v>324.95</v>
       </c>
     </row>
     <row r="161">
@@ -5125,13 +5125,13 @@
         <v>180</v>
       </c>
       <c r="E161" t="n">
-        <v>5.11</v>
+        <v>5.1</v>
       </c>
       <c r="F161" t="n">
-        <v>48.62</v>
+        <v>48.54</v>
       </c>
       <c r="G161" t="n">
-        <v>681.71</v>
+        <v>680</v>
       </c>
     </row>
     <row r="162">
@@ -5148,13 +5148,13 @@
         <v>181</v>
       </c>
       <c r="E162" t="n">
-        <v>7.19</v>
+        <v>7.18</v>
       </c>
       <c r="F162" t="n">
-        <v>98.41</v>
+        <v>98.25</v>
       </c>
       <c r="G162" t="n">
-        <v>1995.87</v>
+        <v>1990.75</v>
       </c>
     </row>
     <row r="163">
@@ -5171,13 +5171,13 @@
         <v>182</v>
       </c>
       <c r="E163" t="n">
-        <v>9.6</v>
+        <v>9.59</v>
       </c>
       <c r="F163" t="n">
-        <v>177.75</v>
+        <v>177.45</v>
       </c>
       <c r="G163" t="n">
-        <v>4892.23</v>
+        <v>4879.55</v>
       </c>
     </row>
     <row r="164">
@@ -5200,7 +5200,7 @@
         <v>1.52</v>
       </c>
       <c r="G164" t="n">
-        <v>2.55</v>
+        <v>2.54</v>
       </c>
     </row>
     <row r="165">
@@ -5223,7 +5223,7 @@
         <v>2.11</v>
       </c>
       <c r="G165" t="n">
-        <v>4.63</v>
+        <v>4.62</v>
       </c>
     </row>
     <row r="166">
@@ -5246,7 +5246,7 @@
         <v>2.65</v>
       </c>
       <c r="G166" t="n">
-        <v>6.87</v>
+        <v>6.86</v>
       </c>
     </row>
     <row r="167">
@@ -5269,7 +5269,7 @@
         <v>3.08</v>
       </c>
       <c r="G167" t="n">
-        <v>8.86</v>
+        <v>8.84</v>
       </c>
     </row>
     <row r="168">
@@ -5286,13 +5286,13 @@
         <v>188</v>
       </c>
       <c r="E168" t="n">
-        <v>1.67</v>
+        <v>1.66</v>
       </c>
       <c r="F168" t="n">
-        <v>4.28</v>
+        <v>4.27</v>
       </c>
       <c r="G168" t="n">
-        <v>15.21</v>
+        <v>15.18</v>
       </c>
     </row>
     <row r="169">
@@ -5312,10 +5312,10 @@
         <v>1.73</v>
       </c>
       <c r="F169" t="n">
-        <v>4.67</v>
+        <v>4.66</v>
       </c>
       <c r="G169" t="n">
-        <v>17.55</v>
+        <v>17.52</v>
       </c>
     </row>
     <row r="170">
@@ -5335,10 +5335,10 @@
         <v>1.86</v>
       </c>
       <c r="F170" t="n">
-        <v>5.54</v>
+        <v>5.53</v>
       </c>
       <c r="G170" t="n">
-        <v>23.11</v>
+        <v>23.07</v>
       </c>
     </row>
     <row r="171">
@@ -5355,13 +5355,13 @@
         <v>191</v>
       </c>
       <c r="E171" t="n">
-        <v>2.02</v>
+        <v>2.01</v>
       </c>
       <c r="F171" t="n">
-        <v>6.63</v>
+        <v>6.62</v>
       </c>
       <c r="G171" t="n">
-        <v>30.87</v>
+        <v>30.81</v>
       </c>
     </row>
     <row r="172">
@@ -5378,13 +5378,13 @@
         <v>192</v>
       </c>
       <c r="E172" t="n">
-        <v>2.95</v>
+        <v>2.94</v>
       </c>
       <c r="F172" t="n">
-        <v>15.26</v>
+        <v>15.24</v>
       </c>
       <c r="G172" t="n">
-        <v>114.47</v>
+        <v>114.22</v>
       </c>
     </row>
     <row r="173">
@@ -5404,10 +5404,10 @@
         <v>3.77</v>
       </c>
       <c r="F173" t="n">
-        <v>25.83</v>
+        <v>25.79</v>
       </c>
       <c r="G173" t="n">
-        <v>258.37</v>
+        <v>257.78</v>
       </c>
     </row>
     <row r="174">
@@ -5427,10 +5427,10 @@
         <v>3.84</v>
       </c>
       <c r="F174" t="n">
-        <v>26.78</v>
+        <v>26.74</v>
       </c>
       <c r="G174" t="n">
-        <v>273.14</v>
+        <v>272.52</v>
       </c>
     </row>
     <row r="175">
@@ -5450,10 +5450,10 @@
         <v>4.1</v>
       </c>
       <c r="F175" t="n">
-        <v>30.78</v>
+        <v>30.73</v>
       </c>
       <c r="G175" t="n">
-        <v>338.38</v>
+        <v>337.61</v>
       </c>
     </row>
     <row r="176">
@@ -5473,10 +5473,10 @@
         <v>4.34</v>
       </c>
       <c r="F176" t="n">
-        <v>34.65</v>
+        <v>34.6</v>
       </c>
       <c r="G176" t="n">
-        <v>405.89</v>
+        <v>404.95</v>
       </c>
     </row>
     <row r="177">
@@ -5493,13 +5493,13 @@
         <v>197</v>
       </c>
       <c r="E177" t="n">
-        <v>4.46</v>
+        <v>4.45</v>
       </c>
       <c r="F177" t="n">
-        <v>36.61</v>
+        <v>36.55</v>
       </c>
       <c r="G177" t="n">
-        <v>441.61</v>
+        <v>440.59</v>
       </c>
     </row>
     <row r="178">
@@ -5519,10 +5519,10 @@
         <v>4.46</v>
       </c>
       <c r="F178" t="n">
-        <v>36.77</v>
+        <v>36.71</v>
       </c>
       <c r="G178" t="n">
-        <v>444.55</v>
+        <v>443.52</v>
       </c>
     </row>
     <row r="179">
@@ -5542,10 +5542,10 @@
         <v>4.93</v>
       </c>
       <c r="F179" t="n">
-        <v>45.19</v>
+        <v>45.13</v>
       </c>
       <c r="G179" t="n">
-        <v>609.73</v>
+        <v>608.31</v>
       </c>
     </row>
     <row r="180">
@@ -5565,10 +5565,10 @@
         <v>5.38</v>
       </c>
       <c r="F180" t="n">
-        <v>54.2</v>
+        <v>54.12</v>
       </c>
       <c r="G180" t="n">
-        <v>804.91</v>
+        <v>803.02</v>
       </c>
     </row>
     <row r="181">
@@ -5585,13 +5585,13 @@
         <v>201</v>
       </c>
       <c r="E181" t="n">
-        <v>6.36</v>
+        <v>6.35</v>
       </c>
       <c r="F181" t="n">
-        <v>76.45</v>
+        <v>76.34</v>
       </c>
       <c r="G181" t="n">
-        <v>1359.62</v>
+        <v>1356.41</v>
       </c>
     </row>
     <row r="182">
@@ -5729,7 +5729,7 @@
         <v>2.82</v>
       </c>
       <c r="G187" t="n">
-        <v>7.65</v>
+        <v>7.64</v>
       </c>
     </row>
     <row r="188">
@@ -5775,7 +5775,7 @@
         <v>3.76</v>
       </c>
       <c r="G189" t="n">
-        <v>12.33</v>
+        <v>12.32</v>
       </c>
     </row>
     <row r="190">
@@ -5798,7 +5798,7 @@
         <v>4.73</v>
       </c>
       <c r="G190" t="n">
-        <v>17.91</v>
+        <v>17.9</v>
       </c>
     </row>
     <row r="191">
@@ -5818,10 +5818,10 @@
         <v>2.69</v>
       </c>
       <c r="F191" t="n">
-        <v>12.52</v>
+        <v>12.51</v>
       </c>
       <c r="G191" t="n">
-        <v>84.05</v>
+        <v>84.01</v>
       </c>
     </row>
     <row r="192">
@@ -5844,7 +5844,7 @@
         <v>18.08</v>
       </c>
       <c r="G192" t="n">
-        <v>148.98</v>
+        <v>148.91</v>
       </c>
     </row>
     <row r="193">
@@ -5867,7 +5867,7 @@
         <v>18.47</v>
       </c>
       <c r="G193" t="n">
-        <v>153.95</v>
+        <v>153.88</v>
       </c>
     </row>
     <row r="194">
@@ -5887,10 +5887,10 @@
         <v>4.07</v>
       </c>
       <c r="F194" t="n">
-        <v>30.36</v>
+        <v>30.35</v>
       </c>
       <c r="G194" t="n">
-        <v>331.34</v>
+        <v>331.19</v>
       </c>
     </row>
     <row r="195">
@@ -5910,10 +5910,10 @@
         <v>4.4</v>
       </c>
       <c r="F195" t="n">
-        <v>35.64</v>
+        <v>35.63</v>
       </c>
       <c r="G195" t="n">
-        <v>423.8</v>
+        <v>423.6</v>
       </c>
     </row>
     <row r="196">
@@ -5933,10 +5933,10 @@
         <v>4.92</v>
       </c>
       <c r="F196" t="n">
-        <v>45.08</v>
+        <v>45.07</v>
       </c>
       <c r="G196" t="n">
-        <v>607.36</v>
+        <v>607.07</v>
       </c>
     </row>
     <row r="197">
@@ -5956,10 +5956,10 @@
         <v>5.07</v>
       </c>
       <c r="F197" t="n">
-        <v>47.97</v>
+        <v>47.96</v>
       </c>
       <c r="G197" t="n">
-        <v>667.91</v>
+        <v>667.59</v>
       </c>
     </row>
     <row r="198">
@@ -5976,13 +5976,13 @@
         <v>220</v>
       </c>
       <c r="E198" t="n">
-        <v>5.97</v>
+        <v>5.96</v>
       </c>
       <c r="F198" t="n">
-        <v>67.07</v>
+        <v>67.05</v>
       </c>
       <c r="G198" t="n">
-        <v>1113.84</v>
+        <v>1113.29</v>
       </c>
     </row>
     <row r="199">
@@ -6002,10 +6002,10 @@
         <v>6.59</v>
       </c>
       <c r="F199" t="n">
-        <v>82.35</v>
+        <v>82.33</v>
       </c>
       <c r="G199" t="n">
-        <v>1522.4</v>
+        <v>1521.65</v>
       </c>
     </row>
     <row r="200">
@@ -6097,7 +6097,7 @@
         <v>3.4</v>
       </c>
       <c r="G203" t="n">
-        <v>10.42</v>
+        <v>10.43</v>
       </c>
     </row>
     <row r="204">
@@ -6120,7 +6120,7 @@
         <v>5.85</v>
       </c>
       <c r="G204" t="n">
-        <v>25.22</v>
+        <v>25.23</v>
       </c>
     </row>
     <row r="205">
@@ -6143,7 +6143,7 @@
         <v>7.19</v>
       </c>
       <c r="G205" t="n">
-        <v>35.07</v>
+        <v>35.09</v>
       </c>
     </row>
     <row r="206">
@@ -6166,7 +6166,7 @@
         <v>7.43</v>
       </c>
       <c r="G206" t="n">
-        <v>36.98</v>
+        <v>37.01</v>
       </c>
     </row>
     <row r="207">
@@ -6183,13 +6183,13 @@
         <v>230</v>
       </c>
       <c r="E207" t="n">
-        <v>2.23</v>
+        <v>2.24</v>
       </c>
       <c r="F207" t="n">
         <v>8.36</v>
       </c>
       <c r="G207" t="n">
-        <v>44.55</v>
+        <v>44.58</v>
       </c>
     </row>
     <row r="208">
@@ -6206,13 +6206,13 @@
         <v>231</v>
       </c>
       <c r="E208" t="n">
-        <v>2.62</v>
+        <v>2.63</v>
       </c>
       <c r="F208" t="n">
-        <v>11.89</v>
+        <v>11.9</v>
       </c>
       <c r="G208" t="n">
-        <v>77.57</v>
+        <v>77.62</v>
       </c>
     </row>
     <row r="209">
@@ -6235,7 +6235,7 @@
         <v>15.07</v>
       </c>
       <c r="G209" t="n">
-        <v>112.2</v>
+        <v>112.27</v>
       </c>
     </row>
     <row r="210">
@@ -6255,10 +6255,10 @@
         <v>3.11</v>
       </c>
       <c r="F210" t="n">
-        <v>17.18</v>
+        <v>17.19</v>
       </c>
       <c r="G210" t="n">
-        <v>137.61</v>
+        <v>137.7</v>
       </c>
     </row>
     <row r="211">
@@ -6278,10 +6278,10 @@
         <v>3.44</v>
       </c>
       <c r="F211" t="n">
-        <v>21.26</v>
+        <v>21.27</v>
       </c>
       <c r="G211" t="n">
-        <v>191.39</v>
+        <v>191.52</v>
       </c>
     </row>
     <row r="212">
@@ -6298,13 +6298,13 @@
         <v>235</v>
       </c>
       <c r="E212" t="n">
-        <v>3.81</v>
+        <v>3.82</v>
       </c>
       <c r="F212" t="n">
-        <v>26.43</v>
+        <v>26.44</v>
       </c>
       <c r="G212" t="n">
-        <v>267.69</v>
+        <v>267.86</v>
       </c>
     </row>
     <row r="213">
@@ -6324,10 +6324,10 @@
         <v>4.51</v>
       </c>
       <c r="F213" t="n">
-        <v>37.5</v>
+        <v>37.51</v>
       </c>
       <c r="G213" t="n">
-        <v>458.14</v>
+        <v>458.45</v>
       </c>
     </row>
     <row r="214">
@@ -6347,10 +6347,10 @@
         <v>4.67</v>
       </c>
       <c r="F214" t="n">
-        <v>40.36</v>
+        <v>40.37</v>
       </c>
       <c r="G214" t="n">
-        <v>512.73</v>
+        <v>513.08</v>
       </c>
     </row>
     <row r="215">
@@ -6367,13 +6367,13 @@
         <v>238</v>
       </c>
       <c r="E215" t="n">
-        <v>4.79</v>
+        <v>4.8</v>
       </c>
       <c r="F215" t="n">
-        <v>42.66</v>
+        <v>42.68</v>
       </c>
       <c r="G215" t="n">
-        <v>558.2</v>
+        <v>558.58</v>
       </c>
     </row>
     <row r="216">
@@ -6390,13 +6390,13 @@
         <v>239</v>
       </c>
       <c r="E216" t="n">
-        <v>4.8</v>
+        <v>4.81</v>
       </c>
       <c r="F216" t="n">
-        <v>42.84</v>
+        <v>42.86</v>
       </c>
       <c r="G216" t="n">
-        <v>561.78</v>
+        <v>562.16</v>
       </c>
     </row>
     <row r="217">
@@ -6416,10 +6416,10 @@
         <v>5.21</v>
       </c>
       <c r="F217" t="n">
-        <v>50.69</v>
+        <v>50.71</v>
       </c>
       <c r="G217" t="n">
-        <v>726.67</v>
+        <v>727.16</v>
       </c>
     </row>
     <row r="218">
@@ -6439,10 +6439,10 @@
         <v>1.27</v>
       </c>
       <c r="F218" t="n">
-        <v>2.18</v>
+        <v>2.19</v>
       </c>
       <c r="G218" t="n">
-        <v>4.89</v>
+        <v>4.95</v>
       </c>
     </row>
     <row r="219">
@@ -6462,10 +6462,10 @@
         <v>1.28</v>
       </c>
       <c r="F219" t="n">
-        <v>2.23</v>
+        <v>2.25</v>
       </c>
       <c r="G219" t="n">
-        <v>5.11</v>
+        <v>5.18</v>
       </c>
     </row>
     <row r="220">
@@ -6482,13 +6482,13 @@
         <v>245</v>
       </c>
       <c r="E220" t="n">
-        <v>1.44</v>
+        <v>1.45</v>
       </c>
       <c r="F220" t="n">
-        <v>3.01</v>
+        <v>3.04</v>
       </c>
       <c r="G220" t="n">
-        <v>8.53</v>
+        <v>8.65</v>
       </c>
     </row>
     <row r="221">
@@ -6505,13 +6505,13 @@
         <v>246</v>
       </c>
       <c r="E221" t="n">
-        <v>1.5</v>
+        <v>1.51</v>
       </c>
       <c r="F221" t="n">
-        <v>3.35</v>
+        <v>3.38</v>
       </c>
       <c r="G221" t="n">
-        <v>10.18</v>
+        <v>10.32</v>
       </c>
     </row>
     <row r="222">
@@ -6531,10 +6531,10 @@
         <v>1.51</v>
       </c>
       <c r="F222" t="n">
-        <v>3.36</v>
+        <v>3.39</v>
       </c>
       <c r="G222" t="n">
-        <v>10.24</v>
+        <v>10.39</v>
       </c>
     </row>
     <row r="223">
@@ -6554,10 +6554,10 @@
         <v>1.69</v>
       </c>
       <c r="F223" t="n">
-        <v>4.4</v>
+        <v>4.44</v>
       </c>
       <c r="G223" t="n">
-        <v>15.92</v>
+        <v>16.16</v>
       </c>
     </row>
     <row r="224">
@@ -6574,13 +6574,13 @@
         <v>249</v>
       </c>
       <c r="E224" t="n">
-        <v>1.72</v>
+        <v>1.73</v>
       </c>
       <c r="F224" t="n">
-        <v>4.62</v>
+        <v>4.66</v>
       </c>
       <c r="G224" t="n">
-        <v>17.26</v>
+        <v>17.52</v>
       </c>
     </row>
     <row r="225">
@@ -6597,13 +6597,13 @@
         <v>250</v>
       </c>
       <c r="E225" t="n">
-        <v>1.86</v>
+        <v>1.87</v>
       </c>
       <c r="F225" t="n">
-        <v>5.55</v>
+        <v>5.6</v>
       </c>
       <c r="G225" t="n">
-        <v>23.19</v>
+        <v>23.55</v>
       </c>
     </row>
     <row r="226">
@@ -6623,10 +6623,10 @@
         <v>1.91</v>
       </c>
       <c r="F226" t="n">
-        <v>5.84</v>
+        <v>5.9</v>
       </c>
       <c r="G226" t="n">
-        <v>25.21</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="227">
@@ -6643,13 +6643,13 @@
         <v>252</v>
       </c>
       <c r="E227" t="n">
-        <v>1.96</v>
+        <v>1.97</v>
       </c>
       <c r="F227" t="n">
-        <v>6.26</v>
+        <v>6.32</v>
       </c>
       <c r="G227" t="n">
-        <v>28.16</v>
+        <v>28.6</v>
       </c>
     </row>
     <row r="228">
@@ -6666,13 +6666,13 @@
         <v>253</v>
       </c>
       <c r="E228" t="n">
-        <v>1.97</v>
+        <v>1.98</v>
       </c>
       <c r="F228" t="n">
-        <v>6.33</v>
+        <v>6.4</v>
       </c>
       <c r="G228" t="n">
-        <v>28.68</v>
+        <v>29.13</v>
       </c>
     </row>
     <row r="229">
@@ -6689,13 +6689,13 @@
         <v>254</v>
       </c>
       <c r="E229" t="n">
-        <v>2.66</v>
+        <v>2.68</v>
       </c>
       <c r="F229" t="n">
-        <v>12.26</v>
+        <v>12.39</v>
       </c>
       <c r="G229" t="n">
-        <v>81.39</v>
+        <v>82.75</v>
       </c>
     </row>
     <row r="230">
@@ -6712,13 +6712,13 @@
         <v>255</v>
       </c>
       <c r="E230" t="n">
-        <v>2.74</v>
+        <v>2.75</v>
       </c>
       <c r="F230" t="n">
-        <v>13.06</v>
+        <v>13.2</v>
       </c>
       <c r="G230" t="n">
-        <v>89.82</v>
+        <v>91.33</v>
       </c>
     </row>
     <row r="231">
@@ -6735,13 +6735,13 @@
         <v>256</v>
       </c>
       <c r="E231" t="n">
-        <v>2.76</v>
+        <v>2.77</v>
       </c>
       <c r="F231" t="n">
-        <v>13.22</v>
+        <v>13.36</v>
       </c>
       <c r="G231" t="n">
-        <v>91.53</v>
+        <v>93.06</v>
       </c>
     </row>
     <row r="232">
@@ -6758,13 +6758,13 @@
         <v>257</v>
       </c>
       <c r="E232" t="n">
-        <v>3.9</v>
+        <v>3.92</v>
       </c>
       <c r="F232" t="n">
-        <v>27.71</v>
+        <v>28.02</v>
       </c>
       <c r="G232" t="n">
-        <v>287.91</v>
+        <v>292.95</v>
       </c>
     </row>
     <row r="233">
@@ -6781,13 +6781,13 @@
         <v>258</v>
       </c>
       <c r="E233" t="n">
-        <v>4.56</v>
+        <v>4.59</v>
       </c>
       <c r="F233" t="n">
-        <v>38.48</v>
+        <v>38.93</v>
       </c>
       <c r="G233" t="n">
-        <v>476.68</v>
+        <v>485.14</v>
       </c>
     </row>
     <row r="234">
@@ -6804,13 +6804,13 @@
         <v>259</v>
       </c>
       <c r="E234" t="n">
-        <v>5.78</v>
+        <v>5.81</v>
       </c>
       <c r="F234" t="n">
-        <v>62.81</v>
+        <v>63.55</v>
       </c>
       <c r="G234" t="n">
-        <v>1007.88</v>
+        <v>1026.05</v>
       </c>
     </row>
     <row r="235">
@@ -6827,13 +6827,13 @@
         <v>260</v>
       </c>
       <c r="E235" t="n">
-        <v>7.43</v>
+        <v>7.47</v>
       </c>
       <c r="F235" t="n">
-        <v>105.21</v>
+        <v>106.47</v>
       </c>
       <c r="G235" t="n">
-        <v>2208.95</v>
+        <v>2249.23</v>
       </c>
     </row>
     <row r="236">
@@ -6850,13 +6850,13 @@
         <v>262</v>
       </c>
       <c r="E236" t="n">
-        <v>1.2</v>
+        <v>1.21</v>
       </c>
       <c r="F236" t="n">
-        <v>1.88</v>
+        <v>1.9</v>
       </c>
       <c r="G236" t="n">
-        <v>3.79</v>
+        <v>3.85</v>
       </c>
     </row>
     <row r="237">
@@ -6876,10 +6876,10 @@
         <v>1.45</v>
       </c>
       <c r="F237" t="n">
-        <v>3.05</v>
+        <v>3.08</v>
       </c>
       <c r="G237" t="n">
-        <v>8.72</v>
+        <v>8.86</v>
       </c>
     </row>
     <row r="238">
@@ -6899,10 +6899,10 @@
         <v>1.56</v>
       </c>
       <c r="F238" t="n">
-        <v>3.65</v>
+        <v>3.69</v>
       </c>
       <c r="G238" t="n">
-        <v>11.73</v>
+        <v>11.93</v>
       </c>
     </row>
     <row r="239">
@@ -6919,13 +6919,13 @@
         <v>265</v>
       </c>
       <c r="E239" t="n">
-        <v>1.71</v>
+        <v>1.72</v>
       </c>
       <c r="F239" t="n">
-        <v>4.55</v>
+        <v>4.6</v>
       </c>
       <c r="G239" t="n">
-        <v>16.83</v>
+        <v>17.13</v>
       </c>
     </row>
     <row r="240">
@@ -6942,13 +6942,13 @@
         <v>266</v>
       </c>
       <c r="E240" t="n">
-        <v>1.71</v>
+        <v>1.72</v>
       </c>
       <c r="F240" t="n">
-        <v>4.57</v>
+        <v>4.62</v>
       </c>
       <c r="G240" t="n">
-        <v>16.97</v>
+        <v>17.27</v>
       </c>
     </row>
     <row r="241">
@@ -6968,10 +6968,10 @@
         <v>1.78</v>
       </c>
       <c r="F241" t="n">
-        <v>4.97</v>
+        <v>5.02</v>
       </c>
       <c r="G241" t="n">
-        <v>19.4</v>
+        <v>19.75</v>
       </c>
     </row>
     <row r="242">
@@ -6988,13 +6988,13 @@
         <v>268</v>
       </c>
       <c r="E242" t="n">
-        <v>1.81</v>
+        <v>1.82</v>
       </c>
       <c r="F242" t="n">
-        <v>5.17</v>
+        <v>5.23</v>
       </c>
       <c r="G242" t="n">
-        <v>20.72</v>
+        <v>21.1</v>
       </c>
     </row>
     <row r="243">
@@ -7011,13 +7011,13 @@
         <v>269</v>
       </c>
       <c r="E243" t="n">
-        <v>1.99</v>
+        <v>2</v>
       </c>
       <c r="F243" t="n">
-        <v>6.42</v>
+        <v>6.5</v>
       </c>
       <c r="G243" t="n">
-        <v>29.31</v>
+        <v>29.86</v>
       </c>
     </row>
     <row r="244">
@@ -7034,13 +7034,13 @@
         <v>270</v>
       </c>
       <c r="E244" t="n">
-        <v>2.01</v>
+        <v>2.03</v>
       </c>
       <c r="F244" t="n">
-        <v>6.63</v>
+        <v>6.71</v>
       </c>
       <c r="G244" t="n">
-        <v>30.83</v>
+        <v>31.41</v>
       </c>
     </row>
     <row r="245">
@@ -7057,13 +7057,13 @@
         <v>271</v>
       </c>
       <c r="E245" t="n">
-        <v>2.44</v>
+        <v>2.46</v>
       </c>
       <c r="F245" t="n">
-        <v>10.17</v>
+        <v>10.29</v>
       </c>
       <c r="G245" t="n">
-        <v>60.67</v>
+        <v>61.86</v>
       </c>
     </row>
     <row r="246">
@@ -7080,13 +7080,13 @@
         <v>272</v>
       </c>
       <c r="E246" t="n">
-        <v>3.24</v>
+        <v>3.26</v>
       </c>
       <c r="F246" t="n">
-        <v>18.75</v>
+        <v>19</v>
       </c>
       <c r="G246" t="n">
-        <v>157.62</v>
+        <v>160.85</v>
       </c>
     </row>
     <row r="247">
@@ -7103,13 +7103,13 @@
         <v>273</v>
       </c>
       <c r="E247" t="n">
-        <v>3.26</v>
+        <v>3.28</v>
       </c>
       <c r="F247" t="n">
-        <v>18.92</v>
+        <v>19.17</v>
       </c>
       <c r="G247" t="n">
-        <v>159.83</v>
+        <v>163.11</v>
       </c>
     </row>
     <row r="248">
@@ -7126,13 +7126,13 @@
         <v>274</v>
       </c>
       <c r="E248" t="n">
-        <v>3.61</v>
+        <v>3.63</v>
       </c>
       <c r="F248" t="n">
-        <v>23.5</v>
+        <v>23.81</v>
       </c>
       <c r="G248" t="n">
-        <v>223.36</v>
+        <v>228</v>
       </c>
     </row>
     <row r="249">
@@ -7149,13 +7149,13 @@
         <v>275</v>
       </c>
       <c r="E249" t="n">
-        <v>3.96</v>
+        <v>3.99</v>
       </c>
       <c r="F249" t="n">
-        <v>28.65</v>
+        <v>29.04</v>
       </c>
       <c r="G249" t="n">
-        <v>303.06</v>
+        <v>309.41</v>
       </c>
     </row>
     <row r="250">
@@ -7172,13 +7172,13 @@
         <v>276</v>
       </c>
       <c r="E250" t="n">
-        <v>5.26</v>
+        <v>5.29</v>
       </c>
       <c r="F250" t="n">
-        <v>51.64</v>
+        <v>52.36</v>
       </c>
       <c r="G250" t="n">
-        <v>747.54</v>
+        <v>763.51</v>
       </c>
     </row>
     <row r="251">
@@ -7195,13 +7195,13 @@
         <v>277</v>
       </c>
       <c r="E251" t="n">
-        <v>5.88</v>
+        <v>5.92</v>
       </c>
       <c r="F251" t="n">
-        <v>65.12</v>
+        <v>66.04</v>
       </c>
       <c r="G251" t="n">
-        <v>1064.89</v>
+        <v>1087.79</v>
       </c>
     </row>
     <row r="252">
@@ -7218,13 +7218,13 @@
         <v>278</v>
       </c>
       <c r="E252" t="n">
-        <v>6.13</v>
+        <v>6.17</v>
       </c>
       <c r="F252" t="n">
-        <v>70.87</v>
+        <v>71.87</v>
       </c>
       <c r="G252" t="n">
-        <v>1211.37</v>
+        <v>1237.48</v>
       </c>
     </row>
     <row r="253">
@@ -7241,13 +7241,13 @@
         <v>279</v>
       </c>
       <c r="E253" t="n">
-        <v>9.86</v>
+        <v>9.93</v>
       </c>
       <c r="F253" t="n">
-        <v>187.84</v>
+        <v>190.56</v>
       </c>
       <c r="G253" t="n">
-        <v>5318.69</v>
+        <v>5435.45</v>
       </c>
     </row>
     <row r="254">
@@ -7264,13 +7264,13 @@
         <v>282</v>
       </c>
       <c r="E254" t="n">
-        <v>1.35</v>
+        <v>1.34</v>
       </c>
       <c r="F254" t="n">
-        <v>2.54</v>
+        <v>2.53</v>
       </c>
       <c r="G254" t="n">
-        <v>6.38</v>
+        <v>6.37</v>
       </c>
     </row>
     <row r="255">
@@ -7293,7 +7293,7 @@
         <v>3.49</v>
       </c>
       <c r="G255" t="n">
-        <v>10.91</v>
+        <v>10.89</v>
       </c>
     </row>
     <row r="256">
@@ -7310,13 +7310,13 @@
         <v>284</v>
       </c>
       <c r="E256" t="n">
-        <v>1.6</v>
+        <v>1.59</v>
       </c>
       <c r="F256" t="n">
-        <v>3.86</v>
+        <v>3.85</v>
       </c>
       <c r="G256" t="n">
-        <v>12.86</v>
+        <v>12.83</v>
       </c>
     </row>
     <row r="257">
@@ -7336,10 +7336,10 @@
         <v>1.69</v>
       </c>
       <c r="F257" t="n">
-        <v>4.41</v>
+        <v>4.4</v>
       </c>
       <c r="G257" t="n">
-        <v>15.97</v>
+        <v>15.93</v>
       </c>
     </row>
     <row r="258">
@@ -7359,10 +7359,10 @@
         <v>1.73</v>
       </c>
       <c r="F258" t="n">
-        <v>4.68</v>
+        <v>4.67</v>
       </c>
       <c r="G258" t="n">
-        <v>17.63</v>
+        <v>17.58</v>
       </c>
     </row>
     <row r="259">
@@ -7382,10 +7382,10 @@
         <v>1.85</v>
       </c>
       <c r="F259" t="n">
-        <v>5.48</v>
+        <v>5.47</v>
       </c>
       <c r="G259" t="n">
-        <v>22.73</v>
+        <v>22.68</v>
       </c>
     </row>
     <row r="260">
@@ -7405,10 +7405,10 @@
         <v>2.12</v>
       </c>
       <c r="F260" t="n">
-        <v>7.41</v>
+        <v>7.39</v>
       </c>
       <c r="G260" t="n">
-        <v>36.78</v>
+        <v>36.69</v>
       </c>
     </row>
     <row r="261">
@@ -7428,10 +7428,10 @@
         <v>2.3</v>
       </c>
       <c r="F261" t="n">
-        <v>8.91</v>
+        <v>8.9</v>
       </c>
       <c r="G261" t="n">
-        <v>49.3</v>
+        <v>49.17</v>
       </c>
     </row>
     <row r="262">
@@ -7451,10 +7451,10 @@
         <v>2.36</v>
       </c>
       <c r="F262" t="n">
-        <v>9.44</v>
+        <v>9.43</v>
       </c>
       <c r="G262" t="n">
-        <v>54.03</v>
+        <v>53.89</v>
       </c>
     </row>
     <row r="263">
@@ -7474,10 +7474,10 @@
         <v>2.92</v>
       </c>
       <c r="F263" t="n">
-        <v>14.97</v>
+        <v>14.94</v>
       </c>
       <c r="G263" t="n">
-        <v>111.07</v>
+        <v>110.77</v>
       </c>
     </row>
     <row r="264">
@@ -7497,10 +7497,10 @@
         <v>2.98</v>
       </c>
       <c r="F264" t="n">
-        <v>15.69</v>
+        <v>15.66</v>
       </c>
       <c r="G264" t="n">
-        <v>119.53</v>
+        <v>119.21</v>
       </c>
     </row>
     <row r="265">
@@ -7517,13 +7517,13 @@
         <v>293</v>
       </c>
       <c r="E265" t="n">
-        <v>4.17</v>
+        <v>4.16</v>
       </c>
       <c r="F265" t="n">
-        <v>31.8</v>
+        <v>31.74</v>
       </c>
       <c r="G265" t="n">
-        <v>355.76</v>
+        <v>354.76</v>
       </c>
     </row>
     <row r="266">
@@ -7540,13 +7540,13 @@
         <v>294</v>
       </c>
       <c r="E266" t="n">
-        <v>4.44</v>
+        <v>4.43</v>
       </c>
       <c r="F266" t="n">
-        <v>36.32</v>
+        <v>36.25</v>
       </c>
       <c r="G266" t="n">
-        <v>436.2</v>
+        <v>434.97</v>
       </c>
     </row>
     <row r="267">
@@ -7566,10 +7566,10 @@
         <v>4.47</v>
       </c>
       <c r="F267" t="n">
-        <v>36.9</v>
+        <v>36.83</v>
       </c>
       <c r="G267" t="n">
-        <v>446.92</v>
+        <v>445.66</v>
       </c>
     </row>
     <row r="268">
@@ -7586,13 +7586,13 @@
         <v>296</v>
       </c>
       <c r="E268" t="n">
-        <v>4.51</v>
+        <v>4.5</v>
       </c>
       <c r="F268" t="n">
-        <v>37.48</v>
+        <v>37.41</v>
       </c>
       <c r="G268" t="n">
-        <v>457.86</v>
+        <v>456.57</v>
       </c>
     </row>
     <row r="269">
@@ -7609,13 +7609,13 @@
         <v>297</v>
       </c>
       <c r="E269" t="n">
-        <v>7.76</v>
+        <v>7.75</v>
       </c>
       <c r="F269" t="n">
-        <v>115.02</v>
+        <v>114.8</v>
       </c>
       <c r="G269" t="n">
-        <v>2529.18</v>
+        <v>2521.83</v>
       </c>
     </row>
     <row r="270">
@@ -7632,13 +7632,13 @@
         <v>298</v>
       </c>
       <c r="E270" t="n">
-        <v>8.26</v>
+        <v>8.25</v>
       </c>
       <c r="F270" t="n">
-        <v>130.82</v>
+        <v>130.57</v>
       </c>
       <c r="G270" t="n">
-        <v>3074.41</v>
+        <v>3065.45</v>
       </c>
     </row>
     <row r="271">
@@ -7655,13 +7655,13 @@
         <v>299</v>
       </c>
       <c r="E271" t="n">
-        <v>9.97</v>
+        <v>9.96</v>
       </c>
       <c r="F271" t="n">
-        <v>191.87</v>
+        <v>191.49</v>
       </c>
       <c r="G271" t="n">
-        <v>5492.01</v>
+        <v>5475.91</v>
       </c>
     </row>
     <row r="272">
@@ -7681,10 +7681,10 @@
         <v>1.26</v>
       </c>
       <c r="F272" t="n">
-        <v>2.12</v>
+        <v>2.11</v>
       </c>
       <c r="G272" t="n">
-        <v>4.66</v>
+        <v>4.65</v>
       </c>
     </row>
     <row r="273">
@@ -7707,7 +7707,7 @@
         <v>2.49</v>
       </c>
       <c r="G273" t="n">
-        <v>6.18</v>
+        <v>6.17</v>
       </c>
     </row>
     <row r="274">
@@ -7730,7 +7730,7 @@
         <v>2.61</v>
       </c>
       <c r="G274" t="n">
-        <v>6.7</v>
+        <v>6.69</v>
       </c>
     </row>
     <row r="275">
@@ -7753,7 +7753,7 @@
         <v>2.69</v>
       </c>
       <c r="G275" t="n">
-        <v>7.05</v>
+        <v>7.04</v>
       </c>
     </row>
     <row r="276">
@@ -7776,7 +7776,7 @@
         <v>3.26</v>
       </c>
       <c r="G276" t="n">
-        <v>9.75</v>
+        <v>9.73</v>
       </c>
     </row>
     <row r="277">
@@ -7799,7 +7799,7 @@
         <v>3.48</v>
       </c>
       <c r="G277" t="n">
-        <v>10.86</v>
+        <v>10.84</v>
       </c>
     </row>
     <row r="278">
@@ -7819,10 +7819,10 @@
         <v>1.73</v>
       </c>
       <c r="F278" t="n">
-        <v>4.65</v>
+        <v>4.64</v>
       </c>
       <c r="G278" t="n">
-        <v>17.43</v>
+        <v>17.4</v>
       </c>
     </row>
     <row r="279">
@@ -7842,10 +7842,10 @@
         <v>1.94</v>
       </c>
       <c r="F279" t="n">
-        <v>6.1</v>
+        <v>6.09</v>
       </c>
       <c r="G279" t="n">
-        <v>27.01</v>
+        <v>26.95</v>
       </c>
     </row>
     <row r="280">
@@ -7865,10 +7865,10 @@
         <v>2.07</v>
       </c>
       <c r="F280" t="n">
-        <v>7.06</v>
+        <v>7.05</v>
       </c>
       <c r="G280" t="n">
-        <v>34.07</v>
+        <v>34.01</v>
       </c>
     </row>
     <row r="281">
@@ -7888,10 +7888,10 @@
         <v>2.3</v>
       </c>
       <c r="F281" t="n">
-        <v>8.89</v>
+        <v>8.88</v>
       </c>
       <c r="G281" t="n">
-        <v>49.15</v>
+        <v>49.05</v>
       </c>
     </row>
     <row r="282">
@@ -7911,10 +7911,10 @@
         <v>2.49</v>
       </c>
       <c r="F282" t="n">
-        <v>10.64</v>
+        <v>10.62</v>
       </c>
       <c r="G282" t="n">
-        <v>65.14</v>
+        <v>65</v>
       </c>
     </row>
     <row r="283">
@@ -7934,10 +7934,10 @@
         <v>2.75</v>
       </c>
       <c r="F283" t="n">
-        <v>13.18</v>
+        <v>13.16</v>
       </c>
       <c r="G283" t="n">
-        <v>91.09</v>
+        <v>90.9</v>
       </c>
     </row>
     <row r="284">
@@ -7957,10 +7957,10 @@
         <v>3.12</v>
       </c>
       <c r="F284" t="n">
-        <v>17.29</v>
+        <v>17.27</v>
       </c>
       <c r="G284" t="n">
-        <v>138.96</v>
+        <v>138.67</v>
       </c>
     </row>
     <row r="285">
@@ -7980,10 +7980,10 @@
         <v>3.69</v>
       </c>
       <c r="F285" t="n">
-        <v>24.62</v>
+        <v>24.58</v>
       </c>
       <c r="G285" t="n">
-        <v>239.95</v>
+        <v>239.42</v>
       </c>
     </row>
     <row r="286">
@@ -8003,10 +8003,10 @@
         <v>3.94</v>
       </c>
       <c r="F286" t="n">
-        <v>28.3</v>
+        <v>28.26</v>
       </c>
       <c r="G286" t="n">
-        <v>297.41</v>
+        <v>296.76</v>
       </c>
     </row>
     <row r="287">
@@ -8023,13 +8023,13 @@
         <v>316</v>
       </c>
       <c r="E287" t="n">
-        <v>4.3</v>
+        <v>4.29</v>
       </c>
       <c r="F287" t="n">
-        <v>33.95</v>
+        <v>33.9</v>
       </c>
       <c r="G287" t="n">
-        <v>393.44</v>
+        <v>392.57</v>
       </c>
     </row>
     <row r="288">
@@ -8049,10 +8049,10 @@
         <v>4.65</v>
       </c>
       <c r="F288" t="n">
-        <v>40.07</v>
+        <v>40.01</v>
       </c>
       <c r="G288" t="n">
-        <v>507.12</v>
+        <v>505.99</v>
       </c>
     </row>
     <row r="289">
@@ -8072,10 +8072,10 @@
         <v>4.78</v>
       </c>
       <c r="F289" t="n">
-        <v>42.45</v>
+        <v>42.39</v>
       </c>
       <c r="G289" t="n">
-        <v>554.01</v>
+        <v>552.77</v>
       </c>
     </row>
     <row r="290">
@@ -8374,7 +8374,7 @@
         <v>15.67</v>
       </c>
       <c r="G302" t="n">
-        <v>119.31</v>
+        <v>119.32</v>
       </c>
     </row>
     <row r="303">
@@ -8443,7 +8443,7 @@
         <v>65.65</v>
       </c>
       <c r="G305" t="n">
-        <v>1077.96</v>
+        <v>1077.98</v>
       </c>
     </row>
     <row r="306">
@@ -8463,10 +8463,10 @@
         <v>6.76</v>
       </c>
       <c r="F306" t="n">
-        <v>86.64</v>
+        <v>86.65</v>
       </c>
       <c r="G306" t="n">
-        <v>1644.67</v>
+        <v>1644.69</v>
       </c>
     </row>
     <row r="307">
@@ -8489,7 +8489,7 @@
         <v>184.32</v>
       </c>
       <c r="G307" t="n">
-        <v>5168.26</v>
+        <v>5168.34</v>
       </c>
     </row>
     <row r="308">
@@ -8788,7 +8788,7 @@
         <v>15.4</v>
       </c>
       <c r="G320" t="n">
-        <v>116.09</v>
+        <v>116.08</v>
       </c>
     </row>
     <row r="321">
@@ -8834,7 +8834,7 @@
         <v>25.46</v>
       </c>
       <c r="G322" t="n">
-        <v>252.72</v>
+        <v>252.71</v>
       </c>
     </row>
     <row r="323">
@@ -8880,7 +8880,7 @@
         <v>38.24</v>
       </c>
       <c r="G324" t="n">
-        <v>472.09</v>
+        <v>472.08</v>
       </c>
     </row>
     <row r="325">
@@ -8903,7 +8903,7 @@
         <v>63.33</v>
       </c>
       <c r="G325" t="n">
-        <v>1020.65</v>
+        <v>1020.63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-08-13 15:58:57
</commit_message>
<xml_diff>
--- a/files/AFL_goalscorers.xlsx
+++ b/files/AFL_goalscorers.xlsx
@@ -2299,10 +2299,10 @@
         <v>1.37</v>
       </c>
       <c r="F38" t="n">
-        <v>2.65</v>
+        <v>2.66</v>
       </c>
       <c r="G38" t="n">
-        <v>6.85</v>
+        <v>6.93</v>
       </c>
     </row>
     <row r="39">
@@ -2319,13 +2319,13 @@
         <v>49</v>
       </c>
       <c r="E39" t="n">
-        <v>1.52</v>
+        <v>1.53</v>
       </c>
       <c r="F39" t="n">
-        <v>3.46</v>
+        <v>3.49</v>
       </c>
       <c r="G39" t="n">
-        <v>10.75</v>
+        <v>10.89</v>
       </c>
     </row>
     <row r="40">
@@ -2342,13 +2342,13 @@
         <v>50</v>
       </c>
       <c r="E40" t="n">
-        <v>1.76</v>
+        <v>1.77</v>
       </c>
       <c r="F40" t="n">
-        <v>4.88</v>
+        <v>4.92</v>
       </c>
       <c r="G40" t="n">
-        <v>18.83</v>
+        <v>19.09</v>
       </c>
     </row>
     <row r="41">
@@ -2365,13 +2365,13 @@
         <v>51</v>
       </c>
       <c r="E41" t="n">
-        <v>1.85</v>
+        <v>1.86</v>
       </c>
       <c r="F41" t="n">
-        <v>5.45</v>
+        <v>5.5</v>
       </c>
       <c r="G41" t="n">
-        <v>22.53</v>
+        <v>22.84</v>
       </c>
     </row>
     <row r="42">
@@ -2388,13 +2388,13 @@
         <v>52</v>
       </c>
       <c r="E42" t="n">
-        <v>1.96</v>
+        <v>1.97</v>
       </c>
       <c r="F42" t="n">
-        <v>6.23</v>
+        <v>6.28</v>
       </c>
       <c r="G42" t="n">
-        <v>27.92</v>
+        <v>28.32</v>
       </c>
     </row>
     <row r="43">
@@ -2411,13 +2411,13 @@
         <v>53</v>
       </c>
       <c r="E43" t="n">
-        <v>2.05</v>
+        <v>2.06</v>
       </c>
       <c r="F43" t="n">
-        <v>6.9</v>
+        <v>6.96</v>
       </c>
       <c r="G43" t="n">
-        <v>32.85</v>
+        <v>33.33</v>
       </c>
     </row>
     <row r="44">
@@ -2434,13 +2434,13 @@
         <v>54</v>
       </c>
       <c r="E44" t="n">
-        <v>2.08</v>
+        <v>2.09</v>
       </c>
       <c r="F44" t="n">
-        <v>7.13</v>
+        <v>7.19</v>
       </c>
       <c r="G44" t="n">
-        <v>34.61</v>
+        <v>35.11</v>
       </c>
     </row>
     <row r="45">
@@ -2457,13 +2457,13 @@
         <v>55</v>
       </c>
       <c r="E45" t="n">
-        <v>2.09</v>
+        <v>2.1</v>
       </c>
       <c r="F45" t="n">
-        <v>7.17</v>
+        <v>7.24</v>
       </c>
       <c r="G45" t="n">
-        <v>34.94</v>
+        <v>35.45</v>
       </c>
     </row>
     <row r="46">
@@ -2480,13 +2480,13 @@
         <v>56</v>
       </c>
       <c r="E46" t="n">
-        <v>2.35</v>
+        <v>2.36</v>
       </c>
       <c r="F46" t="n">
-        <v>9.3</v>
+        <v>9.38</v>
       </c>
       <c r="G46" t="n">
-        <v>52.7</v>
+        <v>53.49</v>
       </c>
     </row>
     <row r="47">
@@ -2503,13 +2503,13 @@
         <v>57</v>
       </c>
       <c r="E47" t="n">
-        <v>3.14</v>
+        <v>3.15</v>
       </c>
       <c r="F47" t="n">
-        <v>17.44</v>
+        <v>17.61</v>
       </c>
       <c r="G47" t="n">
-        <v>140.82</v>
+        <v>143.03</v>
       </c>
     </row>
     <row r="48">
@@ -2526,13 +2526,13 @@
         <v>58</v>
       </c>
       <c r="E48" t="n">
-        <v>3.2</v>
+        <v>3.22</v>
       </c>
       <c r="F48" t="n">
-        <v>18.26</v>
+        <v>18.44</v>
       </c>
       <c r="G48" t="n">
-        <v>151.23</v>
+        <v>153.61</v>
       </c>
     </row>
     <row r="49">
@@ -2549,13 +2549,13 @@
         <v>59</v>
       </c>
       <c r="E49" t="n">
-        <v>4.39</v>
+        <v>4.41</v>
       </c>
       <c r="F49" t="n">
-        <v>35.52</v>
+        <v>35.89</v>
       </c>
       <c r="G49" t="n">
-        <v>421.55</v>
+        <v>428.37</v>
       </c>
     </row>
     <row r="50">
@@ -2572,13 +2572,13 @@
         <v>60</v>
       </c>
       <c r="E50" t="n">
-        <v>4.64</v>
+        <v>4.66</v>
       </c>
       <c r="F50" t="n">
-        <v>39.84</v>
+        <v>40.26</v>
       </c>
       <c r="G50" t="n">
-        <v>502.69</v>
+        <v>510.86</v>
       </c>
     </row>
     <row r="51">
@@ -2595,13 +2595,13 @@
         <v>61</v>
       </c>
       <c r="E51" t="n">
-        <v>6.87</v>
+        <v>6.91</v>
       </c>
       <c r="F51" t="n">
-        <v>89.8</v>
+        <v>90.78</v>
       </c>
       <c r="G51" t="n">
-        <v>1736.73</v>
+        <v>1765.57</v>
       </c>
     </row>
     <row r="52">
@@ -2618,13 +2618,13 @@
         <v>62</v>
       </c>
       <c r="E52" t="n">
-        <v>7.15</v>
+        <v>7.19</v>
       </c>
       <c r="F52" t="n">
-        <v>97.36</v>
+        <v>98.42</v>
       </c>
       <c r="G52" t="n">
-        <v>1963.57</v>
+        <v>1996.24</v>
       </c>
     </row>
     <row r="53">
@@ -2641,13 +2641,13 @@
         <v>63</v>
       </c>
       <c r="E53" t="n">
-        <v>7.18</v>
+        <v>7.22</v>
       </c>
       <c r="F53" t="n">
-        <v>98.21</v>
+        <v>99.28</v>
       </c>
       <c r="G53" t="n">
-        <v>1989.67</v>
+        <v>2022.77</v>
       </c>
     </row>
     <row r="54">
@@ -2664,13 +2664,13 @@
         <v>64</v>
       </c>
       <c r="E54" t="n">
-        <v>10.53</v>
+        <v>10.58</v>
       </c>
       <c r="F54" t="n">
-        <v>214.45</v>
+        <v>216.83</v>
       </c>
       <c r="G54" t="n">
-        <v>6499.08</v>
+        <v>6608.61</v>
       </c>
     </row>
     <row r="55">
@@ -2687,13 +2687,13 @@
         <v>65</v>
       </c>
       <c r="E55" t="n">
-        <v>11.85</v>
+        <v>11.91</v>
       </c>
       <c r="F55" t="n">
-        <v>272.83</v>
+        <v>275.87</v>
       </c>
       <c r="G55" t="n">
-        <v>9352.78</v>
+        <v>9510.88</v>
       </c>
     </row>
     <row r="56">
@@ -2716,7 +2716,7 @@
         <v>1.42</v>
       </c>
       <c r="G56" t="n">
-        <v>2.25</v>
+        <v>2.26</v>
       </c>
     </row>
     <row r="57">
@@ -2739,7 +2739,7 @@
         <v>1.99</v>
       </c>
       <c r="G57" t="n">
-        <v>4.17</v>
+        <v>4.19</v>
       </c>
     </row>
     <row r="58">
@@ -2759,10 +2759,10 @@
         <v>1.31</v>
       </c>
       <c r="F58" t="n">
-        <v>2.35</v>
+        <v>2.36</v>
       </c>
       <c r="G58" t="n">
-        <v>5.59</v>
+        <v>5.63</v>
       </c>
     </row>
     <row r="59">
@@ -2782,10 +2782,10 @@
         <v>1.4</v>
       </c>
       <c r="F59" t="n">
-        <v>2.81</v>
+        <v>2.82</v>
       </c>
       <c r="G59" t="n">
-        <v>7.59</v>
+        <v>7.64</v>
       </c>
     </row>
     <row r="60">
@@ -2805,10 +2805,10 @@
         <v>1.47</v>
       </c>
       <c r="F60" t="n">
-        <v>3.15</v>
+        <v>3.17</v>
       </c>
       <c r="G60" t="n">
-        <v>9.2</v>
+        <v>9.27</v>
       </c>
     </row>
     <row r="61">
@@ -2828,10 +2828,10 @@
         <v>1.51</v>
       </c>
       <c r="F61" t="n">
-        <v>3.36</v>
+        <v>3.37</v>
       </c>
       <c r="G61" t="n">
-        <v>10.22</v>
+        <v>10.3</v>
       </c>
     </row>
     <row r="62">
@@ -2851,10 +2851,10 @@
         <v>1.51</v>
       </c>
       <c r="F62" t="n">
-        <v>3.37</v>
+        <v>3.38</v>
       </c>
       <c r="G62" t="n">
-        <v>10.27</v>
+        <v>10.34</v>
       </c>
     </row>
     <row r="63">
@@ -2874,10 +2874,10 @@
         <v>1.63</v>
       </c>
       <c r="F63" t="n">
-        <v>4.04</v>
+        <v>4.06</v>
       </c>
       <c r="G63" t="n">
-        <v>13.85</v>
+        <v>13.96</v>
       </c>
     </row>
     <row r="64">
@@ -2897,10 +2897,10 @@
         <v>1.79</v>
       </c>
       <c r="F64" t="n">
-        <v>5.03</v>
+        <v>5.05</v>
       </c>
       <c r="G64" t="n">
-        <v>19.79</v>
+        <v>19.95</v>
       </c>
     </row>
     <row r="65">
@@ -2920,10 +2920,10 @@
         <v>1.81</v>
       </c>
       <c r="F65" t="n">
-        <v>5.19</v>
+        <v>5.21</v>
       </c>
       <c r="G65" t="n">
-        <v>20.81</v>
+        <v>20.98</v>
       </c>
     </row>
     <row r="66">
@@ -2940,13 +2940,13 @@
         <v>77</v>
       </c>
       <c r="E66" t="n">
-        <v>1.91</v>
+        <v>1.92</v>
       </c>
       <c r="F66" t="n">
-        <v>5.89</v>
+        <v>5.92</v>
       </c>
       <c r="G66" t="n">
-        <v>25.55</v>
+        <v>25.75</v>
       </c>
     </row>
     <row r="67">
@@ -2963,13 +2963,13 @@
         <v>78</v>
       </c>
       <c r="E67" t="n">
-        <v>2.05</v>
+        <v>2.06</v>
       </c>
       <c r="F67" t="n">
-        <v>6.92</v>
+        <v>6.96</v>
       </c>
       <c r="G67" t="n">
-        <v>33.03</v>
+        <v>33.31</v>
       </c>
     </row>
     <row r="68">
@@ -2986,13 +2986,13 @@
         <v>79</v>
       </c>
       <c r="E68" t="n">
-        <v>2.87</v>
+        <v>2.88</v>
       </c>
       <c r="F68" t="n">
-        <v>14.4</v>
+        <v>14.49</v>
       </c>
       <c r="G68" t="n">
-        <v>104.62</v>
+        <v>105.55</v>
       </c>
     </row>
     <row r="69">
@@ -3009,13 +3009,13 @@
         <v>80</v>
       </c>
       <c r="E69" t="n">
-        <v>3.11</v>
+        <v>3.12</v>
       </c>
       <c r="F69" t="n">
-        <v>17.16</v>
+        <v>17.25</v>
       </c>
       <c r="G69" t="n">
-        <v>137.28</v>
+        <v>138.52</v>
       </c>
     </row>
     <row r="70">
@@ -3032,13 +3032,13 @@
         <v>81</v>
       </c>
       <c r="E70" t="n">
-        <v>3.19</v>
+        <v>3.2</v>
       </c>
       <c r="F70" t="n">
-        <v>18.15</v>
+        <v>18.26</v>
       </c>
       <c r="G70" t="n">
-        <v>149.87</v>
+        <v>151.22</v>
       </c>
     </row>
     <row r="71">
@@ -3055,13 +3055,13 @@
         <v>82</v>
       </c>
       <c r="E71" t="n">
-        <v>4.27</v>
+        <v>4.28</v>
       </c>
       <c r="F71" t="n">
-        <v>33.51</v>
+        <v>33.71</v>
       </c>
       <c r="G71" t="n">
-        <v>385.61</v>
+        <v>389.18</v>
       </c>
     </row>
     <row r="72">
@@ -3078,13 +3078,13 @@
         <v>83</v>
       </c>
       <c r="E72" t="n">
-        <v>4.79</v>
+        <v>4.8</v>
       </c>
       <c r="F72" t="n">
-        <v>42.57</v>
+        <v>42.83</v>
       </c>
       <c r="G72" t="n">
-        <v>556.39</v>
+        <v>561.59</v>
       </c>
     </row>
     <row r="73">
@@ -3101,13 +3101,13 @@
         <v>84</v>
       </c>
       <c r="E73" t="n">
-        <v>7.53</v>
+        <v>7.55</v>
       </c>
       <c r="F73" t="n">
-        <v>108.24</v>
+        <v>108.92</v>
       </c>
       <c r="G73" t="n">
-        <v>2306.35</v>
+        <v>2328.41</v>
       </c>
     </row>
     <row r="74">
@@ -3958,7 +3958,7 @@
         <v>1.5</v>
       </c>
       <c r="G110" t="n">
-        <v>2.49</v>
+        <v>2.48</v>
       </c>
     </row>
     <row r="111">
@@ -4001,10 +4001,10 @@
         <v>1.26</v>
       </c>
       <c r="F112" t="n">
-        <v>2.16</v>
+        <v>2.15</v>
       </c>
       <c r="G112" t="n">
-        <v>4.82</v>
+        <v>4.81</v>
       </c>
     </row>
     <row r="113">
@@ -4027,7 +4027,7 @@
         <v>2.37</v>
       </c>
       <c r="G113" t="n">
-        <v>5.68</v>
+        <v>5.67</v>
       </c>
     </row>
     <row r="114">
@@ -4050,7 +4050,7 @@
         <v>3.51</v>
       </c>
       <c r="G114" t="n">
-        <v>10.99</v>
+        <v>10.97</v>
       </c>
     </row>
     <row r="115">
@@ -4070,10 +4070,10 @@
         <v>1.55</v>
       </c>
       <c r="F115" t="n">
-        <v>3.61</v>
+        <v>3.6</v>
       </c>
       <c r="G115" t="n">
-        <v>11.51</v>
+        <v>11.49</v>
       </c>
     </row>
     <row r="116">
@@ -4096,7 +4096,7 @@
         <v>3.69</v>
       </c>
       <c r="G116" t="n">
-        <v>11.97</v>
+        <v>11.95</v>
       </c>
     </row>
     <row r="117">
@@ -4119,7 +4119,7 @@
         <v>4.06</v>
       </c>
       <c r="G117" t="n">
-        <v>13.99</v>
+        <v>13.97</v>
       </c>
     </row>
     <row r="118">
@@ -4139,10 +4139,10 @@
         <v>2.46</v>
       </c>
       <c r="F118" t="n">
-        <v>10.32</v>
+        <v>10.31</v>
       </c>
       <c r="G118" t="n">
-        <v>62.15</v>
+        <v>62.04</v>
       </c>
     </row>
     <row r="119">
@@ -4159,13 +4159,13 @@
         <v>135</v>
       </c>
       <c r="E119" t="n">
-        <v>2.65</v>
+        <v>2.64</v>
       </c>
       <c r="F119" t="n">
-        <v>12.1</v>
+        <v>12.09</v>
       </c>
       <c r="G119" t="n">
-        <v>79.71</v>
+        <v>79.57</v>
       </c>
     </row>
     <row r="120">
@@ -4182,13 +4182,13 @@
         <v>136</v>
       </c>
       <c r="E120" t="n">
-        <v>2.68</v>
+        <v>2.67</v>
       </c>
       <c r="F120" t="n">
-        <v>12.4</v>
+        <v>12.39</v>
       </c>
       <c r="G120" t="n">
-        <v>82.86</v>
+        <v>82.72</v>
       </c>
     </row>
     <row r="121">
@@ -4208,10 +4208,10 @@
         <v>2.82</v>
       </c>
       <c r="F121" t="n">
-        <v>13.86</v>
+        <v>13.84</v>
       </c>
       <c r="G121" t="n">
-        <v>98.48</v>
+        <v>98.31</v>
       </c>
     </row>
     <row r="122">
@@ -4231,10 +4231,10 @@
         <v>2.84</v>
       </c>
       <c r="F122" t="n">
-        <v>14.07</v>
+        <v>14.06</v>
       </c>
       <c r="G122" t="n">
-        <v>100.91</v>
+        <v>100.73</v>
       </c>
     </row>
     <row r="123">
@@ -4251,13 +4251,13 @@
         <v>139</v>
       </c>
       <c r="E123" t="n">
-        <v>3.58</v>
+        <v>3.57</v>
       </c>
       <c r="F123" t="n">
-        <v>23.06</v>
+        <v>23.03</v>
       </c>
       <c r="G123" t="n">
-        <v>216.98</v>
+        <v>216.58</v>
       </c>
     </row>
     <row r="124">
@@ -4277,10 +4277,10 @@
         <v>3.97</v>
       </c>
       <c r="F124" t="n">
-        <v>28.81</v>
+        <v>28.77</v>
       </c>
       <c r="G124" t="n">
-        <v>305.64</v>
+        <v>305.07</v>
       </c>
     </row>
     <row r="125">
@@ -4300,10 +4300,10 @@
         <v>4.95</v>
       </c>
       <c r="F125" t="n">
-        <v>45.63</v>
+        <v>45.58</v>
       </c>
       <c r="G125" t="n">
-        <v>618.82</v>
+        <v>617.65</v>
       </c>
     </row>
     <row r="126">
@@ -4323,10 +4323,10 @@
         <v>6.09</v>
       </c>
       <c r="F126" t="n">
-        <v>70.01</v>
+        <v>69.93</v>
       </c>
       <c r="G126" t="n">
-        <v>1189.14</v>
+        <v>1186.86</v>
       </c>
     </row>
     <row r="127">
@@ -4343,13 +4343,13 @@
         <v>143</v>
       </c>
       <c r="E127" t="n">
-        <v>10.19</v>
+        <v>10.18</v>
       </c>
       <c r="F127" t="n">
-        <v>200.8</v>
+        <v>200.54</v>
       </c>
       <c r="G127" t="n">
-        <v>5883.63</v>
+        <v>5872.13</v>
       </c>
     </row>
     <row r="128">
@@ -4372,7 +4372,7 @@
         <v>1.9</v>
       </c>
       <c r="G128" t="n">
-        <v>3.85</v>
+        <v>3.84</v>
       </c>
     </row>
     <row r="129">
@@ -4395,7 +4395,7 @@
         <v>2.72</v>
       </c>
       <c r="G129" t="n">
-        <v>7.18</v>
+        <v>7.16</v>
       </c>
     </row>
     <row r="130">
@@ -4415,10 +4415,10 @@
         <v>1.66</v>
       </c>
       <c r="F130" t="n">
-        <v>4.22</v>
+        <v>4.21</v>
       </c>
       <c r="G130" t="n">
-        <v>14.88</v>
+        <v>14.85</v>
       </c>
     </row>
     <row r="131">
@@ -4441,7 +4441,7 @@
         <v>4.69</v>
       </c>
       <c r="G131" t="n">
-        <v>17.7</v>
+        <v>17.66</v>
       </c>
     </row>
     <row r="132">
@@ -4461,10 +4461,10 @@
         <v>1.86</v>
       </c>
       <c r="F132" t="n">
-        <v>5.5</v>
+        <v>5.49</v>
       </c>
       <c r="G132" t="n">
-        <v>22.89</v>
+        <v>22.83</v>
       </c>
     </row>
     <row r="133">
@@ -4484,10 +4484,10 @@
         <v>1.94</v>
       </c>
       <c r="F133" t="n">
-        <v>6.1</v>
+        <v>6.09</v>
       </c>
       <c r="G133" t="n">
-        <v>26.97</v>
+        <v>26.91</v>
       </c>
     </row>
     <row r="134">
@@ -4507,10 +4507,10 @@
         <v>2.37</v>
       </c>
       <c r="F134" t="n">
-        <v>9.49</v>
+        <v>9.47</v>
       </c>
       <c r="G134" t="n">
-        <v>54.43</v>
+        <v>54.29</v>
       </c>
     </row>
     <row r="135">
@@ -4530,10 +4530,10 @@
         <v>2.42</v>
       </c>
       <c r="F135" t="n">
-        <v>9.93</v>
+        <v>9.92</v>
       </c>
       <c r="G135" t="n">
-        <v>58.5</v>
+        <v>58.35</v>
       </c>
     </row>
     <row r="136">
@@ -4553,10 +4553,10 @@
         <v>2.54</v>
       </c>
       <c r="F136" t="n">
-        <v>11.09</v>
+        <v>11.07</v>
       </c>
       <c r="G136" t="n">
-        <v>69.52</v>
+        <v>69.33</v>
       </c>
     </row>
     <row r="137">
@@ -4573,13 +4573,13 @@
         <v>154</v>
       </c>
       <c r="E137" t="n">
-        <v>2.89</v>
+        <v>2.88</v>
       </c>
       <c r="F137" t="n">
-        <v>14.59</v>
+        <v>14.57</v>
       </c>
       <c r="G137" t="n">
-        <v>106.75</v>
+        <v>106.46</v>
       </c>
     </row>
     <row r="138">
@@ -4599,10 +4599,10 @@
         <v>3.85</v>
       </c>
       <c r="F138" t="n">
-        <v>26.99</v>
+        <v>26.95</v>
       </c>
       <c r="G138" t="n">
-        <v>276.57</v>
+        <v>275.8</v>
       </c>
     </row>
     <row r="139">
@@ -4619,13 +4619,13 @@
         <v>156</v>
       </c>
       <c r="E139" t="n">
-        <v>4.08</v>
+        <v>4.07</v>
       </c>
       <c r="F139" t="n">
-        <v>30.38</v>
+        <v>30.33</v>
       </c>
       <c r="G139" t="n">
-        <v>331.69</v>
+        <v>330.76</v>
       </c>
     </row>
     <row r="140">
@@ -4645,10 +4645,10 @@
         <v>4.7</v>
       </c>
       <c r="F140" t="n">
-        <v>40.99</v>
+        <v>40.91</v>
       </c>
       <c r="G140" t="n">
-        <v>525.08</v>
+        <v>523.6</v>
       </c>
     </row>
     <row r="141">
@@ -4665,13 +4665,13 @@
         <v>158</v>
       </c>
       <c r="E141" t="n">
-        <v>4.78</v>
+        <v>4.77</v>
       </c>
       <c r="F141" t="n">
-        <v>42.34</v>
+        <v>42.27</v>
       </c>
       <c r="G141" t="n">
-        <v>551.9</v>
+        <v>550.34</v>
       </c>
     </row>
     <row r="142">
@@ -4691,10 +4691,10 @@
         <v>4.79</v>
       </c>
       <c r="F142" t="n">
-        <v>42.58</v>
+        <v>42.5</v>
       </c>
       <c r="G142" t="n">
-        <v>556.54</v>
+        <v>554.98</v>
       </c>
     </row>
     <row r="143">
@@ -4711,13 +4711,13 @@
         <v>160</v>
       </c>
       <c r="E143" t="n">
-        <v>8.1</v>
+        <v>8.09</v>
       </c>
       <c r="F143" t="n">
-        <v>125.74</v>
+        <v>125.5</v>
       </c>
       <c r="G143" t="n">
-        <v>2895.33</v>
+        <v>2886.97</v>
       </c>
     </row>
     <row r="144">
@@ -4734,13 +4734,13 @@
         <v>161</v>
       </c>
       <c r="E144" t="n">
-        <v>12.24</v>
+        <v>12.22</v>
       </c>
       <c r="F144" t="n">
-        <v>291.12</v>
+        <v>290.56</v>
       </c>
       <c r="G144" t="n">
-        <v>10316.44</v>
+        <v>10286.29</v>
       </c>
     </row>
     <row r="145">
@@ -4757,13 +4757,13 @@
         <v>162</v>
       </c>
       <c r="E145" t="n">
-        <v>14.38</v>
+        <v>14.36</v>
       </c>
       <c r="F145" t="n">
-        <v>403.63</v>
+        <v>402.85</v>
       </c>
       <c r="G145" t="n">
-        <v>16897.1</v>
+        <v>16847.57</v>
       </c>
     </row>
     <row r="146">
@@ -4783,10 +4783,10 @@
         <v>1.29</v>
       </c>
       <c r="F146" t="n">
-        <v>2.28</v>
+        <v>2.29</v>
       </c>
       <c r="G146" t="n">
-        <v>5.31</v>
+        <v>5.35</v>
       </c>
     </row>
     <row r="147">
@@ -4806,10 +4806,10 @@
         <v>1.32</v>
       </c>
       <c r="F147" t="n">
-        <v>2.41</v>
+        <v>2.42</v>
       </c>
       <c r="G147" t="n">
-        <v>5.83</v>
+        <v>5.88</v>
       </c>
     </row>
     <row r="148">
@@ -4826,13 +4826,13 @@
         <v>167</v>
       </c>
       <c r="E148" t="n">
-        <v>1.48</v>
+        <v>1.49</v>
       </c>
       <c r="F148" t="n">
-        <v>3.23</v>
+        <v>3.25</v>
       </c>
       <c r="G148" t="n">
-        <v>9.57</v>
+        <v>9.67</v>
       </c>
     </row>
     <row r="149">
@@ -4849,13 +4849,13 @@
         <v>168</v>
       </c>
       <c r="E149" t="n">
-        <v>1.59</v>
+        <v>1.6</v>
       </c>
       <c r="F149" t="n">
-        <v>3.84</v>
+        <v>3.87</v>
       </c>
       <c r="G149" t="n">
-        <v>12.76</v>
+        <v>12.9</v>
       </c>
     </row>
     <row r="150">
@@ -4872,13 +4872,13 @@
         <v>169</v>
       </c>
       <c r="E150" t="n">
-        <v>1.74</v>
+        <v>1.75</v>
       </c>
       <c r="F150" t="n">
-        <v>4.75</v>
+        <v>4.79</v>
       </c>
       <c r="G150" t="n">
-        <v>18.07</v>
+        <v>18.27</v>
       </c>
     </row>
     <row r="151">
@@ -4898,10 +4898,10 @@
         <v>1.8</v>
       </c>
       <c r="F151" t="n">
-        <v>5.1</v>
+        <v>5.14</v>
       </c>
       <c r="G151" t="n">
-        <v>20.26</v>
+        <v>20.48</v>
       </c>
     </row>
     <row r="152">
@@ -4918,13 +4918,13 @@
         <v>171</v>
       </c>
       <c r="E152" t="n">
-        <v>1.84</v>
+        <v>1.85</v>
       </c>
       <c r="F152" t="n">
-        <v>5.4</v>
+        <v>5.43</v>
       </c>
       <c r="G152" t="n">
-        <v>22.18</v>
+        <v>22.43</v>
       </c>
     </row>
     <row r="153">
@@ -4944,10 +4944,10 @@
         <v>1.98</v>
       </c>
       <c r="F153" t="n">
-        <v>6.34</v>
+        <v>6.38</v>
       </c>
       <c r="G153" t="n">
-        <v>28.71</v>
+        <v>29.04</v>
       </c>
     </row>
     <row r="154">
@@ -4964,13 +4964,13 @@
         <v>173</v>
       </c>
       <c r="E154" t="n">
-        <v>1.98</v>
+        <v>1.99</v>
       </c>
       <c r="F154" t="n">
-        <v>6.4</v>
+        <v>6.45</v>
       </c>
       <c r="G154" t="n">
-        <v>29.18</v>
+        <v>29.51</v>
       </c>
     </row>
     <row r="155">
@@ -4987,13 +4987,13 @@
         <v>174</v>
       </c>
       <c r="E155" t="n">
-        <v>2.34</v>
+        <v>2.35</v>
       </c>
       <c r="F155" t="n">
-        <v>9.25</v>
+        <v>9.32</v>
       </c>
       <c r="G155" t="n">
-        <v>52.31</v>
+        <v>52.93</v>
       </c>
     </row>
     <row r="156">
@@ -5010,13 +5010,13 @@
         <v>175</v>
       </c>
       <c r="E156" t="n">
-        <v>3.23</v>
+        <v>3.25</v>
       </c>
       <c r="F156" t="n">
-        <v>18.62</v>
+        <v>18.77</v>
       </c>
       <c r="G156" t="n">
-        <v>155.85</v>
+        <v>157.79</v>
       </c>
     </row>
     <row r="157">
@@ -5033,13 +5033,13 @@
         <v>176</v>
       </c>
       <c r="E157" t="n">
-        <v>3.49</v>
+        <v>3.51</v>
       </c>
       <c r="F157" t="n">
-        <v>21.95</v>
+        <v>22.13</v>
       </c>
       <c r="G157" t="n">
-        <v>201.07</v>
+        <v>203.59</v>
       </c>
     </row>
     <row r="158">
@@ -5056,13 +5056,13 @@
         <v>177</v>
       </c>
       <c r="E158" t="n">
-        <v>3.71</v>
+        <v>3.72</v>
       </c>
       <c r="F158" t="n">
-        <v>24.92</v>
+        <v>25.12</v>
       </c>
       <c r="G158" t="n">
-        <v>244.52</v>
+        <v>247.62</v>
       </c>
     </row>
     <row r="159">
@@ -5079,13 +5079,13 @@
         <v>178</v>
       </c>
       <c r="E159" t="n">
-        <v>3.9</v>
+        <v>3.92</v>
       </c>
       <c r="F159" t="n">
-        <v>27.72</v>
+        <v>27.95</v>
       </c>
       <c r="G159" t="n">
-        <v>288.08</v>
+        <v>291.74</v>
       </c>
     </row>
     <row r="160">
@@ -5102,13 +5102,13 @@
         <v>179</v>
       </c>
       <c r="E160" t="n">
-        <v>4.05</v>
+        <v>4.07</v>
       </c>
       <c r="F160" t="n">
-        <v>29.98</v>
+        <v>30.23</v>
       </c>
       <c r="G160" t="n">
-        <v>324.95</v>
+        <v>329.09</v>
       </c>
     </row>
     <row r="161">
@@ -5125,13 +5125,13 @@
         <v>180</v>
       </c>
       <c r="E161" t="n">
-        <v>5.1</v>
+        <v>5.12</v>
       </c>
       <c r="F161" t="n">
-        <v>48.54</v>
+        <v>48.95</v>
       </c>
       <c r="G161" t="n">
-        <v>680</v>
+        <v>688.81</v>
       </c>
     </row>
     <row r="162">
@@ -5148,13 +5148,13 @@
         <v>181</v>
       </c>
       <c r="E162" t="n">
-        <v>7.18</v>
+        <v>7.21</v>
       </c>
       <c r="F162" t="n">
-        <v>98.25</v>
+        <v>99.1</v>
       </c>
       <c r="G162" t="n">
-        <v>1990.75</v>
+        <v>2017.02</v>
       </c>
     </row>
     <row r="163">
@@ -5171,13 +5171,13 @@
         <v>182</v>
       </c>
       <c r="E163" t="n">
-        <v>9.59</v>
+        <v>9.63</v>
       </c>
       <c r="F163" t="n">
-        <v>177.45</v>
+        <v>179.01</v>
       </c>
       <c r="G163" t="n">
-        <v>4879.55</v>
+        <v>4944.6</v>
       </c>
     </row>
     <row r="164">
@@ -5200,7 +5200,7 @@
         <v>1.52</v>
       </c>
       <c r="G164" t="n">
-        <v>2.54</v>
+        <v>2.56</v>
       </c>
     </row>
     <row r="165">
@@ -5217,13 +5217,13 @@
         <v>185</v>
       </c>
       <c r="E165" t="n">
-        <v>1.25</v>
+        <v>1.26</v>
       </c>
       <c r="F165" t="n">
-        <v>2.11</v>
+        <v>2.12</v>
       </c>
       <c r="G165" t="n">
-        <v>4.62</v>
+        <v>4.66</v>
       </c>
     </row>
     <row r="166">
@@ -5243,10 +5243,10 @@
         <v>1.37</v>
       </c>
       <c r="F166" t="n">
-        <v>2.65</v>
+        <v>2.66</v>
       </c>
       <c r="G166" t="n">
-        <v>6.86</v>
+        <v>6.92</v>
       </c>
     </row>
     <row r="167">
@@ -5263,13 +5263,13 @@
         <v>187</v>
       </c>
       <c r="E167" t="n">
-        <v>1.45</v>
+        <v>1.46</v>
       </c>
       <c r="F167" t="n">
-        <v>3.08</v>
+        <v>3.1</v>
       </c>
       <c r="G167" t="n">
-        <v>8.84</v>
+        <v>8.92</v>
       </c>
     </row>
     <row r="168">
@@ -5286,13 +5286,13 @@
         <v>188</v>
       </c>
       <c r="E168" t="n">
-        <v>1.66</v>
+        <v>1.67</v>
       </c>
       <c r="F168" t="n">
-        <v>4.27</v>
+        <v>4.3</v>
       </c>
       <c r="G168" t="n">
-        <v>15.18</v>
+        <v>15.33</v>
       </c>
     </row>
     <row r="169">
@@ -5312,10 +5312,10 @@
         <v>1.73</v>
       </c>
       <c r="F169" t="n">
-        <v>4.66</v>
+        <v>4.69</v>
       </c>
       <c r="G169" t="n">
-        <v>17.52</v>
+        <v>17.69</v>
       </c>
     </row>
     <row r="170">
@@ -5332,13 +5332,13 @@
         <v>190</v>
       </c>
       <c r="E170" t="n">
-        <v>1.86</v>
+        <v>1.87</v>
       </c>
       <c r="F170" t="n">
-        <v>5.53</v>
+        <v>5.57</v>
       </c>
       <c r="G170" t="n">
-        <v>23.07</v>
+        <v>23.31</v>
       </c>
     </row>
     <row r="171">
@@ -5355,13 +5355,13 @@
         <v>191</v>
       </c>
       <c r="E171" t="n">
-        <v>2.01</v>
+        <v>2.02</v>
       </c>
       <c r="F171" t="n">
-        <v>6.62</v>
+        <v>6.67</v>
       </c>
       <c r="G171" t="n">
-        <v>30.81</v>
+        <v>31.14</v>
       </c>
     </row>
     <row r="172">
@@ -5378,13 +5378,13 @@
         <v>192</v>
       </c>
       <c r="E172" t="n">
-        <v>2.94</v>
+        <v>2.95</v>
       </c>
       <c r="F172" t="n">
-        <v>15.24</v>
+        <v>15.35</v>
       </c>
       <c r="G172" t="n">
-        <v>114.22</v>
+        <v>115.53</v>
       </c>
     </row>
     <row r="173">
@@ -5401,13 +5401,13 @@
         <v>193</v>
       </c>
       <c r="E173" t="n">
-        <v>3.77</v>
+        <v>3.78</v>
       </c>
       <c r="F173" t="n">
-        <v>25.79</v>
+        <v>25.99</v>
       </c>
       <c r="G173" t="n">
-        <v>257.78</v>
+        <v>260.83</v>
       </c>
     </row>
     <row r="174">
@@ -5424,13 +5424,13 @@
         <v>194</v>
       </c>
       <c r="E174" t="n">
-        <v>3.84</v>
+        <v>3.85</v>
       </c>
       <c r="F174" t="n">
-        <v>26.74</v>
+        <v>26.94</v>
       </c>
       <c r="G174" t="n">
-        <v>272.52</v>
+        <v>275.75</v>
       </c>
     </row>
     <row r="175">
@@ -5447,13 +5447,13 @@
         <v>195</v>
       </c>
       <c r="E175" t="n">
-        <v>4.1</v>
+        <v>4.11</v>
       </c>
       <c r="F175" t="n">
-        <v>30.73</v>
+        <v>30.97</v>
       </c>
       <c r="G175" t="n">
-        <v>337.61</v>
+        <v>341.64</v>
       </c>
     </row>
     <row r="176">
@@ -5470,13 +5470,13 @@
         <v>196</v>
       </c>
       <c r="E176" t="n">
-        <v>4.34</v>
+        <v>4.35</v>
       </c>
       <c r="F176" t="n">
-        <v>34.6</v>
+        <v>34.87</v>
       </c>
       <c r="G176" t="n">
-        <v>404.95</v>
+        <v>409.81</v>
       </c>
     </row>
     <row r="177">
@@ -5493,13 +5493,13 @@
         <v>197</v>
       </c>
       <c r="E177" t="n">
-        <v>4.45</v>
+        <v>4.47</v>
       </c>
       <c r="F177" t="n">
-        <v>36.55</v>
+        <v>36.84</v>
       </c>
       <c r="G177" t="n">
-        <v>440.59</v>
+        <v>445.88</v>
       </c>
     </row>
     <row r="178">
@@ -5516,13 +5516,13 @@
         <v>198</v>
       </c>
       <c r="E178" t="n">
-        <v>4.46</v>
+        <v>4.48</v>
       </c>
       <c r="F178" t="n">
-        <v>36.71</v>
+        <v>37</v>
       </c>
       <c r="G178" t="n">
-        <v>443.52</v>
+        <v>448.85</v>
       </c>
     </row>
     <row r="179">
@@ -5539,13 +5539,13 @@
         <v>199</v>
       </c>
       <c r="E179" t="n">
-        <v>4.93</v>
+        <v>4.94</v>
       </c>
       <c r="F179" t="n">
-        <v>45.13</v>
+        <v>45.48</v>
       </c>
       <c r="G179" t="n">
-        <v>608.31</v>
+        <v>615.67</v>
       </c>
     </row>
     <row r="180">
@@ -5562,13 +5562,13 @@
         <v>200</v>
       </c>
       <c r="E180" t="n">
-        <v>5.38</v>
+        <v>5.4</v>
       </c>
       <c r="F180" t="n">
-        <v>54.12</v>
+        <v>54.55</v>
       </c>
       <c r="G180" t="n">
-        <v>803.02</v>
+        <v>812.8</v>
       </c>
     </row>
     <row r="181">
@@ -5585,13 +5585,13 @@
         <v>201</v>
       </c>
       <c r="E181" t="n">
-        <v>6.35</v>
+        <v>6.38</v>
       </c>
       <c r="F181" t="n">
-        <v>76.34</v>
+        <v>76.95</v>
       </c>
       <c r="G181" t="n">
-        <v>1356.41</v>
+        <v>1373.07</v>
       </c>
     </row>
     <row r="182">
@@ -6439,10 +6439,10 @@
         <v>1.27</v>
       </c>
       <c r="F218" t="n">
-        <v>2.19</v>
+        <v>2.17</v>
       </c>
       <c r="G218" t="n">
-        <v>4.95</v>
+        <v>4.89</v>
       </c>
     </row>
     <row r="219">
@@ -6462,10 +6462,10 @@
         <v>1.28</v>
       </c>
       <c r="F219" t="n">
-        <v>2.25</v>
+        <v>2.23</v>
       </c>
       <c r="G219" t="n">
-        <v>5.18</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="220">
@@ -6482,13 +6482,13 @@
         <v>245</v>
       </c>
       <c r="E220" t="n">
-        <v>1.45</v>
+        <v>1.44</v>
       </c>
       <c r="F220" t="n">
-        <v>3.04</v>
+        <v>3.01</v>
       </c>
       <c r="G220" t="n">
-        <v>8.65</v>
+        <v>8.51</v>
       </c>
     </row>
     <row r="221">
@@ -6505,13 +6505,13 @@
         <v>246</v>
       </c>
       <c r="E221" t="n">
-        <v>1.51</v>
+        <v>1.5</v>
       </c>
       <c r="F221" t="n">
-        <v>3.38</v>
+        <v>3.35</v>
       </c>
       <c r="G221" t="n">
-        <v>10.32</v>
+        <v>10.16</v>
       </c>
     </row>
     <row r="222">
@@ -6531,10 +6531,10 @@
         <v>1.51</v>
       </c>
       <c r="F222" t="n">
-        <v>3.39</v>
+        <v>3.36</v>
       </c>
       <c r="G222" t="n">
-        <v>10.39</v>
+        <v>10.22</v>
       </c>
     </row>
     <row r="223">
@@ -6551,13 +6551,13 @@
         <v>248</v>
       </c>
       <c r="E223" t="n">
-        <v>1.69</v>
+        <v>1.68</v>
       </c>
       <c r="F223" t="n">
-        <v>4.44</v>
+        <v>4.39</v>
       </c>
       <c r="G223" t="n">
-        <v>16.16</v>
+        <v>15.89</v>
       </c>
     </row>
     <row r="224">
@@ -6574,13 +6574,13 @@
         <v>249</v>
       </c>
       <c r="E224" t="n">
-        <v>1.73</v>
+        <v>1.72</v>
       </c>
       <c r="F224" t="n">
-        <v>4.66</v>
+        <v>4.62</v>
       </c>
       <c r="G224" t="n">
-        <v>17.52</v>
+        <v>17.22</v>
       </c>
     </row>
     <row r="225">
@@ -6597,13 +6597,13 @@
         <v>250</v>
       </c>
       <c r="E225" t="n">
-        <v>1.87</v>
+        <v>1.86</v>
       </c>
       <c r="F225" t="n">
-        <v>5.6</v>
+        <v>5.54</v>
       </c>
       <c r="G225" t="n">
-        <v>23.55</v>
+        <v>23.14</v>
       </c>
     </row>
     <row r="226">
@@ -6620,13 +6620,13 @@
         <v>251</v>
       </c>
       <c r="E226" t="n">
-        <v>1.91</v>
+        <v>1.9</v>
       </c>
       <c r="F226" t="n">
-        <v>5.9</v>
+        <v>5.84</v>
       </c>
       <c r="G226" t="n">
-        <v>25.6</v>
+        <v>25.15</v>
       </c>
     </row>
     <row r="227">
@@ -6643,13 +6643,13 @@
         <v>252</v>
       </c>
       <c r="E227" t="n">
-        <v>1.97</v>
+        <v>1.96</v>
       </c>
       <c r="F227" t="n">
-        <v>6.32</v>
+        <v>6.25</v>
       </c>
       <c r="G227" t="n">
-        <v>28.6</v>
+        <v>28.1</v>
       </c>
     </row>
     <row r="228">
@@ -6666,13 +6666,13 @@
         <v>253</v>
       </c>
       <c r="E228" t="n">
-        <v>1.98</v>
+        <v>1.97</v>
       </c>
       <c r="F228" t="n">
-        <v>6.4</v>
+        <v>6.32</v>
       </c>
       <c r="G228" t="n">
-        <v>29.13</v>
+        <v>28.61</v>
       </c>
     </row>
     <row r="229">
@@ -6689,13 +6689,13 @@
         <v>254</v>
       </c>
       <c r="E229" t="n">
-        <v>2.68</v>
+        <v>2.66</v>
       </c>
       <c r="F229" t="n">
-        <v>12.39</v>
+        <v>12.24</v>
       </c>
       <c r="G229" t="n">
-        <v>82.75</v>
+        <v>81.19</v>
       </c>
     </row>
     <row r="230">
@@ -6712,13 +6712,13 @@
         <v>255</v>
       </c>
       <c r="E230" t="n">
-        <v>2.75</v>
+        <v>2.74</v>
       </c>
       <c r="F230" t="n">
-        <v>13.2</v>
+        <v>13.04</v>
       </c>
       <c r="G230" t="n">
-        <v>91.33</v>
+        <v>89.6</v>
       </c>
     </row>
     <row r="231">
@@ -6735,13 +6735,13 @@
         <v>256</v>
       </c>
       <c r="E231" t="n">
-        <v>2.77</v>
+        <v>2.75</v>
       </c>
       <c r="F231" t="n">
-        <v>13.36</v>
+        <v>13.2</v>
       </c>
       <c r="G231" t="n">
-        <v>93.06</v>
+        <v>91.3</v>
       </c>
     </row>
     <row r="232">
@@ -6758,13 +6758,13 @@
         <v>257</v>
       </c>
       <c r="E232" t="n">
-        <v>3.92</v>
+        <v>3.9</v>
       </c>
       <c r="F232" t="n">
-        <v>28.02</v>
+        <v>27.66</v>
       </c>
       <c r="G232" t="n">
-        <v>292.95</v>
+        <v>287.17</v>
       </c>
     </row>
     <row r="233">
@@ -6781,13 +6781,13 @@
         <v>258</v>
       </c>
       <c r="E233" t="n">
-        <v>4.59</v>
+        <v>4.56</v>
       </c>
       <c r="F233" t="n">
-        <v>38.93</v>
+        <v>38.42</v>
       </c>
       <c r="G233" t="n">
-        <v>485.14</v>
+        <v>475.44</v>
       </c>
     </row>
     <row r="234">
@@ -6804,13 +6804,13 @@
         <v>259</v>
       </c>
       <c r="E234" t="n">
-        <v>5.81</v>
+        <v>5.77</v>
       </c>
       <c r="F234" t="n">
-        <v>63.55</v>
+        <v>62.7</v>
       </c>
       <c r="G234" t="n">
-        <v>1026.05</v>
+        <v>1005.23</v>
       </c>
     </row>
     <row r="235">
@@ -6827,13 +6827,13 @@
         <v>260</v>
       </c>
       <c r="E235" t="n">
-        <v>7.47</v>
+        <v>7.42</v>
       </c>
       <c r="F235" t="n">
-        <v>106.47</v>
+        <v>105.02</v>
       </c>
       <c r="G235" t="n">
-        <v>2249.23</v>
+        <v>2203.06</v>
       </c>
     </row>
     <row r="236">
@@ -6850,13 +6850,13 @@
         <v>262</v>
       </c>
       <c r="E236" t="n">
-        <v>1.21</v>
+        <v>1.2</v>
       </c>
       <c r="F236" t="n">
-        <v>1.9</v>
+        <v>1.88</v>
       </c>
       <c r="G236" t="n">
-        <v>3.85</v>
+        <v>3.79</v>
       </c>
     </row>
     <row r="237">
@@ -6876,10 +6876,10 @@
         <v>1.45</v>
       </c>
       <c r="F237" t="n">
-        <v>3.08</v>
+        <v>3.05</v>
       </c>
       <c r="G237" t="n">
-        <v>8.86</v>
+        <v>8.7</v>
       </c>
     </row>
     <row r="238">
@@ -6899,10 +6899,10 @@
         <v>1.56</v>
       </c>
       <c r="F238" t="n">
-        <v>3.69</v>
+        <v>3.64</v>
       </c>
       <c r="G238" t="n">
-        <v>11.93</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="239">
@@ -6919,13 +6919,13 @@
         <v>265</v>
       </c>
       <c r="E239" t="n">
-        <v>1.72</v>
+        <v>1.71</v>
       </c>
       <c r="F239" t="n">
-        <v>4.6</v>
+        <v>4.54</v>
       </c>
       <c r="G239" t="n">
-        <v>17.13</v>
+        <v>16.79</v>
       </c>
     </row>
     <row r="240">
@@ -6942,13 +6942,13 @@
         <v>266</v>
       </c>
       <c r="E240" t="n">
-        <v>1.72</v>
+        <v>1.71</v>
       </c>
       <c r="F240" t="n">
-        <v>4.62</v>
+        <v>4.57</v>
       </c>
       <c r="G240" t="n">
-        <v>17.27</v>
+        <v>16.92</v>
       </c>
     </row>
     <row r="241">
@@ -6965,13 +6965,13 @@
         <v>267</v>
       </c>
       <c r="E241" t="n">
-        <v>1.78</v>
+        <v>1.77</v>
       </c>
       <c r="F241" t="n">
-        <v>5.02</v>
+        <v>4.96</v>
       </c>
       <c r="G241" t="n">
-        <v>19.75</v>
+        <v>19.35</v>
       </c>
     </row>
     <row r="242">
@@ -6988,13 +6988,13 @@
         <v>268</v>
       </c>
       <c r="E242" t="n">
-        <v>1.82</v>
+        <v>1.81</v>
       </c>
       <c r="F242" t="n">
-        <v>5.23</v>
+        <v>5.17</v>
       </c>
       <c r="G242" t="n">
-        <v>21.1</v>
+        <v>20.67</v>
       </c>
     </row>
     <row r="243">
@@ -7011,13 +7011,13 @@
         <v>269</v>
       </c>
       <c r="E243" t="n">
-        <v>2</v>
+        <v>1.99</v>
       </c>
       <c r="F243" t="n">
-        <v>6.5</v>
+        <v>6.41</v>
       </c>
       <c r="G243" t="n">
-        <v>29.86</v>
+        <v>29.23</v>
       </c>
     </row>
     <row r="244">
@@ -7034,13 +7034,13 @@
         <v>270</v>
       </c>
       <c r="E244" t="n">
-        <v>2.03</v>
+        <v>2.01</v>
       </c>
       <c r="F244" t="n">
-        <v>6.71</v>
+        <v>6.62</v>
       </c>
       <c r="G244" t="n">
-        <v>31.41</v>
+        <v>30.74</v>
       </c>
     </row>
     <row r="245">
@@ -7057,13 +7057,13 @@
         <v>271</v>
       </c>
       <c r="E245" t="n">
-        <v>2.46</v>
+        <v>2.44</v>
       </c>
       <c r="F245" t="n">
-        <v>10.29</v>
+        <v>10.15</v>
       </c>
       <c r="G245" t="n">
-        <v>61.86</v>
+        <v>60.5</v>
       </c>
     </row>
     <row r="246">
@@ -7080,13 +7080,13 @@
         <v>272</v>
       </c>
       <c r="E246" t="n">
-        <v>3.26</v>
+        <v>3.24</v>
       </c>
       <c r="F246" t="n">
-        <v>19</v>
+        <v>18.72</v>
       </c>
       <c r="G246" t="n">
-        <v>160.85</v>
+        <v>157.16</v>
       </c>
     </row>
     <row r="247">
@@ -7103,13 +7103,13 @@
         <v>273</v>
       </c>
       <c r="E247" t="n">
-        <v>3.28</v>
+        <v>3.25</v>
       </c>
       <c r="F247" t="n">
-        <v>19.17</v>
+        <v>18.89</v>
       </c>
       <c r="G247" t="n">
-        <v>163.11</v>
+        <v>159.36</v>
       </c>
     </row>
     <row r="248">
@@ -7126,13 +7126,13 @@
         <v>274</v>
       </c>
       <c r="E248" t="n">
-        <v>3.63</v>
+        <v>3.6</v>
       </c>
       <c r="F248" t="n">
-        <v>23.81</v>
+        <v>23.45</v>
       </c>
       <c r="G248" t="n">
-        <v>228</v>
+        <v>222.7</v>
       </c>
     </row>
     <row r="249">
@@ -7149,13 +7149,13 @@
         <v>275</v>
       </c>
       <c r="E249" t="n">
-        <v>3.99</v>
+        <v>3.96</v>
       </c>
       <c r="F249" t="n">
-        <v>29.04</v>
+        <v>28.59</v>
       </c>
       <c r="G249" t="n">
-        <v>309.41</v>
+        <v>302.16</v>
       </c>
     </row>
     <row r="250">
@@ -7172,13 +7172,13 @@
         <v>276</v>
       </c>
       <c r="E250" t="n">
-        <v>5.29</v>
+        <v>5.25</v>
       </c>
       <c r="F250" t="n">
-        <v>52.36</v>
+        <v>51.54</v>
       </c>
       <c r="G250" t="n">
-        <v>763.51</v>
+        <v>745.25</v>
       </c>
     </row>
     <row r="251">
@@ -7195,13 +7195,13 @@
         <v>277</v>
       </c>
       <c r="E251" t="n">
-        <v>5.92</v>
+        <v>5.87</v>
       </c>
       <c r="F251" t="n">
-        <v>66.04</v>
+        <v>64.99</v>
       </c>
       <c r="G251" t="n">
-        <v>1087.79</v>
+        <v>1061.6</v>
       </c>
     </row>
     <row r="252">
@@ -7218,13 +7218,13 @@
         <v>278</v>
       </c>
       <c r="E252" t="n">
-        <v>6.17</v>
+        <v>6.12</v>
       </c>
       <c r="F252" t="n">
-        <v>71.87</v>
+        <v>70.73</v>
       </c>
       <c r="G252" t="n">
-        <v>1237.48</v>
+        <v>1207.62</v>
       </c>
     </row>
     <row r="253">
@@ -7241,13 +7241,13 @@
         <v>279</v>
       </c>
       <c r="E253" t="n">
-        <v>9.93</v>
+        <v>9.85</v>
       </c>
       <c r="F253" t="n">
-        <v>190.56</v>
+        <v>187.45</v>
       </c>
       <c r="G253" t="n">
-        <v>5435.45</v>
+        <v>5301.95</v>
       </c>
     </row>
     <row r="254">
@@ -7264,13 +7264,13 @@
         <v>282</v>
       </c>
       <c r="E254" t="n">
-        <v>1.34</v>
+        <v>1.35</v>
       </c>
       <c r="F254" t="n">
-        <v>2.53</v>
+        <v>2.55</v>
       </c>
       <c r="G254" t="n">
-        <v>6.37</v>
+        <v>6.43</v>
       </c>
     </row>
     <row r="255">
@@ -7290,10 +7290,10 @@
         <v>1.53</v>
       </c>
       <c r="F255" t="n">
-        <v>3.49</v>
+        <v>3.51</v>
       </c>
       <c r="G255" t="n">
-        <v>10.89</v>
+        <v>11.02</v>
       </c>
     </row>
     <row r="256">
@@ -7310,13 +7310,13 @@
         <v>284</v>
       </c>
       <c r="E256" t="n">
-        <v>1.59</v>
+        <v>1.6</v>
       </c>
       <c r="F256" t="n">
-        <v>3.85</v>
+        <v>3.88</v>
       </c>
       <c r="G256" t="n">
-        <v>12.83</v>
+        <v>12.99</v>
       </c>
     </row>
     <row r="257">
@@ -7336,10 +7336,10 @@
         <v>1.69</v>
       </c>
       <c r="F257" t="n">
-        <v>4.4</v>
+        <v>4.43</v>
       </c>
       <c r="G257" t="n">
-        <v>15.93</v>
+        <v>16.13</v>
       </c>
     </row>
     <row r="258">
@@ -7356,13 +7356,13 @@
         <v>286</v>
       </c>
       <c r="E258" t="n">
-        <v>1.73</v>
+        <v>1.74</v>
       </c>
       <c r="F258" t="n">
-        <v>4.67</v>
+        <v>4.71</v>
       </c>
       <c r="G258" t="n">
-        <v>17.58</v>
+        <v>17.81</v>
       </c>
     </row>
     <row r="259">
@@ -7379,13 +7379,13 @@
         <v>287</v>
       </c>
       <c r="E259" t="n">
-        <v>1.85</v>
+        <v>1.86</v>
       </c>
       <c r="F259" t="n">
-        <v>5.47</v>
+        <v>5.52</v>
       </c>
       <c r="G259" t="n">
-        <v>22.68</v>
+        <v>22.97</v>
       </c>
     </row>
     <row r="260">
@@ -7405,10 +7405,10 @@
         <v>2.12</v>
       </c>
       <c r="F260" t="n">
-        <v>7.39</v>
+        <v>7.46</v>
       </c>
       <c r="G260" t="n">
-        <v>36.69</v>
+        <v>37.18</v>
       </c>
     </row>
     <row r="261">
@@ -7425,13 +7425,13 @@
         <v>289</v>
       </c>
       <c r="E261" t="n">
-        <v>2.3</v>
+        <v>2.31</v>
       </c>
       <c r="F261" t="n">
-        <v>8.9</v>
+        <v>8.97</v>
       </c>
       <c r="G261" t="n">
-        <v>49.17</v>
+        <v>49.84</v>
       </c>
     </row>
     <row r="262">
@@ -7448,13 +7448,13 @@
         <v>290</v>
       </c>
       <c r="E262" t="n">
-        <v>2.36</v>
+        <v>2.37</v>
       </c>
       <c r="F262" t="n">
-        <v>9.43</v>
+        <v>9.51</v>
       </c>
       <c r="G262" t="n">
-        <v>53.89</v>
+        <v>54.63</v>
       </c>
     </row>
     <row r="263">
@@ -7471,13 +7471,13 @@
         <v>291</v>
       </c>
       <c r="E263" t="n">
-        <v>2.92</v>
+        <v>2.93</v>
       </c>
       <c r="F263" t="n">
-        <v>14.94</v>
+        <v>15.08</v>
       </c>
       <c r="G263" t="n">
-        <v>110.77</v>
+        <v>112.35</v>
       </c>
     </row>
     <row r="264">
@@ -7494,13 +7494,13 @@
         <v>292</v>
       </c>
       <c r="E264" t="n">
-        <v>2.98</v>
+        <v>2.99</v>
       </c>
       <c r="F264" t="n">
-        <v>15.66</v>
+        <v>15.81</v>
       </c>
       <c r="G264" t="n">
-        <v>119.21</v>
+        <v>120.92</v>
       </c>
     </row>
     <row r="265">
@@ -7517,13 +7517,13 @@
         <v>293</v>
       </c>
       <c r="E265" t="n">
-        <v>4.16</v>
+        <v>4.18</v>
       </c>
       <c r="F265" t="n">
-        <v>31.74</v>
+        <v>32.05</v>
       </c>
       <c r="G265" t="n">
-        <v>354.76</v>
+        <v>360.03</v>
       </c>
     </row>
     <row r="266">
@@ -7540,13 +7540,13 @@
         <v>294</v>
       </c>
       <c r="E266" t="n">
-        <v>4.43</v>
+        <v>4.46</v>
       </c>
       <c r="F266" t="n">
-        <v>36.25</v>
+        <v>36.6</v>
       </c>
       <c r="G266" t="n">
-        <v>434.97</v>
+        <v>441.46</v>
       </c>
     </row>
     <row r="267">
@@ -7563,13 +7563,13 @@
         <v>295</v>
       </c>
       <c r="E267" t="n">
-        <v>4.47</v>
+        <v>4.49</v>
       </c>
       <c r="F267" t="n">
-        <v>36.83</v>
+        <v>37.19</v>
       </c>
       <c r="G267" t="n">
-        <v>445.66</v>
+        <v>452.32</v>
       </c>
     </row>
     <row r="268">
@@ -7586,13 +7586,13 @@
         <v>296</v>
       </c>
       <c r="E268" t="n">
-        <v>4.5</v>
+        <v>4.52</v>
       </c>
       <c r="F268" t="n">
-        <v>37.41</v>
+        <v>37.78</v>
       </c>
       <c r="G268" t="n">
-        <v>456.57</v>
+        <v>463.39</v>
       </c>
     </row>
     <row r="269">
@@ -7609,13 +7609,13 @@
         <v>297</v>
       </c>
       <c r="E269" t="n">
-        <v>7.75</v>
+        <v>7.79</v>
       </c>
       <c r="F269" t="n">
-        <v>114.8</v>
+        <v>115.96</v>
       </c>
       <c r="G269" t="n">
-        <v>2521.83</v>
+        <v>2560.64</v>
       </c>
     </row>
     <row r="270">
@@ -7632,13 +7632,13 @@
         <v>298</v>
       </c>
       <c r="E270" t="n">
-        <v>8.25</v>
+        <v>8.29</v>
       </c>
       <c r="F270" t="n">
-        <v>130.57</v>
+        <v>131.89</v>
       </c>
       <c r="G270" t="n">
-        <v>3065.45</v>
+        <v>3112.75</v>
       </c>
     </row>
     <row r="271">
@@ -7655,13 +7655,13 @@
         <v>299</v>
       </c>
       <c r="E271" t="n">
-        <v>9.96</v>
+        <v>10.01</v>
       </c>
       <c r="F271" t="n">
-        <v>191.49</v>
+        <v>193.45</v>
       </c>
       <c r="G271" t="n">
-        <v>5475.91</v>
+        <v>5560.9</v>
       </c>
     </row>
     <row r="272">
@@ -7681,10 +7681,10 @@
         <v>1.26</v>
       </c>
       <c r="F272" t="n">
-        <v>2.11</v>
+        <v>2.12</v>
       </c>
       <c r="G272" t="n">
-        <v>4.65</v>
+        <v>4.69</v>
       </c>
     </row>
     <row r="273">
@@ -7704,10 +7704,10 @@
         <v>1.34</v>
       </c>
       <c r="F273" t="n">
-        <v>2.49</v>
+        <v>2.5</v>
       </c>
       <c r="G273" t="n">
-        <v>6.17</v>
+        <v>6.22</v>
       </c>
     </row>
     <row r="274">
@@ -7727,10 +7727,10 @@
         <v>1.36</v>
       </c>
       <c r="F274" t="n">
-        <v>2.61</v>
+        <v>2.62</v>
       </c>
       <c r="G274" t="n">
-        <v>6.69</v>
+        <v>6.75</v>
       </c>
     </row>
     <row r="275">
@@ -7750,10 +7750,10 @@
         <v>1.38</v>
       </c>
       <c r="F275" t="n">
-        <v>2.69</v>
+        <v>2.7</v>
       </c>
       <c r="G275" t="n">
-        <v>7.04</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="276">
@@ -7773,10 +7773,10 @@
         <v>1.49</v>
       </c>
       <c r="F276" t="n">
-        <v>3.26</v>
+        <v>3.28</v>
       </c>
       <c r="G276" t="n">
-        <v>9.73</v>
+        <v>9.82</v>
       </c>
     </row>
     <row r="277">
@@ -7796,10 +7796,10 @@
         <v>1.53</v>
       </c>
       <c r="F277" t="n">
-        <v>3.48</v>
+        <v>3.5</v>
       </c>
       <c r="G277" t="n">
-        <v>10.84</v>
+        <v>10.94</v>
       </c>
     </row>
     <row r="278">
@@ -7819,10 +7819,10 @@
         <v>1.73</v>
       </c>
       <c r="F278" t="n">
-        <v>4.64</v>
+        <v>4.67</v>
       </c>
       <c r="G278" t="n">
-        <v>17.4</v>
+        <v>17.57</v>
       </c>
     </row>
     <row r="279">
@@ -7839,13 +7839,13 @@
         <v>308</v>
       </c>
       <c r="E279" t="n">
-        <v>1.94</v>
+        <v>1.95</v>
       </c>
       <c r="F279" t="n">
-        <v>6.09</v>
+        <v>6.13</v>
       </c>
       <c r="G279" t="n">
-        <v>26.95</v>
+        <v>27.22</v>
       </c>
     </row>
     <row r="280">
@@ -7862,13 +7862,13 @@
         <v>309</v>
       </c>
       <c r="E280" t="n">
-        <v>2.07</v>
+        <v>2.08</v>
       </c>
       <c r="F280" t="n">
-        <v>7.05</v>
+        <v>7.09</v>
       </c>
       <c r="G280" t="n">
-        <v>34.01</v>
+        <v>34.35</v>
       </c>
     </row>
     <row r="281">
@@ -7888,10 +7888,10 @@
         <v>2.3</v>
       </c>
       <c r="F281" t="n">
-        <v>8.88</v>
+        <v>8.94</v>
       </c>
       <c r="G281" t="n">
-        <v>49.05</v>
+        <v>49.55</v>
       </c>
     </row>
     <row r="282">
@@ -7908,13 +7908,13 @@
         <v>311</v>
       </c>
       <c r="E282" t="n">
-        <v>2.49</v>
+        <v>2.5</v>
       </c>
       <c r="F282" t="n">
-        <v>10.62</v>
+        <v>10.69</v>
       </c>
       <c r="G282" t="n">
-        <v>65</v>
+        <v>65.68</v>
       </c>
     </row>
     <row r="283">
@@ -7931,13 +7931,13 @@
         <v>312</v>
       </c>
       <c r="E283" t="n">
-        <v>2.75</v>
+        <v>2.76</v>
       </c>
       <c r="F283" t="n">
-        <v>13.16</v>
+        <v>13.25</v>
       </c>
       <c r="G283" t="n">
-        <v>90.9</v>
+        <v>91.86</v>
       </c>
     </row>
     <row r="284">
@@ -7954,13 +7954,13 @@
         <v>313</v>
       </c>
       <c r="E284" t="n">
-        <v>3.12</v>
+        <v>3.13</v>
       </c>
       <c r="F284" t="n">
-        <v>17.27</v>
+        <v>17.39</v>
       </c>
       <c r="G284" t="n">
-        <v>138.67</v>
+        <v>140.17</v>
       </c>
     </row>
     <row r="285">
@@ -7977,13 +7977,13 @@
         <v>314</v>
       </c>
       <c r="E285" t="n">
-        <v>3.69</v>
+        <v>3.7</v>
       </c>
       <c r="F285" t="n">
-        <v>24.58</v>
+        <v>24.76</v>
       </c>
       <c r="G285" t="n">
-        <v>239.42</v>
+        <v>242.07</v>
       </c>
     </row>
     <row r="286">
@@ -8000,13 +8000,13 @@
         <v>315</v>
       </c>
       <c r="E286" t="n">
-        <v>3.94</v>
+        <v>3.95</v>
       </c>
       <c r="F286" t="n">
-        <v>28.26</v>
+        <v>28.46</v>
       </c>
       <c r="G286" t="n">
-        <v>296.76</v>
+        <v>300.06</v>
       </c>
     </row>
     <row r="287">
@@ -8023,13 +8023,13 @@
         <v>316</v>
       </c>
       <c r="E287" t="n">
-        <v>4.29</v>
+        <v>4.31</v>
       </c>
       <c r="F287" t="n">
-        <v>33.9</v>
+        <v>34.15</v>
       </c>
       <c r="G287" t="n">
-        <v>392.57</v>
+        <v>396.96</v>
       </c>
     </row>
     <row r="288">
@@ -8046,13 +8046,13 @@
         <v>317</v>
       </c>
       <c r="E288" t="n">
-        <v>4.65</v>
+        <v>4.67</v>
       </c>
       <c r="F288" t="n">
-        <v>40.01</v>
+        <v>40.3</v>
       </c>
       <c r="G288" t="n">
-        <v>505.99</v>
+        <v>511.69</v>
       </c>
     </row>
     <row r="289">
@@ -8069,13 +8069,13 @@
         <v>318</v>
       </c>
       <c r="E289" t="n">
-        <v>4.78</v>
+        <v>4.8</v>
       </c>
       <c r="F289" t="n">
-        <v>42.39</v>
+        <v>42.7</v>
       </c>
       <c r="G289" t="n">
-        <v>552.77</v>
+        <v>559.01</v>
       </c>
     </row>
     <row r="290">

</xml_diff>

<commit_message>
Update model outputs 2026-08-19 08:47:53
</commit_message>
<xml_diff>
--- a/files/AFL_goalscorers.xlsx
+++ b/files/AFL_goalscorers.xlsx
@@ -1468,13 +1468,13 @@
         <v>9</v>
       </c>
       <c r="E2" t="n">
-        <v>1.2</v>
+        <v>1.21</v>
       </c>
       <c r="F2" t="n">
-        <v>1.89</v>
+        <v>1.92</v>
       </c>
       <c r="G2" t="n">
-        <v>3.81</v>
+        <v>3.91</v>
       </c>
     </row>
     <row r="3">
@@ -1491,13 +1491,13 @@
         <v>10</v>
       </c>
       <c r="E3" t="n">
-        <v>1.2</v>
+        <v>1.21</v>
       </c>
       <c r="F3" t="n">
-        <v>1.89</v>
+        <v>1.92</v>
       </c>
       <c r="G3" t="n">
-        <v>3.82</v>
+        <v>3.92</v>
       </c>
     </row>
     <row r="4">
@@ -1514,13 +1514,13 @@
         <v>11</v>
       </c>
       <c r="E4" t="n">
-        <v>1.27</v>
+        <v>1.28</v>
       </c>
       <c r="F4" t="n">
-        <v>2.17</v>
+        <v>2.21</v>
       </c>
       <c r="G4" t="n">
-        <v>4.89</v>
+        <v>5.03</v>
       </c>
     </row>
     <row r="5">
@@ -1537,13 +1537,13 @@
         <v>12</v>
       </c>
       <c r="E5" t="n">
-        <v>1.36</v>
+        <v>1.37</v>
       </c>
       <c r="F5" t="n">
-        <v>2.6</v>
+        <v>2.65</v>
       </c>
       <c r="G5" t="n">
-        <v>6.66</v>
+        <v>6.86</v>
       </c>
     </row>
     <row r="6">
@@ -1560,13 +1560,13 @@
         <v>13</v>
       </c>
       <c r="E6" t="n">
-        <v>1.52</v>
+        <v>1.53</v>
       </c>
       <c r="F6" t="n">
-        <v>3.42</v>
+        <v>3.49</v>
       </c>
       <c r="G6" t="n">
-        <v>10.54</v>
+        <v>10.89</v>
       </c>
     </row>
     <row r="7">
@@ -1583,13 +1583,13 @@
         <v>14</v>
       </c>
       <c r="E7" t="n">
-        <v>1.78</v>
+        <v>1.8</v>
       </c>
       <c r="F7" t="n">
-        <v>5.02</v>
+        <v>5.13</v>
       </c>
       <c r="G7" t="n">
-        <v>19.75</v>
+        <v>20.45</v>
       </c>
     </row>
     <row r="8">
@@ -1606,13 +1606,13 @@
         <v>15</v>
       </c>
       <c r="E8" t="n">
-        <v>1.82</v>
+        <v>1.83</v>
       </c>
       <c r="F8" t="n">
-        <v>5.22</v>
+        <v>5.34</v>
       </c>
       <c r="G8" t="n">
-        <v>21.05</v>
+        <v>21.81</v>
       </c>
     </row>
     <row r="9">
@@ -1629,13 +1629,13 @@
         <v>16</v>
       </c>
       <c r="E9" t="n">
-        <v>1.85</v>
+        <v>1.86</v>
       </c>
       <c r="F9" t="n">
-        <v>5.44</v>
+        <v>5.56</v>
       </c>
       <c r="G9" t="n">
-        <v>22.46</v>
+        <v>23.26</v>
       </c>
     </row>
     <row r="10">
@@ -1652,13 +1652,13 @@
         <v>17</v>
       </c>
       <c r="E10" t="n">
-        <v>1.87</v>
+        <v>1.88</v>
       </c>
       <c r="F10" t="n">
-        <v>5.57</v>
+        <v>5.69</v>
       </c>
       <c r="G10" t="n">
-        <v>23.32</v>
+        <v>24.16</v>
       </c>
     </row>
     <row r="11">
@@ -1675,13 +1675,13 @@
         <v>18</v>
       </c>
       <c r="E11" t="n">
-        <v>1.98</v>
+        <v>2</v>
       </c>
       <c r="F11" t="n">
-        <v>6.37</v>
+        <v>6.52</v>
       </c>
       <c r="G11" t="n">
-        <v>28.96</v>
+        <v>30.03</v>
       </c>
     </row>
     <row r="12">
@@ -1698,13 +1698,13 @@
         <v>19</v>
       </c>
       <c r="E12" t="n">
-        <v>2.94</v>
+        <v>2.97</v>
       </c>
       <c r="F12" t="n">
-        <v>15.15</v>
+        <v>15.53</v>
       </c>
       <c r="G12" t="n">
-        <v>113.16</v>
+        <v>117.66</v>
       </c>
     </row>
     <row r="13">
@@ -1721,13 +1721,13 @@
         <v>20</v>
       </c>
       <c r="E13" t="n">
-        <v>3.16</v>
+        <v>3.19</v>
       </c>
       <c r="F13" t="n">
-        <v>17.68</v>
+        <v>18.13</v>
       </c>
       <c r="G13" t="n">
-        <v>143.86</v>
+        <v>149.63</v>
       </c>
     </row>
     <row r="14">
@@ -1744,13 +1744,13 @@
         <v>21</v>
       </c>
       <c r="E14" t="n">
-        <v>3.2</v>
+        <v>3.24</v>
       </c>
       <c r="F14" t="n">
-        <v>18.26</v>
+        <v>18.73</v>
       </c>
       <c r="G14" t="n">
-        <v>151.22</v>
+        <v>157.29</v>
       </c>
     </row>
     <row r="15">
@@ -1767,13 +1767,13 @@
         <v>22</v>
       </c>
       <c r="E15" t="n">
-        <v>3.42</v>
+        <v>3.46</v>
       </c>
       <c r="F15" t="n">
-        <v>21.02</v>
+        <v>21.57</v>
       </c>
       <c r="G15" t="n">
-        <v>188.03</v>
+        <v>195.64</v>
       </c>
     </row>
     <row r="16">
@@ -1790,13 +1790,13 @@
         <v>23</v>
       </c>
       <c r="E16" t="n">
-        <v>3.55</v>
+        <v>3.6</v>
       </c>
       <c r="F16" t="n">
-        <v>22.76</v>
+        <v>23.35</v>
       </c>
       <c r="G16" t="n">
-        <v>212.6</v>
+        <v>221.24</v>
       </c>
     </row>
     <row r="17">
@@ -1813,13 +1813,13 @@
         <v>24</v>
       </c>
       <c r="E17" t="n">
-        <v>4.5</v>
+        <v>4.56</v>
       </c>
       <c r="F17" t="n">
-        <v>37.38</v>
+        <v>38.38</v>
       </c>
       <c r="G17" t="n">
-        <v>455.94</v>
+        <v>474.85</v>
       </c>
     </row>
     <row r="18">
@@ -1836,13 +1836,13 @@
         <v>25</v>
       </c>
       <c r="E18" t="n">
-        <v>6.39</v>
+        <v>6.48</v>
       </c>
       <c r="F18" t="n">
-        <v>77.36</v>
+        <v>79.5</v>
       </c>
       <c r="G18" t="n">
-        <v>1384.12</v>
+        <v>1442.77</v>
       </c>
     </row>
     <row r="19">
@@ -1859,13 +1859,13 @@
         <v>26</v>
       </c>
       <c r="E19" t="n">
-        <v>8.51</v>
+        <v>8.63</v>
       </c>
       <c r="F19" t="n">
-        <v>139.21</v>
+        <v>143.12</v>
       </c>
       <c r="G19" t="n">
-        <v>3378.37</v>
+        <v>3523.21</v>
       </c>
     </row>
     <row r="20">
@@ -1882,13 +1882,13 @@
         <v>28</v>
       </c>
       <c r="E20" t="n">
-        <v>1.26</v>
+        <v>1.27</v>
       </c>
       <c r="F20" t="n">
-        <v>2.15</v>
+        <v>2.19</v>
       </c>
       <c r="G20" t="n">
-        <v>4.78</v>
+        <v>4.96</v>
       </c>
     </row>
     <row r="21">
@@ -1905,13 +1905,13 @@
         <v>29</v>
       </c>
       <c r="E21" t="n">
-        <v>1.27</v>
+        <v>1.28</v>
       </c>
       <c r="F21" t="n">
-        <v>2.2</v>
+        <v>2.24</v>
       </c>
       <c r="G21" t="n">
-        <v>4.97</v>
+        <v>5.15</v>
       </c>
     </row>
     <row r="22">
@@ -1928,13 +1928,13 @@
         <v>30</v>
       </c>
       <c r="E22" t="n">
-        <v>1.36</v>
+        <v>1.37</v>
       </c>
       <c r="F22" t="n">
-        <v>2.59</v>
+        <v>2.65</v>
       </c>
       <c r="G22" t="n">
-        <v>6.62</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="23">
@@ -1951,13 +1951,13 @@
         <v>31</v>
       </c>
       <c r="E23" t="n">
-        <v>1.48</v>
+        <v>1.5</v>
       </c>
       <c r="F23" t="n">
-        <v>3.24</v>
+        <v>3.32</v>
       </c>
       <c r="G23" t="n">
-        <v>9.62</v>
+        <v>10.02</v>
       </c>
     </row>
     <row r="24">
@@ -1974,13 +1974,13 @@
         <v>32</v>
       </c>
       <c r="E24" t="n">
-        <v>1.8</v>
+        <v>1.82</v>
       </c>
       <c r="F24" t="n">
-        <v>5.1</v>
+        <v>5.24</v>
       </c>
       <c r="G24" t="n">
-        <v>20.26</v>
+        <v>21.18</v>
       </c>
     </row>
     <row r="25">
@@ -1997,13 +1997,13 @@
         <v>33</v>
       </c>
       <c r="E25" t="n">
-        <v>1.87</v>
+        <v>1.89</v>
       </c>
       <c r="F25" t="n">
-        <v>5.57</v>
+        <v>5.73</v>
       </c>
       <c r="G25" t="n">
-        <v>23.33</v>
+        <v>24.41</v>
       </c>
     </row>
     <row r="26">
@@ -2020,13 +2020,13 @@
         <v>34</v>
       </c>
       <c r="E26" t="n">
-        <v>1.9</v>
+        <v>1.93</v>
       </c>
       <c r="F26" t="n">
-        <v>5.82</v>
+        <v>5.99</v>
       </c>
       <c r="G26" t="n">
-        <v>25.06</v>
+        <v>26.23</v>
       </c>
     </row>
     <row r="27">
@@ -2043,13 +2043,13 @@
         <v>35</v>
       </c>
       <c r="E27" t="n">
-        <v>2.79</v>
+        <v>2.83</v>
       </c>
       <c r="F27" t="n">
-        <v>13.57</v>
+        <v>14</v>
       </c>
       <c r="G27" t="n">
-        <v>95.32</v>
+        <v>100.13</v>
       </c>
     </row>
     <row r="28">
@@ -2066,13 +2066,13 @@
         <v>36</v>
       </c>
       <c r="E28" t="n">
-        <v>2.94</v>
+        <v>2.99</v>
       </c>
       <c r="F28" t="n">
-        <v>15.23</v>
+        <v>15.73</v>
       </c>
       <c r="G28" t="n">
-        <v>114.13</v>
+        <v>119.94</v>
       </c>
     </row>
     <row r="29">
@@ -2089,13 +2089,13 @@
         <v>37</v>
       </c>
       <c r="E29" t="n">
-        <v>3.37</v>
+        <v>3.42</v>
       </c>
       <c r="F29" t="n">
-        <v>20.37</v>
+        <v>21.05</v>
       </c>
       <c r="G29" t="n">
-        <v>179.11</v>
+        <v>188.38</v>
       </c>
     </row>
     <row r="30">
@@ -2112,13 +2112,13 @@
         <v>38</v>
       </c>
       <c r="E30" t="n">
-        <v>3.5</v>
+        <v>3.56</v>
       </c>
       <c r="F30" t="n">
-        <v>22.06</v>
+        <v>22.79</v>
       </c>
       <c r="G30" t="n">
-        <v>202.54</v>
+        <v>213.07</v>
       </c>
     </row>
     <row r="31">
@@ -2135,13 +2135,13 @@
         <v>39</v>
       </c>
       <c r="E31" t="n">
-        <v>3.63</v>
+        <v>3.69</v>
       </c>
       <c r="F31" t="n">
-        <v>23.83</v>
+        <v>24.63</v>
       </c>
       <c r="G31" t="n">
-        <v>228.21</v>
+        <v>240.12</v>
       </c>
     </row>
     <row r="32">
@@ -2158,13 +2158,13 @@
         <v>40</v>
       </c>
       <c r="E32" t="n">
-        <v>3.64</v>
+        <v>3.7</v>
       </c>
       <c r="F32" t="n">
-        <v>24</v>
+        <v>24.81</v>
       </c>
       <c r="G32" t="n">
-        <v>230.77</v>
+        <v>242.82</v>
       </c>
     </row>
     <row r="33">
@@ -2181,13 +2181,13 @@
         <v>41</v>
       </c>
       <c r="E33" t="n">
-        <v>4.71</v>
+        <v>4.78</v>
       </c>
       <c r="F33" t="n">
-        <v>41.05</v>
+        <v>42.47</v>
       </c>
       <c r="G33" t="n">
-        <v>526.24</v>
+        <v>554.33</v>
       </c>
     </row>
     <row r="34">
@@ -2204,13 +2204,13 @@
         <v>42</v>
       </c>
       <c r="E34" t="n">
-        <v>5.3</v>
+        <v>5.39</v>
       </c>
       <c r="F34" t="n">
-        <v>52.6</v>
+        <v>54.44</v>
       </c>
       <c r="G34" t="n">
-        <v>768.88</v>
+        <v>810.24</v>
       </c>
     </row>
     <row r="35">
@@ -2227,13 +2227,13 @@
         <v>43</v>
       </c>
       <c r="E35" t="n">
-        <v>6.48</v>
+        <v>6.59</v>
       </c>
       <c r="F35" t="n">
-        <v>79.56</v>
+        <v>82.38</v>
       </c>
       <c r="G35" t="n">
-        <v>1444.61</v>
+        <v>1523.17</v>
       </c>
     </row>
     <row r="36">
@@ -2250,13 +2250,13 @@
         <v>44</v>
       </c>
       <c r="E36" t="n">
-        <v>8.21</v>
+        <v>8.36</v>
       </c>
       <c r="F36" t="n">
-        <v>129.33</v>
+        <v>133.97</v>
       </c>
       <c r="G36" t="n">
-        <v>3021.38</v>
+        <v>3187.3</v>
       </c>
     </row>
     <row r="37">
@@ -2273,13 +2273,13 @@
         <v>45</v>
       </c>
       <c r="E37" t="n">
-        <v>13.9</v>
+        <v>14.15</v>
       </c>
       <c r="F37" t="n">
-        <v>377.01</v>
+        <v>390.79</v>
       </c>
       <c r="G37" t="n">
-        <v>15243.23</v>
+        <v>16092.35</v>
       </c>
     </row>
     <row r="38">
@@ -4786,7 +4786,7 @@
         <v>1.57</v>
       </c>
       <c r="G146" t="n">
-        <v>2.71</v>
+        <v>2.73</v>
       </c>
     </row>
     <row r="147">
@@ -4803,13 +4803,13 @@
         <v>166</v>
       </c>
       <c r="E147" t="n">
-        <v>1.17</v>
+        <v>1.18</v>
       </c>
       <c r="F147" t="n">
         <v>1.76</v>
       </c>
       <c r="G147" t="n">
-        <v>3.34</v>
+        <v>3.36</v>
       </c>
     </row>
     <row r="148">
@@ -4826,13 +4826,13 @@
         <v>167</v>
       </c>
       <c r="E148" t="n">
-        <v>1.24</v>
+        <v>1.25</v>
       </c>
       <c r="F148" t="n">
-        <v>2.06</v>
+        <v>2.07</v>
       </c>
       <c r="G148" t="n">
-        <v>4.46</v>
+        <v>4.49</v>
       </c>
     </row>
     <row r="149">
@@ -4849,13 +4849,13 @@
         <v>168</v>
       </c>
       <c r="E149" t="n">
-        <v>1.28</v>
+        <v>1.29</v>
       </c>
       <c r="F149" t="n">
         <v>2.25</v>
       </c>
       <c r="G149" t="n">
-        <v>5.17</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="150">
@@ -4875,10 +4875,10 @@
         <v>1.35</v>
       </c>
       <c r="F150" t="n">
-        <v>2.56</v>
+        <v>2.57</v>
       </c>
       <c r="G150" t="n">
-        <v>6.46</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="151">
@@ -4898,10 +4898,10 @@
         <v>1.36</v>
       </c>
       <c r="F151" t="n">
-        <v>2.62</v>
+        <v>2.63</v>
       </c>
       <c r="G151" t="n">
-        <v>6.74</v>
+        <v>6.78</v>
       </c>
     </row>
     <row r="152">
@@ -4921,10 +4921,10 @@
         <v>1.44</v>
       </c>
       <c r="F152" t="n">
-        <v>2.99</v>
+        <v>3</v>
       </c>
       <c r="G152" t="n">
-        <v>8.41</v>
+        <v>8.47</v>
       </c>
     </row>
     <row r="153">
@@ -4944,10 +4944,10 @@
         <v>1.52</v>
       </c>
       <c r="F153" t="n">
-        <v>3.43</v>
+        <v>3.45</v>
       </c>
       <c r="G153" t="n">
-        <v>10.59</v>
+        <v>10.67</v>
       </c>
     </row>
     <row r="154">
@@ -4967,10 +4967,10 @@
         <v>1.68</v>
       </c>
       <c r="F154" t="n">
-        <v>4.37</v>
+        <v>4.39</v>
       </c>
       <c r="G154" t="n">
-        <v>15.77</v>
+        <v>15.9</v>
       </c>
     </row>
     <row r="155">
@@ -4990,10 +4990,10 @@
         <v>2.61</v>
       </c>
       <c r="F155" t="n">
-        <v>11.7</v>
+        <v>11.77</v>
       </c>
       <c r="G155" t="n">
-        <v>75.64</v>
+        <v>76.33</v>
       </c>
     </row>
     <row r="156">
@@ -5010,13 +5010,13 @@
         <v>175</v>
       </c>
       <c r="E156" t="n">
-        <v>2.71</v>
+        <v>2.72</v>
       </c>
       <c r="F156" t="n">
-        <v>12.76</v>
+        <v>12.83</v>
       </c>
       <c r="G156" t="n">
-        <v>86.6</v>
+        <v>87.39</v>
       </c>
     </row>
     <row r="157">
@@ -5033,13 +5033,13 @@
         <v>176</v>
       </c>
       <c r="E157" t="n">
-        <v>3.07</v>
+        <v>3.08</v>
       </c>
       <c r="F157" t="n">
-        <v>16.63</v>
+        <v>16.73</v>
       </c>
       <c r="G157" t="n">
-        <v>130.8</v>
+        <v>132.03</v>
       </c>
     </row>
     <row r="158">
@@ -5056,13 +5056,13 @@
         <v>177</v>
       </c>
       <c r="E158" t="n">
-        <v>3.77</v>
+        <v>3.78</v>
       </c>
       <c r="F158" t="n">
-        <v>25.75</v>
+        <v>25.91</v>
       </c>
       <c r="G158" t="n">
-        <v>257.19</v>
+        <v>259.65</v>
       </c>
     </row>
     <row r="159">
@@ -5079,13 +5079,13 @@
         <v>178</v>
       </c>
       <c r="E159" t="n">
-        <v>3.91</v>
+        <v>3.93</v>
       </c>
       <c r="F159" t="n">
-        <v>27.9</v>
+        <v>28.08</v>
       </c>
       <c r="G159" t="n">
-        <v>291.03</v>
+        <v>293.83</v>
       </c>
     </row>
     <row r="160">
@@ -5102,13 +5102,13 @@
         <v>179</v>
       </c>
       <c r="E160" t="n">
-        <v>4.23</v>
+        <v>4.24</v>
       </c>
       <c r="F160" t="n">
-        <v>32.85</v>
+        <v>33.06</v>
       </c>
       <c r="G160" t="n">
-        <v>374.08</v>
+        <v>377.7</v>
       </c>
     </row>
     <row r="161">
@@ -5125,13 +5125,13 @@
         <v>180</v>
       </c>
       <c r="E161" t="n">
-        <v>4.97</v>
+        <v>4.98</v>
       </c>
       <c r="F161" t="n">
-        <v>45.96</v>
+        <v>46.25</v>
       </c>
       <c r="G161" t="n">
-        <v>625.56</v>
+        <v>631.69</v>
       </c>
     </row>
     <row r="162">
@@ -5148,13 +5148,13 @@
         <v>181</v>
       </c>
       <c r="E162" t="n">
-        <v>5.26</v>
+        <v>5.27</v>
       </c>
       <c r="F162" t="n">
-        <v>51.67</v>
+        <v>52.01</v>
       </c>
       <c r="G162" t="n">
-        <v>748.25</v>
+        <v>755.61</v>
       </c>
     </row>
     <row r="163">
@@ -5171,13 +5171,13 @@
         <v>182</v>
       </c>
       <c r="E163" t="n">
-        <v>5.89</v>
+        <v>5.91</v>
       </c>
       <c r="F163" t="n">
-        <v>65.36</v>
+        <v>65.79</v>
       </c>
       <c r="G163" t="n">
-        <v>1070.95</v>
+        <v>1081.55</v>
       </c>
     </row>
     <row r="164">
@@ -5197,10 +5197,10 @@
         <v>1.45</v>
       </c>
       <c r="F164" t="n">
-        <v>3.05</v>
+        <v>3.07</v>
       </c>
       <c r="G164" t="n">
-        <v>8.7</v>
+        <v>8.82</v>
       </c>
     </row>
     <row r="165">
@@ -5217,13 +5217,13 @@
         <v>185</v>
       </c>
       <c r="E165" t="n">
-        <v>1.63</v>
+        <v>1.64</v>
       </c>
       <c r="F165" t="n">
-        <v>4.07</v>
+        <v>4.11</v>
       </c>
       <c r="G165" t="n">
-        <v>14.06</v>
+        <v>14.27</v>
       </c>
     </row>
     <row r="166">
@@ -5240,13 +5240,13 @@
         <v>186</v>
       </c>
       <c r="E166" t="n">
-        <v>1.8</v>
+        <v>1.81</v>
       </c>
       <c r="F166" t="n">
-        <v>5.12</v>
+        <v>5.17</v>
       </c>
       <c r="G166" t="n">
-        <v>20.41</v>
+        <v>20.73</v>
       </c>
     </row>
     <row r="167">
@@ -5263,13 +5263,13 @@
         <v>187</v>
       </c>
       <c r="E167" t="n">
-        <v>1.84</v>
+        <v>1.85</v>
       </c>
       <c r="F167" t="n">
-        <v>5.39</v>
+        <v>5.45</v>
       </c>
       <c r="G167" t="n">
-        <v>22.16</v>
+        <v>22.5</v>
       </c>
     </row>
     <row r="168">
@@ -5286,13 +5286,13 @@
         <v>188</v>
       </c>
       <c r="E168" t="n">
-        <v>1.92</v>
+        <v>1.93</v>
       </c>
       <c r="F168" t="n">
-        <v>5.92</v>
+        <v>5.98</v>
       </c>
       <c r="G168" t="n">
-        <v>25.75</v>
+        <v>26.16</v>
       </c>
     </row>
     <row r="169">
@@ -5309,13 +5309,13 @@
         <v>189</v>
       </c>
       <c r="E169" t="n">
-        <v>2.03</v>
+        <v>2.04</v>
       </c>
       <c r="F169" t="n">
-        <v>6.73</v>
+        <v>6.8</v>
       </c>
       <c r="G169" t="n">
-        <v>31.62</v>
+        <v>32.13</v>
       </c>
     </row>
     <row r="170">
@@ -5332,13 +5332,13 @@
         <v>190</v>
       </c>
       <c r="E170" t="n">
-        <v>2.3</v>
+        <v>2.31</v>
       </c>
       <c r="F170" t="n">
-        <v>8.9</v>
+        <v>9</v>
       </c>
       <c r="G170" t="n">
-        <v>49.24</v>
+        <v>50.06</v>
       </c>
     </row>
     <row r="171">
@@ -5355,13 +5355,13 @@
         <v>191</v>
       </c>
       <c r="E171" t="n">
-        <v>2.53</v>
+        <v>2.54</v>
       </c>
       <c r="F171" t="n">
-        <v>10.95</v>
+        <v>11.07</v>
       </c>
       <c r="G171" t="n">
-        <v>68.2</v>
+        <v>69.35</v>
       </c>
     </row>
     <row r="172">
@@ -5378,13 +5378,13 @@
         <v>192</v>
       </c>
       <c r="E172" t="n">
-        <v>2.61</v>
+        <v>2.62</v>
       </c>
       <c r="F172" t="n">
-        <v>11.75</v>
+        <v>11.88</v>
       </c>
       <c r="G172" t="n">
-        <v>76.16</v>
+        <v>77.46</v>
       </c>
     </row>
     <row r="173">
@@ -5401,13 +5401,13 @@
         <v>193</v>
       </c>
       <c r="E173" t="n">
-        <v>3.26</v>
+        <v>3.28</v>
       </c>
       <c r="F173" t="n">
-        <v>19.01</v>
+        <v>19.22</v>
       </c>
       <c r="G173" t="n">
-        <v>160.95</v>
+        <v>163.78</v>
       </c>
     </row>
     <row r="174">
@@ -5424,13 +5424,13 @@
         <v>194</v>
       </c>
       <c r="E174" t="n">
-        <v>3.42</v>
+        <v>3.44</v>
       </c>
       <c r="F174" t="n">
-        <v>20.97</v>
+        <v>21.21</v>
       </c>
       <c r="G174" t="n">
-        <v>187.33</v>
+        <v>190.65</v>
       </c>
     </row>
     <row r="175">
@@ -5447,13 +5447,13 @@
         <v>195</v>
       </c>
       <c r="E175" t="n">
-        <v>4.61</v>
+        <v>4.63</v>
       </c>
       <c r="F175" t="n">
-        <v>39.25</v>
+        <v>39.72</v>
       </c>
       <c r="G175" t="n">
-        <v>491.42</v>
+        <v>500.35</v>
       </c>
     </row>
     <row r="176">
@@ -5470,13 +5470,13 @@
         <v>196</v>
       </c>
       <c r="E176" t="n">
-        <v>4.84</v>
+        <v>4.87</v>
       </c>
       <c r="F176" t="n">
-        <v>43.56</v>
+        <v>44.08</v>
       </c>
       <c r="G176" t="n">
-        <v>576.32</v>
+        <v>586.82</v>
       </c>
     </row>
     <row r="177">
@@ -5493,13 +5493,13 @@
         <v>197</v>
       </c>
       <c r="E177" t="n">
-        <v>5.21</v>
+        <v>5.24</v>
       </c>
       <c r="F177" t="n">
-        <v>50.69</v>
+        <v>51.29</v>
       </c>
       <c r="G177" t="n">
-        <v>726.59</v>
+        <v>739.89</v>
       </c>
     </row>
     <row r="178">
@@ -5516,13 +5516,13 @@
         <v>198</v>
       </c>
       <c r="E178" t="n">
-        <v>5.38</v>
+        <v>5.41</v>
       </c>
       <c r="F178" t="n">
-        <v>54.23</v>
+        <v>54.87</v>
       </c>
       <c r="G178" t="n">
-        <v>805.41</v>
+        <v>820.18</v>
       </c>
     </row>
     <row r="179">
@@ -5539,13 +5539,13 @@
         <v>199</v>
       </c>
       <c r="E179" t="n">
-        <v>9.12</v>
+        <v>9.17</v>
       </c>
       <c r="F179" t="n">
-        <v>160.07</v>
+        <v>162.04</v>
       </c>
       <c r="G179" t="n">
-        <v>4174.27</v>
+        <v>4252.63</v>
       </c>
     </row>
     <row r="180">
@@ -5562,13 +5562,13 @@
         <v>200</v>
       </c>
       <c r="E180" t="n">
-        <v>9.51</v>
+        <v>9.57</v>
       </c>
       <c r="F180" t="n">
-        <v>174.45</v>
+        <v>176.61</v>
       </c>
       <c r="G180" t="n">
-        <v>4755.32</v>
+        <v>4844.71</v>
       </c>
     </row>
     <row r="181">
@@ -5585,13 +5585,13 @@
         <v>201</v>
       </c>
       <c r="E181" t="n">
-        <v>11.63</v>
+        <v>11.7</v>
       </c>
       <c r="F181" t="n">
-        <v>262.58</v>
+        <v>265.85</v>
       </c>
       <c r="G181" t="n">
-        <v>8826.91</v>
+        <v>8993.73</v>
       </c>
     </row>
     <row r="182">
@@ -7264,13 +7264,13 @@
         <v>282</v>
       </c>
       <c r="E254" t="n">
-        <v>1.29</v>
+        <v>1.33</v>
       </c>
       <c r="F254" t="n">
-        <v>2.29</v>
+        <v>2.44</v>
       </c>
       <c r="G254" t="n">
-        <v>5.33</v>
+        <v>5.98</v>
       </c>
     </row>
     <row r="255">
@@ -7287,13 +7287,13 @@
         <v>283</v>
       </c>
       <c r="E255" t="n">
-        <v>1.41</v>
+        <v>1.45</v>
       </c>
       <c r="F255" t="n">
-        <v>2.83</v>
+        <v>3.05</v>
       </c>
       <c r="G255" t="n">
-        <v>7.69</v>
+        <v>8.7</v>
       </c>
     </row>
     <row r="256">
@@ -7310,13 +7310,13 @@
         <v>284</v>
       </c>
       <c r="E256" t="n">
-        <v>1.48</v>
+        <v>1.52</v>
       </c>
       <c r="F256" t="n">
-        <v>3.19</v>
+        <v>3.45</v>
       </c>
       <c r="G256" t="n">
-        <v>9.4</v>
+        <v>10.69</v>
       </c>
     </row>
     <row r="257">
@@ -7333,13 +7333,13 @@
         <v>285</v>
       </c>
       <c r="E257" t="n">
-        <v>1.53</v>
+        <v>1.58</v>
       </c>
       <c r="F257" t="n">
-        <v>3.48</v>
+        <v>3.77</v>
       </c>
       <c r="G257" t="n">
-        <v>10.86</v>
+        <v>12.37</v>
       </c>
     </row>
     <row r="258">
@@ -7356,13 +7356,13 @@
         <v>286</v>
       </c>
       <c r="E258" t="n">
-        <v>1.89</v>
+        <v>1.96</v>
       </c>
       <c r="F258" t="n">
-        <v>5.72</v>
+        <v>6.25</v>
       </c>
       <c r="G258" t="n">
-        <v>24.35</v>
+        <v>28.06</v>
       </c>
     </row>
     <row r="259">
@@ -7379,13 +7379,13 @@
         <v>287</v>
       </c>
       <c r="E259" t="n">
-        <v>2.15</v>
+        <v>2.25</v>
       </c>
       <c r="F259" t="n">
-        <v>7.69</v>
+        <v>8.44</v>
       </c>
       <c r="G259" t="n">
-        <v>39.07</v>
+        <v>45.26</v>
       </c>
     </row>
     <row r="260">
@@ -7402,13 +7402,13 @@
         <v>288</v>
       </c>
       <c r="E260" t="n">
-        <v>2.25</v>
+        <v>2.35</v>
       </c>
       <c r="F260" t="n">
-        <v>8.49</v>
+        <v>9.32</v>
       </c>
       <c r="G260" t="n">
-        <v>45.64</v>
+        <v>52.95</v>
       </c>
     </row>
     <row r="261">
@@ -7425,13 +7425,13 @@
         <v>289</v>
       </c>
       <c r="E261" t="n">
-        <v>2.35</v>
+        <v>2.46</v>
       </c>
       <c r="F261" t="n">
-        <v>9.36</v>
+        <v>10.3</v>
       </c>
       <c r="G261" t="n">
-        <v>53.31</v>
+        <v>61.93</v>
       </c>
     </row>
     <row r="262">
@@ -7448,13 +7448,13 @@
         <v>290</v>
       </c>
       <c r="E262" t="n">
-        <v>2.76</v>
+        <v>2.89</v>
       </c>
       <c r="F262" t="n">
-        <v>13.24</v>
+        <v>14.62</v>
       </c>
       <c r="G262" t="n">
-        <v>91.76</v>
+        <v>107.03</v>
       </c>
     </row>
     <row r="263">
@@ -7471,13 +7471,13 @@
         <v>291</v>
       </c>
       <c r="E263" t="n">
-        <v>2.96</v>
+        <v>3.1</v>
       </c>
       <c r="F263" t="n">
-        <v>15.43</v>
+        <v>17.06</v>
       </c>
       <c r="G263" t="n">
-        <v>116.45</v>
+        <v>136.04</v>
       </c>
     </row>
     <row r="264">
@@ -7494,13 +7494,13 @@
         <v>292</v>
       </c>
       <c r="E264" t="n">
-        <v>2.99</v>
+        <v>3.14</v>
       </c>
       <c r="F264" t="n">
-        <v>15.78</v>
+        <v>17.45</v>
       </c>
       <c r="G264" t="n">
-        <v>120.62</v>
+        <v>140.95</v>
       </c>
     </row>
     <row r="265">
@@ -7517,13 +7517,13 @@
         <v>293</v>
       </c>
       <c r="E265" t="n">
-        <v>3.64</v>
+        <v>3.82</v>
       </c>
       <c r="F265" t="n">
-        <v>23.94</v>
+        <v>26.54</v>
       </c>
       <c r="G265" t="n">
-        <v>229.84</v>
+        <v>269.51</v>
       </c>
     </row>
     <row r="266">
@@ -7540,13 +7540,13 @@
         <v>294</v>
       </c>
       <c r="E266" t="n">
-        <v>4.04</v>
+        <v>4.25</v>
       </c>
       <c r="F266" t="n">
-        <v>29.86</v>
+        <v>33.15</v>
       </c>
       <c r="G266" t="n">
-        <v>323.01</v>
+        <v>379.32</v>
       </c>
     </row>
     <row r="267">
@@ -7563,13 +7563,13 @@
         <v>295</v>
       </c>
       <c r="E267" t="n">
-        <v>4.8</v>
+        <v>5.05</v>
       </c>
       <c r="F267" t="n">
-        <v>42.75</v>
+        <v>47.56</v>
       </c>
       <c r="G267" t="n">
-        <v>560.1</v>
+        <v>659.11</v>
       </c>
     </row>
     <row r="268">
@@ -7586,13 +7586,13 @@
         <v>296</v>
       </c>
       <c r="E268" t="n">
-        <v>4.84</v>
+        <v>5.09</v>
       </c>
       <c r="F268" t="n">
-        <v>43.47</v>
+        <v>48.36</v>
       </c>
       <c r="G268" t="n">
-        <v>574.54</v>
+        <v>676.16</v>
       </c>
     </row>
     <row r="269">
@@ -7609,13 +7609,13 @@
         <v>297</v>
       </c>
       <c r="E269" t="n">
-        <v>5.08</v>
+        <v>5.35</v>
       </c>
       <c r="F269" t="n">
-        <v>48.18</v>
+        <v>53.62</v>
       </c>
       <c r="G269" t="n">
-        <v>672.35</v>
+        <v>791.67</v>
       </c>
     </row>
     <row r="270">
@@ -7632,13 +7632,13 @@
         <v>298</v>
       </c>
       <c r="E270" t="n">
-        <v>5.2</v>
+        <v>5.47</v>
       </c>
       <c r="F270" t="n">
-        <v>50.4</v>
+        <v>56.1</v>
       </c>
       <c r="G270" t="n">
-        <v>720.27</v>
+        <v>848.29</v>
       </c>
     </row>
     <row r="271">
@@ -7655,13 +7655,13 @@
         <v>299</v>
       </c>
       <c r="E271" t="n">
-        <v>5.46</v>
+        <v>5.75</v>
       </c>
       <c r="F271" t="n">
-        <v>55.83</v>
+        <v>62.17</v>
       </c>
       <c r="G271" t="n">
-        <v>841.98</v>
+        <v>992.09</v>
       </c>
     </row>
     <row r="272">
@@ -7678,13 +7678,13 @@
         <v>301</v>
       </c>
       <c r="E272" t="n">
-        <v>1.1</v>
+        <v>1.11</v>
       </c>
       <c r="F272" t="n">
-        <v>1.43</v>
+        <v>1.47</v>
       </c>
       <c r="G272" t="n">
-        <v>2.29</v>
+        <v>2.41</v>
       </c>
     </row>
     <row r="273">
@@ -7701,13 +7701,13 @@
         <v>302</v>
       </c>
       <c r="E273" t="n">
-        <v>1.19</v>
+        <v>1.21</v>
       </c>
       <c r="F273" t="n">
-        <v>1.84</v>
+        <v>1.91</v>
       </c>
       <c r="G273" t="n">
-        <v>3.64</v>
+        <v>3.89</v>
       </c>
     </row>
     <row r="274">
@@ -7724,13 +7724,13 @@
         <v>303</v>
       </c>
       <c r="E274" t="n">
-        <v>1.32</v>
+        <v>1.34</v>
       </c>
       <c r="F274" t="n">
-        <v>2.42</v>
+        <v>2.53</v>
       </c>
       <c r="G274" t="n">
-        <v>5.87</v>
+        <v>6.33</v>
       </c>
     </row>
     <row r="275">
@@ -7747,13 +7747,13 @@
         <v>304</v>
       </c>
       <c r="E275" t="n">
-        <v>1.39</v>
+        <v>1.41</v>
       </c>
       <c r="F275" t="n">
-        <v>2.74</v>
+        <v>2.87</v>
       </c>
       <c r="G275" t="n">
-        <v>7.25</v>
+        <v>7.84</v>
       </c>
     </row>
     <row r="276">
@@ -7770,13 +7770,13 @@
         <v>305</v>
       </c>
       <c r="E276" t="n">
-        <v>1.51</v>
+        <v>1.54</v>
       </c>
       <c r="F276" t="n">
-        <v>3.37</v>
+        <v>3.54</v>
       </c>
       <c r="G276" t="n">
-        <v>10.27</v>
+        <v>11.16</v>
       </c>
     </row>
     <row r="277">
@@ -7793,13 +7793,13 @@
         <v>306</v>
       </c>
       <c r="E277" t="n">
-        <v>1.51</v>
+        <v>1.54</v>
       </c>
       <c r="F277" t="n">
-        <v>3.38</v>
+        <v>3.55</v>
       </c>
       <c r="G277" t="n">
-        <v>10.31</v>
+        <v>11.21</v>
       </c>
     </row>
     <row r="278">
@@ -7816,13 +7816,13 @@
         <v>307</v>
       </c>
       <c r="E278" t="n">
-        <v>1.52</v>
+        <v>1.55</v>
       </c>
       <c r="F278" t="n">
-        <v>3.45</v>
+        <v>3.63</v>
       </c>
       <c r="G278" t="n">
-        <v>10.68</v>
+        <v>11.61</v>
       </c>
     </row>
     <row r="279">
@@ -7839,13 +7839,13 @@
         <v>308</v>
       </c>
       <c r="E279" t="n">
-        <v>1.63</v>
+        <v>1.66</v>
       </c>
       <c r="F279" t="n">
-        <v>4.04</v>
+        <v>4.26</v>
       </c>
       <c r="G279" t="n">
-        <v>13.89</v>
+        <v>15.14</v>
       </c>
     </row>
     <row r="280">
@@ -7862,13 +7862,13 @@
         <v>309</v>
       </c>
       <c r="E280" t="n">
-        <v>1.81</v>
+        <v>1.86</v>
       </c>
       <c r="F280" t="n">
-        <v>5.2</v>
+        <v>5.5</v>
       </c>
       <c r="G280" t="n">
-        <v>20.87</v>
+        <v>22.84</v>
       </c>
     </row>
     <row r="281">
@@ -7885,13 +7885,13 @@
         <v>310</v>
       </c>
       <c r="E281" t="n">
-        <v>1.82</v>
+        <v>1.87</v>
       </c>
       <c r="F281" t="n">
-        <v>5.28</v>
+        <v>5.59</v>
       </c>
       <c r="G281" t="n">
-        <v>21.43</v>
+        <v>23.46</v>
       </c>
     </row>
     <row r="282">
@@ -7908,13 +7908,13 @@
         <v>311</v>
       </c>
       <c r="E282" t="n">
-        <v>1.87</v>
+        <v>1.91</v>
       </c>
       <c r="F282" t="n">
-        <v>5.56</v>
+        <v>5.89</v>
       </c>
       <c r="G282" t="n">
-        <v>23.3</v>
+        <v>25.52</v>
       </c>
     </row>
     <row r="283">
@@ -7931,13 +7931,13 @@
         <v>312</v>
       </c>
       <c r="E283" t="n">
-        <v>2.05</v>
+        <v>2.1</v>
       </c>
       <c r="F283" t="n">
-        <v>6.89</v>
+        <v>7.31</v>
       </c>
       <c r="G283" t="n">
-        <v>32.83</v>
+        <v>36.05</v>
       </c>
     </row>
     <row r="284">
@@ -7954,13 +7954,13 @@
         <v>313</v>
       </c>
       <c r="E284" t="n">
-        <v>2.91</v>
+        <v>3</v>
       </c>
       <c r="F284" t="n">
-        <v>14.9</v>
+        <v>15.88</v>
       </c>
       <c r="G284" t="n">
-        <v>110.23</v>
+        <v>121.81</v>
       </c>
     </row>
     <row r="285">
@@ -7977,13 +7977,13 @@
         <v>314</v>
       </c>
       <c r="E285" t="n">
-        <v>2.97</v>
+        <v>3.06</v>
       </c>
       <c r="F285" t="n">
-        <v>15.52</v>
+        <v>16.56</v>
       </c>
       <c r="G285" t="n">
-        <v>117.56</v>
+        <v>129.94</v>
       </c>
     </row>
     <row r="286">
@@ -8000,13 +8000,13 @@
         <v>315</v>
       </c>
       <c r="E286" t="n">
-        <v>3.16</v>
+        <v>3.26</v>
       </c>
       <c r="F286" t="n">
-        <v>17.74</v>
+        <v>18.94</v>
       </c>
       <c r="G286" t="n">
-        <v>144.64</v>
+        <v>160</v>
       </c>
     </row>
     <row r="287">
@@ -8023,13 +8023,13 @@
         <v>316</v>
       </c>
       <c r="E287" t="n">
-        <v>4.42</v>
+        <v>4.57</v>
       </c>
       <c r="F287" t="n">
-        <v>36.06</v>
+        <v>38.59</v>
       </c>
       <c r="G287" t="n">
-        <v>431.43</v>
+        <v>478.81</v>
       </c>
     </row>
     <row r="288">
@@ -8046,13 +8046,13 @@
         <v>317</v>
       </c>
       <c r="E288" t="n">
-        <v>4.59</v>
+        <v>4.75</v>
       </c>
       <c r="F288" t="n">
-        <v>39.02</v>
+        <v>41.78</v>
       </c>
       <c r="G288" t="n">
-        <v>487.01</v>
+        <v>540.65</v>
       </c>
     </row>
     <row r="289">
@@ -8069,13 +8069,13 @@
         <v>318</v>
       </c>
       <c r="E289" t="n">
-        <v>8.2</v>
+        <v>8.49</v>
       </c>
       <c r="F289" t="n">
-        <v>128.9</v>
+        <v>138.38</v>
       </c>
       <c r="G289" t="n">
-        <v>3006.49</v>
+        <v>3348</v>
       </c>
     </row>
     <row r="290">

</xml_diff>